<commit_message>
Integrate Home folders, assessment handoff, community contacts and tutorials
</commit_message>
<xml_diff>
--- a/public/templates/pipeline-assessment-workbook.xlsx
+++ b/public/templates/pipeline-assessment-workbook.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R1a23fde255764b76"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="R535acc6d22ca45bb"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R459e4e8d11994188"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="R44e423caa8a54be8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="R04430115208d4b28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="R77bcad7dc1af46a1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="R754e052385da4a99"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="R12063c5eb47640a9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Rf8e17db6897b44c3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R347a107ddac84647"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="Rfe271eeabca34583"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R84349ecb9ec542b7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="Rfa40a56107f445e2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="Rfbc20790698342dd" state="veryHidden"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="R53f414f4cb3541ee"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R6d07ac8bfe794c3e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="Red20ff0add3b4b2b"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R3d4b1515133243a7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="Rc9a0a5f88eb447bb"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Rb8ad1d3d91504ba8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="R8d123d25cf9b485b"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="R2088732c87bd4722"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="R511995de280b4cb4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Rcbe07b2a3d2d493e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R01ce518e638e4e9d"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="Ree8be1cb492b4089"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R6b3b45a78eda492e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="Re757407f23304570"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="Rea432ea5061f4986" state="veryHidden"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="Reedcadc7684d4c32"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Confirm the basics'!$B$1:$E$16</definedName>
@@ -7880,7 +7880,7 @@
         <v>Questionnaire fingerprint</v>
       </c>
       <c r="B2" t="str">
-        <v>3456169589fa9f7f00f4046d618edb6230d90223cf93fd8ca1c9cdc0a289f18d</v>
+        <v>90679cc7ae50bccf1ece35ed905f975b61e0b1af883344804bb08d07b0fc4ea8</v>
       </c>
     </row>
     <row r="3">
@@ -11874,7 +11874,7 @@
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" s="29" t="str">
-        <v>Assessment date</v>
+        <v>Date assessment performed</v>
       </c>
       <c r="C8" s="29" t="str">
         <v>Date (YYYY-MM-DD)</v>
@@ -14035,7 +14035,7 @@
         <v>assessment_date</v>
       </c>
       <c r="B9" s="13" t="str">
-        <v>Assessment date</v>
+        <v>Date assessment performed</v>
       </c>
       <c r="C9" t="str" s="51"/>
       <c r="D9" t="str" s="48"/>

</xml_diff>

<commit_message>
Integrate Home folders, assessment handoff, community contacts and tutorials (#144)
</commit_message>
<xml_diff>
--- a/public/templates/pipeline-assessment-workbook.xlsx
+++ b/public/templates/pipeline-assessment-workbook.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R1a23fde255764b76"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="R535acc6d22ca45bb"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R459e4e8d11994188"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="R44e423caa8a54be8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="R04430115208d4b28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="R77bcad7dc1af46a1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="R754e052385da4a99"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="R12063c5eb47640a9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Rf8e17db6897b44c3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R347a107ddac84647"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="Rfe271eeabca34583"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R84349ecb9ec542b7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="Rfa40a56107f445e2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="Rfbc20790698342dd" state="veryHidden"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="R53f414f4cb3541ee"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R6d07ac8bfe794c3e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="Red20ff0add3b4b2b"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R3d4b1515133243a7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="Rc9a0a5f88eb447bb"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Rb8ad1d3d91504ba8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="R8d123d25cf9b485b"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="R2088732c87bd4722"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="R511995de280b4cb4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Rcbe07b2a3d2d493e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R01ce518e638e4e9d"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="Ree8be1cb492b4089"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R6b3b45a78eda492e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="Re757407f23304570"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="Rea432ea5061f4986" state="veryHidden"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="Reedcadc7684d4c32"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Confirm the basics'!$B$1:$E$16</definedName>
@@ -7880,7 +7880,7 @@
         <v>Questionnaire fingerprint</v>
       </c>
       <c r="B2" t="str">
-        <v>3456169589fa9f7f00f4046d618edb6230d90223cf93fd8ca1c9cdc0a289f18d</v>
+        <v>90679cc7ae50bccf1ece35ed905f975b61e0b1af883344804bb08d07b0fc4ea8</v>
       </c>
     </row>
     <row r="3">
@@ -11874,7 +11874,7 @@
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" s="29" t="str">
-        <v>Assessment date</v>
+        <v>Date assessment performed</v>
       </c>
       <c r="C8" s="29" t="str">
         <v>Date (YYYY-MM-DD)</v>
@@ -14035,7 +14035,7 @@
         <v>assessment_date</v>
       </c>
       <c r="B9" s="13" t="str">
-        <v>Assessment date</v>
+        <v>Date assessment performed</v>
       </c>
       <c r="C9" t="str" s="51"/>
       <c r="D9" t="str" s="48"/>

</xml_diff>

<commit_message>
Keep resident numbers internal to records and workbook recovery
</commit_message>
<xml_diff>
--- a/public/templates/pipeline-assessment-workbook.xlsx
+++ b/public/templates/pipeline-assessment-workbook.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R6d07ac8bfe794c3e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="Red20ff0add3b4b2b"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R3d4b1515133243a7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="Rc9a0a5f88eb447bb"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Rb8ad1d3d91504ba8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="R8d123d25cf9b485b"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="R2088732c87bd4722"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="R511995de280b4cb4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Rcbe07b2a3d2d493e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R01ce518e638e4e9d"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="Ree8be1cb492b4089"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R6b3b45a78eda492e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="Re757407f23304570"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="Rea432ea5061f4986" state="veryHidden"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="Reedcadc7684d4c32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Raba6eabfa2c0467e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="R6d3c53b35ab2451e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R19ade892a9e9487f"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="R8b151a64b22b4af9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Rbf3a71609d6743d6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="Rfd66ce774fc94e99"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="R387c3a8951cc4843"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="Rf20811a60f024902"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Red12527f76d5406e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R7fbf3f91f3294651"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="R647a55aefa954e92"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="Rc2f47f3707024ecf"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="R78cf9d19b64649d0"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="R5721e6970feb49ce" state="veryHidden"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="Rfcdada3041aa4328"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Confirm the basics'!$B$1:$E$16</definedName>
@@ -7880,7 +7880,7 @@
         <v>Questionnaire fingerprint</v>
       </c>
       <c r="B2" t="str">
-        <v>90679cc7ae50bccf1ece35ed905f975b61e0b1af883344804bb08d07b0fc4ea8</v>
+        <v>44ee09c0df7abcd44bc76e520cf2da27dbdbae70d31aef5d40cbd527d55bed9c</v>
       </c>
     </row>
     <row r="3">
@@ -11949,26 +11949,26 @@
       </c>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" ht="34" customHeight="1">
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="3"/>
       <c r="B14" s="29" t="str">
-        <v>Resident number</v>
+        <v>Diagnosis categories</v>
       </c>
       <c r="C14" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Schizophrenia; Schizoaffective disorder; Bipolar disorder; Personality disorder; Substance use disorder; Psychosis; Delusional disorder; Physical health condition; Other</v>
       </c>
       <c r="D14" s="29" t="str">
-        <v>01 Confirm the basics</v>
+        <v>02 How things are now</v>
       </c>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15" ht="34" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="29" t="str">
-        <v>Diagnosis categories</v>
+        <v>Other diagnosis</v>
       </c>
       <c r="C15" s="29" t="str">
-        <v>Schizophrenia; Schizoaffective disorder; Bipolar disorder; Personality disorder; Substance use disorder; Psychosis; Delusional disorder; Physical health condition; Other</v>
+        <v>Text or notes</v>
       </c>
       <c r="D15" s="29" t="str">
         <v>02 How things are now</v>
@@ -11978,10 +11978,10 @@
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="29" t="str">
-        <v>Other diagnosis</v>
+        <v>Secondary diagnosis</v>
       </c>
       <c r="C16" s="29" t="str">
-        <v>Text or notes</v>
+        <v>One item per line</v>
       </c>
       <c r="D16" s="29" t="str">
         <v>02 How things are now</v>
@@ -11991,10 +11991,10 @@
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="3"/>
       <c r="B17" s="29" t="str">
-        <v>Secondary diagnosis</v>
+        <v>Current symptoms</v>
       </c>
       <c r="C17" s="29" t="str">
-        <v>One item per line</v>
+        <v>Text or notes</v>
       </c>
       <c r="D17" s="29" t="str">
         <v>02 How things are now</v>
@@ -12004,7 +12004,7 @@
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="29" t="str">
-        <v>Current symptoms</v>
+        <v>Cognition / orientation</v>
       </c>
       <c r="C18" s="29" t="str">
         <v>Text or notes</v>
@@ -12017,7 +12017,7 @@
     <row r="19" ht="34" customHeight="1">
       <c r="A19" s="3"/>
       <c r="B19" s="29" t="str">
-        <v>Cognition / orientation</v>
+        <v>Primary diagnosis</v>
       </c>
       <c r="C19" s="29" t="str">
         <v>Text or notes</v>
@@ -12030,7 +12030,7 @@
     <row r="20" ht="34" customHeight="1">
       <c r="A20" s="3"/>
       <c r="B20" s="29" t="str">
-        <v>Primary diagnosis</v>
+        <v>Acuity level</v>
       </c>
       <c r="C20" s="29" t="str">
         <v>Text or notes</v>
@@ -12043,23 +12043,23 @@
     <row r="21" ht="34" customHeight="1">
       <c r="A21" s="3"/>
       <c r="B21" s="29" t="str">
-        <v>Acuity level</v>
+        <v>Ability to dress</v>
       </c>
       <c r="C21" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Independent; Some assistance; Total assistance</v>
       </c>
       <c r="D21" s="29" t="str">
-        <v>02 How things are now</v>
+        <v>03 A usual day</v>
       </c>
       <c r="E21" s="3"/>
     </row>
     <row r="22" ht="34" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="29" t="str">
-        <v>Ability to dress</v>
+        <v>Dressing assistance needed</v>
       </c>
       <c r="C22" s="29" t="str">
-        <v>Independent; Some assistance; Total assistance</v>
+        <v>Text or notes</v>
       </c>
       <c r="D22" s="29" t="str">
         <v>03 A usual day</v>
@@ -12069,10 +12069,10 @@
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="29" t="str">
-        <v>Dressing assistance needed</v>
+        <v>Ability to bathe</v>
       </c>
       <c r="C23" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Independent; Some assistance; Total assistance</v>
       </c>
       <c r="D23" s="29" t="str">
         <v>03 A usual day</v>
@@ -12082,10 +12082,10 @@
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="29" t="str">
-        <v>Ability to bathe</v>
+        <v>Bathing assistance needed</v>
       </c>
       <c r="C24" s="29" t="str">
-        <v>Independent; Some assistance; Total assistance</v>
+        <v>Text or notes</v>
       </c>
       <c r="D24" s="29" t="str">
         <v>03 A usual day</v>
@@ -12095,10 +12095,10 @@
     <row r="25" ht="34" customHeight="1">
       <c r="A25" s="3"/>
       <c r="B25" s="29" t="str">
-        <v>Bathing assistance needed</v>
+        <v>Overall hygiene</v>
       </c>
       <c r="C25" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D25" s="29" t="str">
         <v>03 A usual day</v>
@@ -12108,10 +12108,10 @@
     <row r="26" ht="34" customHeight="1">
       <c r="A26" s="3"/>
       <c r="B26" s="29" t="str">
-        <v>Overall hygiene</v>
+        <v>ADL needs</v>
       </c>
       <c r="C26" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D26" s="29" t="str">
         <v>03 A usual day</v>
@@ -12121,7 +12121,7 @@
     <row r="27" ht="34" customHeight="1">
       <c r="A27" s="3"/>
       <c r="B27" s="29" t="str">
-        <v>ADL needs</v>
+        <v>Prompting level</v>
       </c>
       <c r="C27" s="29" t="str">
         <v>Text or notes</v>
@@ -12134,7 +12134,7 @@
     <row r="28" ht="34" customHeight="1">
       <c r="A28" s="3"/>
       <c r="B28" s="29" t="str">
-        <v>Prompting level</v>
+        <v>Self-care status</v>
       </c>
       <c r="C28" s="29" t="str">
         <v>Text or notes</v>
@@ -12147,10 +12147,10 @@
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="3"/>
       <c r="B29" s="29" t="str">
-        <v>Self-care status</v>
+        <v>Ambulatory</v>
       </c>
       <c r="C29" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D29" s="29" t="str">
         <v>03 A usual day</v>
@@ -12160,10 +12160,10 @@
     <row r="30" ht="34" customHeight="1">
       <c r="A30" s="3"/>
       <c r="B30" s="29" t="str">
-        <v>Ambulatory</v>
+        <v>Type of device</v>
       </c>
       <c r="C30" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D30" s="29" t="str">
         <v>03 A usual day</v>
@@ -12173,10 +12173,10 @@
     <row r="31" ht="34" customHeight="1">
       <c r="A31" s="3"/>
       <c r="B31" s="29" t="str">
-        <v>Type of device</v>
+        <v>Language barrier</v>
       </c>
       <c r="C31" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D31" s="29" t="str">
         <v>03 A usual day</v>
@@ -12186,10 +12186,10 @@
     <row r="32" ht="34" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="29" t="str">
-        <v>Language barrier</v>
+        <v>Language support needed</v>
       </c>
       <c r="C32" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D32" s="29" t="str">
         <v>03 A usual day</v>
@@ -12199,10 +12199,10 @@
     <row r="33" ht="34" customHeight="1">
       <c r="A33" s="3"/>
       <c r="B33" s="29" t="str">
-        <v>Language support needed</v>
+        <v>Can hold a linear conversation</v>
       </c>
       <c r="C33" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D33" s="29" t="str">
         <v>03 A usual day</v>
@@ -12212,10 +12212,10 @@
     <row r="34" ht="34" customHeight="1">
       <c r="A34" s="3"/>
       <c r="B34" s="29" t="str">
-        <v>Can hold a linear conversation</v>
+        <v>Conversation barriers</v>
       </c>
       <c r="C34" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D34" s="29" t="str">
         <v>03 A usual day</v>
@@ -12225,10 +12225,10 @@
     <row r="35" ht="34" customHeight="1">
       <c r="A35" s="3"/>
       <c r="B35" s="29" t="str">
-        <v>Conversation barriers</v>
+        <v>Interaction with peers</v>
       </c>
       <c r="C35" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D35" s="29" t="str">
         <v>03 A usual day</v>
@@ -12238,10 +12238,10 @@
     <row r="36" ht="34" customHeight="1">
       <c r="A36" s="3"/>
       <c r="B36" s="29" t="str">
-        <v>Interaction with peers</v>
+        <v>Peer interaction notes</v>
       </c>
       <c r="C36" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D36" s="29" t="str">
         <v>03 A usual day</v>
@@ -12251,10 +12251,10 @@
     <row r="37" ht="34" customHeight="1">
       <c r="A37" s="3"/>
       <c r="B37" s="29" t="str">
-        <v>Peer interaction notes</v>
+        <v>Interaction with staff</v>
       </c>
       <c r="C37" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D37" s="29" t="str">
         <v>03 A usual day</v>
@@ -12264,10 +12264,10 @@
     <row r="38" ht="34" customHeight="1">
       <c r="A38" s="3"/>
       <c r="B38" s="29" t="str">
-        <v>Interaction with staff</v>
+        <v>Staff interaction notes</v>
       </c>
       <c r="C38" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D38" s="29" t="str">
         <v>03 A usual day</v>
@@ -12277,10 +12277,10 @@
     <row r="39" ht="34" customHeight="1">
       <c r="A39" s="3"/>
       <c r="B39" s="29" t="str">
-        <v>Staff interaction notes</v>
+        <v>Participates in programming</v>
       </c>
       <c r="C39" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D39" s="29" t="str">
         <v>03 A usual day</v>
@@ -12290,10 +12290,10 @@
     <row r="40" ht="34" customHeight="1">
       <c r="A40" s="3"/>
       <c r="B40" s="29" t="str">
-        <v>Participates in programming</v>
+        <v>Programming notes</v>
       </c>
       <c r="C40" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D40" s="29" t="str">
         <v>03 A usual day</v>
@@ -12303,23 +12303,23 @@
     <row r="41" ht="34" customHeight="1">
       <c r="A41" s="3"/>
       <c r="B41" s="29" t="str">
-        <v>Programming notes</v>
+        <v>Physical health concerns</v>
       </c>
       <c r="C41" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D41" s="29" t="str">
-        <v>03 A usual day</v>
+        <v>04 Health and comfort</v>
       </c>
       <c r="E41" s="3"/>
     </row>
     <row r="42" ht="34" customHeight="1">
       <c r="A42" s="3"/>
       <c r="B42" s="29" t="str">
-        <v>Physical health concerns</v>
+        <v>Physical health diagnoses</v>
       </c>
       <c r="C42" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D42" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12329,7 +12329,7 @@
     <row r="43" ht="34" customHeight="1">
       <c r="A43" s="3"/>
       <c r="B43" s="29" t="str">
-        <v>Physical health diagnoses</v>
+        <v>Current health measures</v>
       </c>
       <c r="C43" s="29" t="str">
         <v>Text or notes</v>
@@ -12342,10 +12342,10 @@
     <row r="44" ht="34" customHeight="1">
       <c r="A44" s="3"/>
       <c r="B44" s="29" t="str">
-        <v>Current health measures</v>
+        <v>Diabetic</v>
       </c>
       <c r="C44" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D44" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12355,10 +12355,10 @@
     <row r="45" ht="34" customHeight="1">
       <c r="A45" s="3"/>
       <c r="B45" s="29" t="str">
-        <v>Diabetic</v>
+        <v>Diabetes care details</v>
       </c>
       <c r="C45" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D45" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12368,10 +12368,10 @@
     <row r="46" ht="34" customHeight="1">
       <c r="A46" s="3"/>
       <c r="B46" s="29" t="str">
-        <v>Diabetes care details</v>
+        <v>Special diet</v>
       </c>
       <c r="C46" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D46" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12381,10 +12381,10 @@
     <row r="47" ht="34" customHeight="1">
       <c r="A47" s="3"/>
       <c r="B47" s="29" t="str">
-        <v>Special diet</v>
+        <v>Dietary restrictions</v>
       </c>
       <c r="C47" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D47" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12394,10 +12394,10 @@
     <row r="48" ht="34" customHeight="1">
       <c r="A48" s="3"/>
       <c r="B48" s="29" t="str">
-        <v>Dietary restrictions</v>
+        <v>Skin integrity issue</v>
       </c>
       <c r="C48" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D48" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12407,10 +12407,10 @@
     <row r="49" ht="34" customHeight="1">
       <c r="A49" s="3"/>
       <c r="B49" s="29" t="str">
-        <v>Skin integrity issue</v>
+        <v>Skin integrity details</v>
       </c>
       <c r="C49" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D49" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12420,10 +12420,10 @@
     <row r="50" ht="34" customHeight="1">
       <c r="A50" s="3"/>
       <c r="B50" s="29" t="str">
-        <v>Skin integrity details</v>
+        <v>Dentures</v>
       </c>
       <c r="C50" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D50" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12433,7 +12433,7 @@
     <row r="51" ht="34" customHeight="1">
       <c r="A51" s="3"/>
       <c r="B51" s="29" t="str">
-        <v>Dentures</v>
+        <v>Hearing aids</v>
       </c>
       <c r="C51" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12446,7 +12446,7 @@
     <row r="52" ht="34" customHeight="1">
       <c r="A52" s="3"/>
       <c r="B52" s="29" t="str">
-        <v>Hearing aids</v>
+        <v>Glasses</v>
       </c>
       <c r="C52" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12459,7 +12459,7 @@
     <row r="53" ht="34" customHeight="1">
       <c r="A53" s="3"/>
       <c r="B53" s="29" t="str">
-        <v>Glasses</v>
+        <v>Oxygen</v>
       </c>
       <c r="C53" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12472,7 +12472,7 @@
     <row r="54" ht="34" customHeight="1">
       <c r="A54" s="3"/>
       <c r="B54" s="29" t="str">
-        <v>Oxygen</v>
+        <v>Hospital bed</v>
       </c>
       <c r="C54" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12485,7 +12485,7 @@
     <row r="55" ht="34" customHeight="1">
       <c r="A55" s="3"/>
       <c r="B55" s="29" t="str">
-        <v>Hospital bed</v>
+        <v>CPAP</v>
       </c>
       <c r="C55" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12498,7 +12498,7 @@
     <row r="56" ht="34" customHeight="1">
       <c r="A56" s="3"/>
       <c r="B56" s="29" t="str">
-        <v>CPAP</v>
+        <v>Catheter care</v>
       </c>
       <c r="C56" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12511,7 +12511,7 @@
     <row r="57" ht="34" customHeight="1">
       <c r="A57" s="3"/>
       <c r="B57" s="29" t="str">
-        <v>Catheter care</v>
+        <v>Colostomy</v>
       </c>
       <c r="C57" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12524,7 +12524,7 @@
     <row r="58" ht="34" customHeight="1">
       <c r="A58" s="3"/>
       <c r="B58" s="29" t="str">
-        <v>Colostomy</v>
+        <v>Ileostomy</v>
       </c>
       <c r="C58" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12537,7 +12537,7 @@
     <row r="59" ht="34" customHeight="1">
       <c r="A59" s="3"/>
       <c r="B59" s="29" t="str">
-        <v>Ileostomy</v>
+        <v>Incontinence issues</v>
       </c>
       <c r="C59" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12547,26 +12547,26 @@
       </c>
       <c r="E59" s="3"/>
     </row>
-    <row r="60" ht="34" customHeight="1">
+    <row r="60" ht="44" customHeight="1">
       <c r="A60" s="3"/>
       <c r="B60" s="29" t="str">
-        <v>Incontinence issues</v>
+        <v>Support</v>
       </c>
       <c r="C60" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Client independently changes briefs; Client needs help changing briefs; Client needs briefs changed</v>
       </c>
       <c r="D60" s="29" t="str">
         <v>04 Health and comfort</v>
       </c>
       <c r="E60" s="3"/>
     </row>
-    <row r="61" ht="44" customHeight="1">
+    <row r="61" ht="34" customHeight="1">
       <c r="A61" s="3"/>
       <c r="B61" s="29" t="str">
-        <v>Support</v>
+        <v>Additional health information</v>
       </c>
       <c r="C61" s="29" t="str">
-        <v>Client independently changes briefs; Client needs help changing briefs; Client needs briefs changed</v>
+        <v>Text or notes</v>
       </c>
       <c r="D61" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12576,23 +12576,23 @@
     <row r="62" ht="34" customHeight="1">
       <c r="A62" s="3"/>
       <c r="B62" s="29" t="str">
-        <v>Additional health information</v>
+        <v>Medication compliant</v>
       </c>
       <c r="C62" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D62" s="29" t="str">
-        <v>04 Health and comfort</v>
+        <v>05 Medication</v>
       </c>
       <c r="E62" s="3"/>
     </row>
     <row r="63" ht="34" customHeight="1">
       <c r="A63" s="3"/>
       <c r="B63" s="29" t="str">
-        <v>Medication compliant</v>
+        <v>Date of last medication refusal</v>
       </c>
       <c r="C63" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D63" s="29" t="str">
         <v>05 Medication</v>
@@ -12602,10 +12602,10 @@
     <row r="64" ht="34" customHeight="1">
       <c r="A64" s="3"/>
       <c r="B64" s="29" t="str">
-        <v>Date of last medication refusal</v>
+        <v>Medication refused</v>
       </c>
       <c r="C64" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D64" s="29" t="str">
         <v>05 Medication</v>
@@ -12615,10 +12615,10 @@
     <row r="65" ht="34" customHeight="1">
       <c r="A65" s="3"/>
       <c r="B65" s="29" t="str">
-        <v>Medication refused</v>
+        <v>Refusals in the last 30 days</v>
       </c>
       <c r="C65" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D65" s="29" t="str">
         <v>05 Medication</v>
@@ -12628,10 +12628,10 @@
     <row r="66" ht="34" customHeight="1">
       <c r="A66" s="3"/>
       <c r="B66" s="29" t="str">
-        <v>Refusals in the last 30 days</v>
+        <v>Medications at intake</v>
       </c>
       <c r="C66" s="29" t="str">
-        <v>Whole number</v>
+        <v>One item per line</v>
       </c>
       <c r="D66" s="29" t="str">
         <v>05 Medication</v>
@@ -12641,10 +12641,10 @@
     <row r="67" ht="34" customHeight="1">
       <c r="A67" s="3"/>
       <c r="B67" s="29" t="str">
-        <v>Medications at intake</v>
+        <v>PRN patterns</v>
       </c>
       <c r="C67" s="29" t="str">
-        <v>One item per line</v>
+        <v>Text or notes</v>
       </c>
       <c r="D67" s="29" t="str">
         <v>05 Medication</v>
@@ -12654,10 +12654,10 @@
     <row r="68" ht="34" customHeight="1">
       <c r="A68" s="3"/>
       <c r="B68" s="29" t="str">
-        <v>PRN patterns</v>
+        <v>IM injections</v>
       </c>
       <c r="C68" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D68" s="29" t="str">
         <v>05 Medication</v>
@@ -12667,10 +12667,10 @@
     <row r="69" ht="34" customHeight="1">
       <c r="A69" s="3"/>
       <c r="B69" s="29" t="str">
-        <v>IM injections</v>
+        <v>Injection details</v>
       </c>
       <c r="C69" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D69" s="29" t="str">
         <v>05 Medication</v>
@@ -12680,7 +12680,7 @@
     <row r="70" ht="34" customHeight="1">
       <c r="A70" s="3"/>
       <c r="B70" s="29" t="str">
-        <v>Injection details</v>
+        <v>Injection frequency</v>
       </c>
       <c r="C70" s="29" t="str">
         <v>Text or notes</v>
@@ -12693,7 +12693,7 @@
     <row r="71" ht="34" customHeight="1">
       <c r="A71" s="3"/>
       <c r="B71" s="29" t="str">
-        <v>Injection frequency</v>
+        <v>Last injection</v>
       </c>
       <c r="C71" s="29" t="str">
         <v>Text or notes</v>
@@ -12706,7 +12706,7 @@
     <row r="72" ht="34" customHeight="1">
       <c r="A72" s="3"/>
       <c r="B72" s="29" t="str">
-        <v>Last injection</v>
+        <v>Next injection due</v>
       </c>
       <c r="C72" s="29" t="str">
         <v>Text or notes</v>
@@ -12719,7 +12719,7 @@
     <row r="73" ht="34" customHeight="1">
       <c r="A73" s="3"/>
       <c r="B73" s="29" t="str">
-        <v>Next injection due</v>
+        <v>LAI vs oral</v>
       </c>
       <c r="C73" s="29" t="str">
         <v>Text or notes</v>
@@ -12732,36 +12732,36 @@
     <row r="74" ht="34" customHeight="1">
       <c r="A74" s="3"/>
       <c r="B74" s="29" t="str">
-        <v>LAI vs oral</v>
+        <v>County</v>
       </c>
       <c r="C74" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D74" s="29" t="str">
-        <v>05 Medication</v>
+        <v>06 Living situation</v>
       </c>
       <c r="E74" s="3"/>
     </row>
-    <row r="75" ht="34" customHeight="1">
+    <row r="75" ht="76" customHeight="1">
       <c r="A75" s="3"/>
       <c r="B75" s="29" t="str">
-        <v>County</v>
+        <v>Prior setting type</v>
       </c>
       <c r="C75" s="29" t="str">
-        <v>Text or notes</v>
+        <v>State hospital; Acute psychiatric hospital; IMD / MHRC; Skilled nursing facility; Board and care; Residential program; Jail / forensic setting; Independent or family home; Unhoused; Other</v>
       </c>
       <c r="D75" s="29" t="str">
         <v>06 Living situation</v>
       </c>
       <c r="E75" s="3"/>
     </row>
-    <row r="76" ht="76" customHeight="1">
+    <row r="76" ht="34" customHeight="1">
       <c r="A76" s="3"/>
       <c r="B76" s="29" t="str">
-        <v>Prior setting type</v>
+        <v>Prior placement name</v>
       </c>
       <c r="C76" s="29" t="str">
-        <v>State hospital; Acute psychiatric hospital; IMD / MHRC; Skilled nursing facility; Board and care; Residential program; Jail / forensic setting; Independent or family home; Unhoused; Other</v>
+        <v>Text or notes</v>
       </c>
       <c r="D76" s="29" t="str">
         <v>06 Living situation</v>
@@ -12771,10 +12771,10 @@
     <row r="77" ht="34" customHeight="1">
       <c r="A77" s="3"/>
       <c r="B77" s="29" t="str">
-        <v>Prior placement name</v>
+        <v>Admit date</v>
       </c>
       <c r="C77" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D77" s="29" t="str">
         <v>06 Living situation</v>
@@ -12784,20 +12784,20 @@
     <row r="78" ht="34" customHeight="1">
       <c r="A78" s="3"/>
       <c r="B78" s="29" t="str">
-        <v>Admit date</v>
+        <v>Prior placements</v>
       </c>
       <c r="C78" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D78" s="29" t="str">
-        <v>06 Living situation</v>
+        <v>07 Recent care and history</v>
       </c>
       <c r="E78" s="3"/>
     </row>
     <row r="79" ht="34" customHeight="1">
       <c r="A79" s="3"/>
       <c r="B79" s="29" t="str">
-        <v>Prior placements</v>
+        <v>Prior AWOL / failed placements</v>
       </c>
       <c r="C79" s="29" t="str">
         <v>Text or notes</v>
@@ -12810,10 +12810,10 @@
     <row r="80" ht="34" customHeight="1">
       <c r="A80" s="3"/>
       <c r="B80" s="29" t="str">
-        <v>Prior AWOL / failed placements</v>
+        <v>Prior hospitalizations</v>
       </c>
       <c r="C80" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D80" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -12823,10 +12823,10 @@
     <row r="81" ht="34" customHeight="1">
       <c r="A81" s="3"/>
       <c r="B81" s="29" t="str">
-        <v>Prior hospitalizations</v>
+        <v>Most recent hospitalization</v>
       </c>
       <c r="C81" s="29" t="str">
-        <v>Whole number</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D81" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -12836,10 +12836,10 @@
     <row r="82" ht="34" customHeight="1">
       <c r="A82" s="3"/>
       <c r="B82" s="29" t="str">
-        <v>Most recent hospitalization</v>
+        <v>Prior 5150 / 5250 holds</v>
       </c>
       <c r="C82" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D82" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -12849,7 +12849,7 @@
     <row r="83" ht="34" customHeight="1">
       <c r="A83" s="3"/>
       <c r="B83" s="29" t="str">
-        <v>Prior 5150 / 5250 holds</v>
+        <v>Crisis / ER utilization</v>
       </c>
       <c r="C83" s="29" t="str">
         <v>Text or notes</v>
@@ -12862,20 +12862,20 @@
     <row r="84" ht="34" customHeight="1">
       <c r="A84" s="3"/>
       <c r="B84" s="29" t="str">
-        <v>Crisis / ER utilization</v>
+        <v>History of substance abuse</v>
       </c>
       <c r="C84" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D84" s="29" t="str">
-        <v>07 Recent care and history</v>
+        <v>08 Substance use and recovery</v>
       </c>
       <c r="E84" s="3"/>
     </row>
     <row r="85" ht="34" customHeight="1">
       <c r="A85" s="3"/>
       <c r="B85" s="29" t="str">
-        <v>History of substance abuse</v>
+        <v>Active substance use</v>
       </c>
       <c r="C85" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12888,10 +12888,10 @@
     <row r="86" ht="34" customHeight="1">
       <c r="A86" s="3"/>
       <c r="B86" s="29" t="str">
-        <v>Active substance use</v>
+        <v>Substances</v>
       </c>
       <c r="C86" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Opioids; Amphetamines; Marijuana; Alcohol; Other</v>
       </c>
       <c r="D86" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12901,10 +12901,10 @@
     <row r="87" ht="34" customHeight="1">
       <c r="A87" s="3"/>
       <c r="B87" s="29" t="str">
-        <v>Substances</v>
+        <v>Last substance use</v>
       </c>
       <c r="C87" s="29" t="str">
-        <v>Opioids; Amphetamines; Marijuana; Alcohol; Other</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D87" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12914,10 +12914,10 @@
     <row r="88" ht="34" customHeight="1">
       <c r="A88" s="3"/>
       <c r="B88" s="29" t="str">
-        <v>Last substance use</v>
+        <v>Use pattern</v>
       </c>
       <c r="C88" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Daily; Weekly; Sporadic; Rarely</v>
       </c>
       <c r="D88" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12927,49 +12927,49 @@
     <row r="89" ht="34" customHeight="1">
       <c r="A89" s="3"/>
       <c r="B89" s="29" t="str">
-        <v>Use pattern</v>
+        <v>Effect on baseline behavior</v>
       </c>
       <c r="C89" s="29" t="str">
-        <v>Daily; Weekly; Sporadic; Rarely</v>
+        <v>Text or notes</v>
       </c>
       <c r="D89" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" ht="34" customHeight="1">
+    <row r="90" ht="60" customHeight="1">
       <c r="A90" s="3"/>
       <c r="B90" s="29" t="str">
-        <v>Effect on baseline behavior</v>
+        <v>Longest sobriety in the last five years</v>
       </c>
       <c r="C90" s="29" t="str">
-        <v>Text or notes</v>
+        <v>1 month; 2 months; 3 months; 4 months; 5 months; 6 months; 7 months; 8 months; 9 months; 10 months; 11 months; 1 year; 18 months; 2 years; More than 2 years</v>
       </c>
       <c r="D90" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" ht="60" customHeight="1">
+    <row r="91" ht="44" customHeight="1">
       <c r="A91" s="3"/>
       <c r="B91" s="29" t="str">
-        <v>Longest sobriety in the last five years</v>
+        <v>Acknowledgment of substance-use impact</v>
       </c>
       <c r="C91" s="29" t="str">
-        <v>1 month; 2 months; 3 months; 4 months; 5 months; 6 months; 7 months; 8 months; 9 months; 10 months; 11 months; 1 year; 18 months; 2 years; More than 2 years</v>
+        <v>Acknowledges impact; Partially acknowledges impact; Does not acknowledge impact; Not discussed</v>
       </c>
       <c r="D91" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" ht="44" customHeight="1">
+    <row r="92" ht="34" customHeight="1">
       <c r="A92" s="3"/>
       <c r="B92" s="29" t="str">
-        <v>Acknowledgment of substance-use impact</v>
+        <v>Substance-use impact notes</v>
       </c>
       <c r="C92" s="29" t="str">
-        <v>Acknowledges impact; Partially acknowledges impact; Does not acknowledge impact; Not discussed</v>
+        <v>Text or notes</v>
       </c>
       <c r="D92" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12979,7 +12979,7 @@
     <row r="93" ht="34" customHeight="1">
       <c r="A93" s="3"/>
       <c r="B93" s="29" t="str">
-        <v>Substance-use impact notes</v>
+        <v>Treatment history</v>
       </c>
       <c r="C93" s="29" t="str">
         <v>Text or notes</v>
@@ -12992,10 +12992,10 @@
     <row r="94" ht="34" customHeight="1">
       <c r="A94" s="3"/>
       <c r="B94" s="29" t="str">
-        <v>Treatment history</v>
+        <v>Longest sobriety in the last five years</v>
       </c>
       <c r="C94" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D94" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13005,23 +13005,23 @@
     <row r="95" ht="34" customHeight="1">
       <c r="A95" s="3"/>
       <c r="B95" s="29" t="str">
-        <v>Longest sobriety in the last five years</v>
+        <v>Behavioral history</v>
       </c>
       <c r="C95" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D95" s="29" t="str">
-        <v>08 Substance use and recovery</v>
+        <v>09 Safety and support</v>
       </c>
       <c r="E95" s="3"/>
     </row>
     <row r="96" ht="34" customHeight="1">
       <c r="A96" s="3"/>
       <c r="B96" s="29" t="str">
-        <v>Behavioral history</v>
+        <v>Physical altercations</v>
       </c>
       <c r="C96" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D96" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13031,10 +13031,10 @@
     <row r="97" ht="34" customHeight="1">
       <c r="A97" s="3"/>
       <c r="B97" s="29" t="str">
-        <v>Physical altercations</v>
+        <v>Physical altercation details</v>
       </c>
       <c r="C97" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D97" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13044,10 +13044,10 @@
     <row r="98" ht="34" customHeight="1">
       <c r="A98" s="3"/>
       <c r="B98" s="29" t="str">
-        <v>Physical altercation details</v>
+        <v>History of self-harm</v>
       </c>
       <c r="C98" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D98" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13057,10 +13057,10 @@
     <row r="99" ht="34" customHeight="1">
       <c r="A99" s="3"/>
       <c r="B99" s="29" t="str">
-        <v>History of self-harm</v>
+        <v>Last documented self-harm incident</v>
       </c>
       <c r="C99" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D99" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13070,10 +13070,10 @@
     <row r="100" ht="34" customHeight="1">
       <c r="A100" s="3"/>
       <c r="B100" s="29" t="str">
-        <v>Last documented self-harm incident</v>
+        <v>Current self-harm ideation</v>
       </c>
       <c r="C100" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D100" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13083,10 +13083,10 @@
     <row r="101" ht="34" customHeight="1">
       <c r="A101" s="3"/>
       <c r="B101" s="29" t="str">
-        <v>Current self-harm ideation</v>
+        <v>Current self-harm ideation details</v>
       </c>
       <c r="C101" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D101" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13096,7 +13096,7 @@
     <row r="102" ht="34" customHeight="1">
       <c r="A102" s="3"/>
       <c r="B102" s="29" t="str">
-        <v>Current self-harm ideation details</v>
+        <v>Current safety measures</v>
       </c>
       <c r="C102" s="29" t="str">
         <v>Text or notes</v>
@@ -13109,10 +13109,10 @@
     <row r="103" ht="34" customHeight="1">
       <c r="A103" s="3"/>
       <c r="B103" s="29" t="str">
-        <v>Current safety measures</v>
+        <v>History of assaults</v>
       </c>
       <c r="C103" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D103" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13122,10 +13122,10 @@
     <row r="104" ht="34" customHeight="1">
       <c r="A104" s="3"/>
       <c r="B104" s="29" t="str">
-        <v>History of assaults</v>
+        <v>Most recent assault</v>
       </c>
       <c r="C104" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D104" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13135,10 +13135,10 @@
     <row r="105" ht="34" customHeight="1">
       <c r="A105" s="3"/>
       <c r="B105" s="29" t="str">
-        <v>Most recent assault</v>
+        <v>Assaults in the last two years</v>
       </c>
       <c r="C105" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D105" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13148,10 +13148,10 @@
     <row r="106" ht="34" customHeight="1">
       <c r="A106" s="3"/>
       <c r="B106" s="29" t="str">
-        <v>Assaults in the last two years</v>
+        <v>History of elopement</v>
       </c>
       <c r="C106" s="29" t="str">
-        <v>Whole number</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D106" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13161,10 +13161,10 @@
     <row r="107" ht="34" customHeight="1">
       <c r="A107" s="3"/>
       <c r="B107" s="29" t="str">
-        <v>History of elopement</v>
+        <v>Elopement risk</v>
       </c>
       <c r="C107" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D107" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13174,7 +13174,7 @@
     <row r="108" ht="34" customHeight="1">
       <c r="A108" s="3"/>
       <c r="B108" s="29" t="str">
-        <v>Elopement risk</v>
+        <v>SI / HI history</v>
       </c>
       <c r="C108" s="29" t="str">
         <v>Text or notes</v>
@@ -13187,7 +13187,7 @@
     <row r="109" ht="34" customHeight="1">
       <c r="A109" s="3"/>
       <c r="B109" s="29" t="str">
-        <v>SI / HI history</v>
+        <v>Triggers and what helps</v>
       </c>
       <c r="C109" s="29" t="str">
         <v>Text or notes</v>
@@ -13200,7 +13200,7 @@
     <row r="110" ht="34" customHeight="1">
       <c r="A110" s="3"/>
       <c r="B110" s="29" t="str">
-        <v>Triggers and what helps</v>
+        <v>Aggression risk</v>
       </c>
       <c r="C110" s="29" t="str">
         <v>Text or notes</v>
@@ -13213,7 +13213,7 @@
     <row r="111" ht="34" customHeight="1">
       <c r="A111" s="3"/>
       <c r="B111" s="29" t="str">
-        <v>Aggression risk</v>
+        <v>Responds to internal stimuli</v>
       </c>
       <c r="C111" s="29" t="str">
         <v>Text or notes</v>
@@ -13226,7 +13226,7 @@
     <row r="112" ht="34" customHeight="1">
       <c r="A112" s="3"/>
       <c r="B112" s="29" t="str">
-        <v>Responds to internal stimuli</v>
+        <v>Auditory hallucinations</v>
       </c>
       <c r="C112" s="29" t="str">
         <v>Text or notes</v>
@@ -13239,7 +13239,7 @@
     <row r="113" ht="34" customHeight="1">
       <c r="A113" s="3"/>
       <c r="B113" s="29" t="str">
-        <v>Auditory hallucinations</v>
+        <v>Nature of auditory hallucinations</v>
       </c>
       <c r="C113" s="29" t="str">
         <v>Text or notes</v>
@@ -13252,7 +13252,7 @@
     <row r="114" ht="34" customHeight="1">
       <c r="A114" s="3"/>
       <c r="B114" s="29" t="str">
-        <v>Nature of auditory hallucinations</v>
+        <v>Current auditory frequency</v>
       </c>
       <c r="C114" s="29" t="str">
         <v>Text or notes</v>
@@ -13265,7 +13265,7 @@
     <row r="115" ht="34" customHeight="1">
       <c r="A115" s="3"/>
       <c r="B115" s="29" t="str">
-        <v>Current auditory frequency</v>
+        <v>Auditory triggers</v>
       </c>
       <c r="C115" s="29" t="str">
         <v>Text or notes</v>
@@ -13278,7 +13278,7 @@
     <row r="116" ht="34" customHeight="1">
       <c r="A116" s="3"/>
       <c r="B116" s="29" t="str">
-        <v>Auditory triggers</v>
+        <v>Visual hallucinations</v>
       </c>
       <c r="C116" s="29" t="str">
         <v>Text or notes</v>
@@ -13291,7 +13291,7 @@
     <row r="117" ht="34" customHeight="1">
       <c r="A117" s="3"/>
       <c r="B117" s="29" t="str">
-        <v>Visual hallucinations</v>
+        <v>Nature and frequency of visual hallucinations</v>
       </c>
       <c r="C117" s="29" t="str">
         <v>Text or notes</v>
@@ -13304,7 +13304,7 @@
     <row r="118" ht="34" customHeight="1">
       <c r="A118" s="3"/>
       <c r="B118" s="29" t="str">
-        <v>Nature and frequency of visual hallucinations</v>
+        <v>Recent visual hallucinations</v>
       </c>
       <c r="C118" s="29" t="str">
         <v>Text or notes</v>
@@ -13317,7 +13317,7 @@
     <row r="119" ht="34" customHeight="1">
       <c r="A119" s="3"/>
       <c r="B119" s="29" t="str">
-        <v>Recent visual hallucinations</v>
+        <v>Olfactory hallucinations</v>
       </c>
       <c r="C119" s="29" t="str">
         <v>Text or notes</v>
@@ -13330,7 +13330,7 @@
     <row r="120" ht="34" customHeight="1">
       <c r="A120" s="3"/>
       <c r="B120" s="29" t="str">
-        <v>Olfactory hallucinations</v>
+        <v>Olfactory hallucination details</v>
       </c>
       <c r="C120" s="29" t="str">
         <v>Text or notes</v>
@@ -13343,7 +13343,7 @@
     <row r="121" ht="34" customHeight="1">
       <c r="A121" s="3"/>
       <c r="B121" s="29" t="str">
-        <v>Olfactory hallucination details</v>
+        <v>Impact of olfactory hallucinations</v>
       </c>
       <c r="C121" s="29" t="str">
         <v>Text or notes</v>
@@ -13356,7 +13356,7 @@
     <row r="122" ht="34" customHeight="1">
       <c r="A122" s="3"/>
       <c r="B122" s="29" t="str">
-        <v>Impact of olfactory hallucinations</v>
+        <v>Tactile hallucinations</v>
       </c>
       <c r="C122" s="29" t="str">
         <v>Text or notes</v>
@@ -13369,7 +13369,7 @@
     <row r="123" ht="34" customHeight="1">
       <c r="A123" s="3"/>
       <c r="B123" s="29" t="str">
-        <v>Tactile hallucinations</v>
+        <v>Tactile hallucination details</v>
       </c>
       <c r="C123" s="29" t="str">
         <v>Text or notes</v>
@@ -13382,7 +13382,7 @@
     <row r="124" ht="34" customHeight="1">
       <c r="A124" s="3"/>
       <c r="B124" s="29" t="str">
-        <v>Tactile hallucination details</v>
+        <v>Tactile hallucination frequency</v>
       </c>
       <c r="C124" s="29" t="str">
         <v>Text or notes</v>
@@ -13395,7 +13395,7 @@
     <row r="125" ht="34" customHeight="1">
       <c r="A125" s="3"/>
       <c r="B125" s="29" t="str">
-        <v>Tactile hallucination frequency</v>
+        <v>Gustatory hallucinations</v>
       </c>
       <c r="C125" s="29" t="str">
         <v>Text or notes</v>
@@ -13408,7 +13408,7 @@
     <row r="126" ht="34" customHeight="1">
       <c r="A126" s="3"/>
       <c r="B126" s="29" t="str">
-        <v>Gustatory hallucinations</v>
+        <v>Gustatory hallucination details</v>
       </c>
       <c r="C126" s="29" t="str">
         <v>Text or notes</v>
@@ -13421,7 +13421,7 @@
     <row r="127" ht="34" customHeight="1">
       <c r="A127" s="3"/>
       <c r="B127" s="29" t="str">
-        <v>Gustatory hallucination details</v>
+        <v>Hallucination coping strategies</v>
       </c>
       <c r="C127" s="29" t="str">
         <v>Text or notes</v>
@@ -13434,7 +13434,7 @@
     <row r="128" ht="34" customHeight="1">
       <c r="A128" s="3"/>
       <c r="B128" s="29" t="str">
-        <v>Hallucination coping strategies</v>
+        <v>Hallucination distress or impairment</v>
       </c>
       <c r="C128" s="29" t="str">
         <v>Text or notes</v>
@@ -13447,7 +13447,7 @@
     <row r="129" ht="34" customHeight="1">
       <c r="A129" s="3"/>
       <c r="B129" s="29" t="str">
-        <v>Hallucination distress or impairment</v>
+        <v>Impact on daily functioning</v>
       </c>
       <c r="C129" s="29" t="str">
         <v>Text or notes</v>
@@ -13460,7 +13460,7 @@
     <row r="130" ht="34" customHeight="1">
       <c r="A130" s="3"/>
       <c r="B130" s="29" t="str">
-        <v>Impact on daily functioning</v>
+        <v>Professional discussion and treatment</v>
       </c>
       <c r="C130" s="29" t="str">
         <v>Text or notes</v>
@@ -13473,23 +13473,23 @@
     <row r="131" ht="34" customHeight="1">
       <c r="A131" s="3"/>
       <c r="B131" s="29" t="str">
-        <v>Professional discussion and treatment</v>
+        <v>Conserved status</v>
       </c>
       <c r="C131" s="29" t="str">
-        <v>Text or notes</v>
+        <v>LPS; TCon; Murphy's; Non-Conserved</v>
       </c>
       <c r="D131" s="29" t="str">
-        <v>09 Safety and support</v>
+        <v>10 Decisions and legal support</v>
       </c>
       <c r="E131" s="3"/>
     </row>
     <row r="132" ht="34" customHeight="1">
       <c r="A132" s="3"/>
       <c r="B132" s="29" t="str">
-        <v>Conserved status</v>
+        <v>Conservator name</v>
       </c>
       <c r="C132" s="29" t="str">
-        <v>LPS; TCon; Murphy's; Non-Conserved</v>
+        <v>Text or notes</v>
       </c>
       <c r="D132" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13499,7 +13499,7 @@
     <row r="133" ht="34" customHeight="1">
       <c r="A133" s="3"/>
       <c r="B133" s="29" t="str">
-        <v>Conservator name</v>
+        <v>Conservatorship details</v>
       </c>
       <c r="C133" s="29" t="str">
         <v>Text or notes</v>
@@ -13512,7 +13512,7 @@
     <row r="134" ht="34" customHeight="1">
       <c r="A134" s="3"/>
       <c r="B134" s="29" t="str">
-        <v>Conservatorship details</v>
+        <v>Hold type</v>
       </c>
       <c r="C134" s="29" t="str">
         <v>Text or notes</v>
@@ -13525,10 +13525,10 @@
     <row r="135" ht="34" customHeight="1">
       <c r="A135" s="3"/>
       <c r="B135" s="29" t="str">
-        <v>Hold type</v>
+        <v>Forensic involvement</v>
       </c>
       <c r="C135" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D135" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13538,10 +13538,10 @@
     <row r="136" ht="34" customHeight="1">
       <c r="A136" s="3"/>
       <c r="B136" s="29" t="str">
-        <v>Forensic involvement</v>
+        <v>Forensic involvement details</v>
       </c>
       <c r="C136" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D136" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13551,10 +13551,10 @@
     <row r="137" ht="34" customHeight="1">
       <c r="A137" s="3"/>
       <c r="B137" s="29" t="str">
-        <v>Forensic involvement details</v>
+        <v>History of arrest</v>
       </c>
       <c r="C137" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D137" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13564,10 +13564,10 @@
     <row r="138" ht="34" customHeight="1">
       <c r="A138" s="3"/>
       <c r="B138" s="29" t="str">
-        <v>History of arrest</v>
+        <v>Most recent arrest date</v>
       </c>
       <c r="C138" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D138" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13577,10 +13577,10 @@
     <row r="139" ht="34" customHeight="1">
       <c r="A139" s="3"/>
       <c r="B139" s="29" t="str">
-        <v>Most recent arrest date</v>
+        <v>Most recent arrest charge</v>
       </c>
       <c r="C139" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D139" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13590,7 +13590,7 @@
     <row r="140" ht="34" customHeight="1">
       <c r="A140" s="3"/>
       <c r="B140" s="29" t="str">
-        <v>Most recent arrest charge</v>
+        <v>Time in jail</v>
       </c>
       <c r="C140" s="29" t="str">
         <v>Text or notes</v>
@@ -13603,10 +13603,10 @@
     <row r="141" ht="34" customHeight="1">
       <c r="A141" s="3"/>
       <c r="B141" s="29" t="str">
-        <v>Time in jail</v>
+        <v>Arrest in the last two years</v>
       </c>
       <c r="C141" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D141" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13616,10 +13616,10 @@
     <row r="142" ht="34" customHeight="1">
       <c r="A142" s="3"/>
       <c r="B142" s="29" t="str">
-        <v>Arrest in the last two years</v>
+        <v>Recent arrest details</v>
       </c>
       <c r="C142" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D142" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13629,10 +13629,10 @@
     <row r="143" ht="34" customHeight="1">
       <c r="A143" s="3"/>
       <c r="B143" s="29" t="str">
-        <v>Recent arrest details</v>
+        <v>Total recorded arrests</v>
       </c>
       <c r="C143" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D143" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13642,10 +13642,10 @@
     <row r="144" ht="34" customHeight="1">
       <c r="A144" s="3"/>
       <c r="B144" s="29" t="str">
-        <v>Total recorded arrests</v>
+        <v>PC 290 registration</v>
       </c>
       <c r="C144" s="29" t="str">
-        <v>Whole number</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D144" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13655,7 +13655,7 @@
     <row r="145" ht="34" customHeight="1">
       <c r="A145" s="3"/>
       <c r="B145" s="29" t="str">
-        <v>PC 290 registration</v>
+        <v>Arson history</v>
       </c>
       <c r="C145" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13668,7 +13668,7 @@
     <row r="146" ht="34" customHeight="1">
       <c r="A146" s="3"/>
       <c r="B146" s="29" t="str">
-        <v>Arson history</v>
+        <v>Diversion client</v>
       </c>
       <c r="C146" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13681,10 +13681,10 @@
     <row r="147" ht="34" customHeight="1">
       <c r="A147" s="3"/>
       <c r="B147" s="29" t="str">
-        <v>Diversion client</v>
+        <v>Court requirements</v>
       </c>
       <c r="C147" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D147" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13694,7 +13694,7 @@
     <row r="148" ht="34" customHeight="1">
       <c r="A148" s="3"/>
       <c r="B148" s="29" t="str">
-        <v>Court requirements</v>
+        <v>Court dates</v>
       </c>
       <c r="C148" s="29" t="str">
         <v>Text or notes</v>
@@ -13707,7 +13707,7 @@
     <row r="149" ht="34" customHeight="1">
       <c r="A149" s="3"/>
       <c r="B149" s="29" t="str">
-        <v>Court dates</v>
+        <v>Probation / parole / justice</v>
       </c>
       <c r="C149" s="29" t="str">
         <v>Text or notes</v>
@@ -13720,20 +13720,20 @@
     <row r="150" ht="34" customHeight="1">
       <c r="A150" s="3"/>
       <c r="B150" s="29" t="str">
-        <v>Probation / parole / justice</v>
+        <v>Family involvement</v>
       </c>
       <c r="C150" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D150" s="29" t="str">
-        <v>10 Decisions and legal support</v>
+        <v>11 What matters next</v>
       </c>
       <c r="E150" s="3"/>
     </row>
     <row r="151" ht="34" customHeight="1">
       <c r="A151" s="3"/>
       <c r="B151" s="29" t="str">
-        <v>Family involvement</v>
+        <v>Friendships and social connections</v>
       </c>
       <c r="C151" s="29" t="str">
         <v>Text or notes</v>
@@ -13746,7 +13746,7 @@
     <row r="152" ht="34" customHeight="1">
       <c r="A152" s="3"/>
       <c r="B152" s="29" t="str">
-        <v>Friendships and social connections</v>
+        <v>Prior living situation</v>
       </c>
       <c r="C152" s="29" t="str">
         <v>Text or notes</v>
@@ -13759,7 +13759,7 @@
     <row r="153" ht="34" customHeight="1">
       <c r="A153" s="3"/>
       <c r="B153" s="29" t="str">
-        <v>Prior living situation</v>
+        <v>Housing history</v>
       </c>
       <c r="C153" s="29" t="str">
         <v>Text or notes</v>
@@ -13772,7 +13772,7 @@
     <row r="154" ht="34" customHeight="1">
       <c r="A154" s="3"/>
       <c r="B154" s="29" t="str">
-        <v>Housing history</v>
+        <v>Benefits / income status</v>
       </c>
       <c r="C154" s="29" t="str">
         <v>Text or notes</v>
@@ -13785,7 +13785,7 @@
     <row r="155" ht="34" customHeight="1">
       <c r="A155" s="3"/>
       <c r="B155" s="29" t="str">
-        <v>Benefits / income status</v>
+        <v>Preferred facility characteristics</v>
       </c>
       <c r="C155" s="29" t="str">
         <v>Text or notes</v>
@@ -13798,7 +13798,7 @@
     <row r="156" ht="34" customHeight="1">
       <c r="A156" s="3"/>
       <c r="B156" s="29" t="str">
-        <v>Preferred facility characteristics</v>
+        <v>Discharge planning goals</v>
       </c>
       <c r="C156" s="29" t="str">
         <v>Text or notes</v>
@@ -13811,7 +13811,7 @@
     <row r="157" ht="34" customHeight="1">
       <c r="A157" s="3"/>
       <c r="B157" s="29" t="str">
-        <v>Discharge planning goals</v>
+        <v>Placement preferences and concerns</v>
       </c>
       <c r="C157" s="29" t="str">
         <v>Text or notes</v>
@@ -13824,20 +13824,20 @@
     <row r="158" ht="34" customHeight="1">
       <c r="A158" s="3"/>
       <c r="B158" s="29" t="str">
-        <v>Placement preferences and concerns</v>
+        <v>Additional information</v>
       </c>
       <c r="C158" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D158" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>12 Anything else</v>
       </c>
       <c r="E158" s="3"/>
     </row>
     <row r="159" ht="34" customHeight="1">
       <c r="A159" s="3"/>
       <c r="B159" s="29" t="str">
-        <v>Additional information</v>
+        <v>Placement questions or concerns</v>
       </c>
       <c r="C159" s="29" t="str">
         <v>Text or notes</v>
@@ -13850,7 +13850,7 @@
     <row r="160" ht="34" customHeight="1">
       <c r="A160" s="3"/>
       <c r="B160" s="29" t="str">
-        <v>Placement questions or concerns</v>
+        <v>Assessment notes</v>
       </c>
       <c r="C160" s="29" t="str">
         <v>Text or notes</v>
@@ -13860,17 +13860,11 @@
       </c>
       <c r="E160" s="3"/>
     </row>
-    <row r="161" ht="34" customHeight="1">
+    <row r="161">
       <c r="A161" s="3"/>
-      <c r="B161" s="29" t="str">
-        <v>Assessment notes</v>
-      </c>
-      <c r="C161" s="29" t="str">
-        <v>Text or notes</v>
-      </c>
-      <c r="D161" s="29" t="str">
-        <v>12 Anything else</v>
-      </c>
+      <c r="B161" s="3"/>
+      <c r="C161" s="3"/>
+      <c r="D161" s="3"/>
       <c r="E161" s="3"/>
     </row>
     <row r="162">
@@ -14114,18 +14108,36 @@
         <v>Optional</v>
       </c>
     </row>
-    <row r="15" ht="34" customHeight="1">
+    <row r="15" ht="39" customHeight="1" hidden="1">
       <c r="A15" s="3" t="str">
         <v>resident_number</v>
       </c>
-      <c r="B15" s="13" t="str">
-        <v>Resident number</v>
-      </c>
-      <c r="C15" t="str" s="50"/>
-      <c r="D15" t="str" s="48"/>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="12"/>
+              <color rgb="FF233B32"/>
+            </rPr>
+            <t>Resident number</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="0"/>
+              <sz val="10"/>
+              <color rgb="FF59675F"/>
+            </rPr>
+            <t xml:space="preserve">
+Reference only.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C15" s="23" t="str"/>
+      <c r="D15" s="15" t="str"/>
       <c r="E15" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C15))&gt;0,LEN(TRIM(D15))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D15))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D15))&gt;0)),"Explain why",IF(LEN(TRIM(C15))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
+        <f>"Reference only"</f>
+        <v>Reference only</v>
       </c>
     </row>
     <row r="16" ht="39" customHeight="1">

</xml_diff>

<commit_message>
Fix handoff snapshots and improve chart document access (#164)
* Fix handoff placement snapshots and assessment return behavior

* Keep document upload visible above saved charts

* Keep resident numbers internal to records and workbook recovery

* Refresh registries for chart and handoff fixes
</commit_message>
<xml_diff>
--- a/public/templates/pipeline-assessment-workbook.xlsx
+++ b/public/templates/pipeline-assessment-workbook.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R6d07ac8bfe794c3e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="Red20ff0add3b4b2b"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R3d4b1515133243a7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="Rc9a0a5f88eb447bb"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Rb8ad1d3d91504ba8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="R8d123d25cf9b485b"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="R2088732c87bd4722"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="R511995de280b4cb4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Rcbe07b2a3d2d493e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R01ce518e638e4e9d"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="Ree8be1cb492b4089"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R6b3b45a78eda492e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="Re757407f23304570"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="Rea432ea5061f4986" state="veryHidden"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="Reedcadc7684d4c32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Raba6eabfa2c0467e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="R6d3c53b35ab2451e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R19ade892a9e9487f"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="R8b151a64b22b4af9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Rbf3a71609d6743d6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="Rfd66ce774fc94e99"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="R387c3a8951cc4843"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="Rf20811a60f024902"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Red12527f76d5406e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R7fbf3f91f3294651"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="R647a55aefa954e92"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="Rc2f47f3707024ecf"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="R78cf9d19b64649d0"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="R5721e6970feb49ce" state="veryHidden"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="Rfcdada3041aa4328"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Confirm the basics'!$B$1:$E$16</definedName>
@@ -7880,7 +7880,7 @@
         <v>Questionnaire fingerprint</v>
       </c>
       <c r="B2" t="str">
-        <v>90679cc7ae50bccf1ece35ed905f975b61e0b1af883344804bb08d07b0fc4ea8</v>
+        <v>44ee09c0df7abcd44bc76e520cf2da27dbdbae70d31aef5d40cbd527d55bed9c</v>
       </c>
     </row>
     <row r="3">
@@ -11949,26 +11949,26 @@
       </c>
       <c r="E13" s="3"/>
     </row>
-    <row r="14" ht="34" customHeight="1">
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="3"/>
       <c r="B14" s="29" t="str">
-        <v>Resident number</v>
+        <v>Diagnosis categories</v>
       </c>
       <c r="C14" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Schizophrenia; Schizoaffective disorder; Bipolar disorder; Personality disorder; Substance use disorder; Psychosis; Delusional disorder; Physical health condition; Other</v>
       </c>
       <c r="D14" s="29" t="str">
-        <v>01 Confirm the basics</v>
+        <v>02 How things are now</v>
       </c>
       <c r="E14" s="3"/>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15" ht="34" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="29" t="str">
-        <v>Diagnosis categories</v>
+        <v>Other diagnosis</v>
       </c>
       <c r="C15" s="29" t="str">
-        <v>Schizophrenia; Schizoaffective disorder; Bipolar disorder; Personality disorder; Substance use disorder; Psychosis; Delusional disorder; Physical health condition; Other</v>
+        <v>Text or notes</v>
       </c>
       <c r="D15" s="29" t="str">
         <v>02 How things are now</v>
@@ -11978,10 +11978,10 @@
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="29" t="str">
-        <v>Other diagnosis</v>
+        <v>Secondary diagnosis</v>
       </c>
       <c r="C16" s="29" t="str">
-        <v>Text or notes</v>
+        <v>One item per line</v>
       </c>
       <c r="D16" s="29" t="str">
         <v>02 How things are now</v>
@@ -11991,10 +11991,10 @@
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="3"/>
       <c r="B17" s="29" t="str">
-        <v>Secondary diagnosis</v>
+        <v>Current symptoms</v>
       </c>
       <c r="C17" s="29" t="str">
-        <v>One item per line</v>
+        <v>Text or notes</v>
       </c>
       <c r="D17" s="29" t="str">
         <v>02 How things are now</v>
@@ -12004,7 +12004,7 @@
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="29" t="str">
-        <v>Current symptoms</v>
+        <v>Cognition / orientation</v>
       </c>
       <c r="C18" s="29" t="str">
         <v>Text or notes</v>
@@ -12017,7 +12017,7 @@
     <row r="19" ht="34" customHeight="1">
       <c r="A19" s="3"/>
       <c r="B19" s="29" t="str">
-        <v>Cognition / orientation</v>
+        <v>Primary diagnosis</v>
       </c>
       <c r="C19" s="29" t="str">
         <v>Text or notes</v>
@@ -12030,7 +12030,7 @@
     <row r="20" ht="34" customHeight="1">
       <c r="A20" s="3"/>
       <c r="B20" s="29" t="str">
-        <v>Primary diagnosis</v>
+        <v>Acuity level</v>
       </c>
       <c r="C20" s="29" t="str">
         <v>Text or notes</v>
@@ -12043,23 +12043,23 @@
     <row r="21" ht="34" customHeight="1">
       <c r="A21" s="3"/>
       <c r="B21" s="29" t="str">
-        <v>Acuity level</v>
+        <v>Ability to dress</v>
       </c>
       <c r="C21" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Independent; Some assistance; Total assistance</v>
       </c>
       <c r="D21" s="29" t="str">
-        <v>02 How things are now</v>
+        <v>03 A usual day</v>
       </c>
       <c r="E21" s="3"/>
     </row>
     <row r="22" ht="34" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="29" t="str">
-        <v>Ability to dress</v>
+        <v>Dressing assistance needed</v>
       </c>
       <c r="C22" s="29" t="str">
-        <v>Independent; Some assistance; Total assistance</v>
+        <v>Text or notes</v>
       </c>
       <c r="D22" s="29" t="str">
         <v>03 A usual day</v>
@@ -12069,10 +12069,10 @@
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="29" t="str">
-        <v>Dressing assistance needed</v>
+        <v>Ability to bathe</v>
       </c>
       <c r="C23" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Independent; Some assistance; Total assistance</v>
       </c>
       <c r="D23" s="29" t="str">
         <v>03 A usual day</v>
@@ -12082,10 +12082,10 @@
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="29" t="str">
-        <v>Ability to bathe</v>
+        <v>Bathing assistance needed</v>
       </c>
       <c r="C24" s="29" t="str">
-        <v>Independent; Some assistance; Total assistance</v>
+        <v>Text or notes</v>
       </c>
       <c r="D24" s="29" t="str">
         <v>03 A usual day</v>
@@ -12095,10 +12095,10 @@
     <row r="25" ht="34" customHeight="1">
       <c r="A25" s="3"/>
       <c r="B25" s="29" t="str">
-        <v>Bathing assistance needed</v>
+        <v>Overall hygiene</v>
       </c>
       <c r="C25" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D25" s="29" t="str">
         <v>03 A usual day</v>
@@ -12108,10 +12108,10 @@
     <row r="26" ht="34" customHeight="1">
       <c r="A26" s="3"/>
       <c r="B26" s="29" t="str">
-        <v>Overall hygiene</v>
+        <v>ADL needs</v>
       </c>
       <c r="C26" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D26" s="29" t="str">
         <v>03 A usual day</v>
@@ -12121,7 +12121,7 @@
     <row r="27" ht="34" customHeight="1">
       <c r="A27" s="3"/>
       <c r="B27" s="29" t="str">
-        <v>ADL needs</v>
+        <v>Prompting level</v>
       </c>
       <c r="C27" s="29" t="str">
         <v>Text or notes</v>
@@ -12134,7 +12134,7 @@
     <row r="28" ht="34" customHeight="1">
       <c r="A28" s="3"/>
       <c r="B28" s="29" t="str">
-        <v>Prompting level</v>
+        <v>Self-care status</v>
       </c>
       <c r="C28" s="29" t="str">
         <v>Text or notes</v>
@@ -12147,10 +12147,10 @@
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="3"/>
       <c r="B29" s="29" t="str">
-        <v>Self-care status</v>
+        <v>Ambulatory</v>
       </c>
       <c r="C29" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D29" s="29" t="str">
         <v>03 A usual day</v>
@@ -12160,10 +12160,10 @@
     <row r="30" ht="34" customHeight="1">
       <c r="A30" s="3"/>
       <c r="B30" s="29" t="str">
-        <v>Ambulatory</v>
+        <v>Type of device</v>
       </c>
       <c r="C30" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D30" s="29" t="str">
         <v>03 A usual day</v>
@@ -12173,10 +12173,10 @@
     <row r="31" ht="34" customHeight="1">
       <c r="A31" s="3"/>
       <c r="B31" s="29" t="str">
-        <v>Type of device</v>
+        <v>Language barrier</v>
       </c>
       <c r="C31" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D31" s="29" t="str">
         <v>03 A usual day</v>
@@ -12186,10 +12186,10 @@
     <row r="32" ht="34" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="29" t="str">
-        <v>Language barrier</v>
+        <v>Language support needed</v>
       </c>
       <c r="C32" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D32" s="29" t="str">
         <v>03 A usual day</v>
@@ -12199,10 +12199,10 @@
     <row r="33" ht="34" customHeight="1">
       <c r="A33" s="3"/>
       <c r="B33" s="29" t="str">
-        <v>Language support needed</v>
+        <v>Can hold a linear conversation</v>
       </c>
       <c r="C33" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D33" s="29" t="str">
         <v>03 A usual day</v>
@@ -12212,10 +12212,10 @@
     <row r="34" ht="34" customHeight="1">
       <c r="A34" s="3"/>
       <c r="B34" s="29" t="str">
-        <v>Can hold a linear conversation</v>
+        <v>Conversation barriers</v>
       </c>
       <c r="C34" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D34" s="29" t="str">
         <v>03 A usual day</v>
@@ -12225,10 +12225,10 @@
     <row r="35" ht="34" customHeight="1">
       <c r="A35" s="3"/>
       <c r="B35" s="29" t="str">
-        <v>Conversation barriers</v>
+        <v>Interaction with peers</v>
       </c>
       <c r="C35" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D35" s="29" t="str">
         <v>03 A usual day</v>
@@ -12238,10 +12238,10 @@
     <row r="36" ht="34" customHeight="1">
       <c r="A36" s="3"/>
       <c r="B36" s="29" t="str">
-        <v>Interaction with peers</v>
+        <v>Peer interaction notes</v>
       </c>
       <c r="C36" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D36" s="29" t="str">
         <v>03 A usual day</v>
@@ -12251,10 +12251,10 @@
     <row r="37" ht="34" customHeight="1">
       <c r="A37" s="3"/>
       <c r="B37" s="29" t="str">
-        <v>Peer interaction notes</v>
+        <v>Interaction with staff</v>
       </c>
       <c r="C37" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D37" s="29" t="str">
         <v>03 A usual day</v>
@@ -12264,10 +12264,10 @@
     <row r="38" ht="34" customHeight="1">
       <c r="A38" s="3"/>
       <c r="B38" s="29" t="str">
-        <v>Interaction with staff</v>
+        <v>Staff interaction notes</v>
       </c>
       <c r="C38" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D38" s="29" t="str">
         <v>03 A usual day</v>
@@ -12277,10 +12277,10 @@
     <row r="39" ht="34" customHeight="1">
       <c r="A39" s="3"/>
       <c r="B39" s="29" t="str">
-        <v>Staff interaction notes</v>
+        <v>Participates in programming</v>
       </c>
       <c r="C39" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D39" s="29" t="str">
         <v>03 A usual day</v>
@@ -12290,10 +12290,10 @@
     <row r="40" ht="34" customHeight="1">
       <c r="A40" s="3"/>
       <c r="B40" s="29" t="str">
-        <v>Participates in programming</v>
+        <v>Programming notes</v>
       </c>
       <c r="C40" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D40" s="29" t="str">
         <v>03 A usual day</v>
@@ -12303,23 +12303,23 @@
     <row r="41" ht="34" customHeight="1">
       <c r="A41" s="3"/>
       <c r="B41" s="29" t="str">
-        <v>Programming notes</v>
+        <v>Physical health concerns</v>
       </c>
       <c r="C41" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D41" s="29" t="str">
-        <v>03 A usual day</v>
+        <v>04 Health and comfort</v>
       </c>
       <c r="E41" s="3"/>
     </row>
     <row r="42" ht="34" customHeight="1">
       <c r="A42" s="3"/>
       <c r="B42" s="29" t="str">
-        <v>Physical health concerns</v>
+        <v>Physical health diagnoses</v>
       </c>
       <c r="C42" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D42" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12329,7 +12329,7 @@
     <row r="43" ht="34" customHeight="1">
       <c r="A43" s="3"/>
       <c r="B43" s="29" t="str">
-        <v>Physical health diagnoses</v>
+        <v>Current health measures</v>
       </c>
       <c r="C43" s="29" t="str">
         <v>Text or notes</v>
@@ -12342,10 +12342,10 @@
     <row r="44" ht="34" customHeight="1">
       <c r="A44" s="3"/>
       <c r="B44" s="29" t="str">
-        <v>Current health measures</v>
+        <v>Diabetic</v>
       </c>
       <c r="C44" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D44" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12355,10 +12355,10 @@
     <row r="45" ht="34" customHeight="1">
       <c r="A45" s="3"/>
       <c r="B45" s="29" t="str">
-        <v>Diabetic</v>
+        <v>Diabetes care details</v>
       </c>
       <c r="C45" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D45" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12368,10 +12368,10 @@
     <row r="46" ht="34" customHeight="1">
       <c r="A46" s="3"/>
       <c r="B46" s="29" t="str">
-        <v>Diabetes care details</v>
+        <v>Special diet</v>
       </c>
       <c r="C46" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D46" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12381,10 +12381,10 @@
     <row r="47" ht="34" customHeight="1">
       <c r="A47" s="3"/>
       <c r="B47" s="29" t="str">
-        <v>Special diet</v>
+        <v>Dietary restrictions</v>
       </c>
       <c r="C47" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D47" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12394,10 +12394,10 @@
     <row r="48" ht="34" customHeight="1">
       <c r="A48" s="3"/>
       <c r="B48" s="29" t="str">
-        <v>Dietary restrictions</v>
+        <v>Skin integrity issue</v>
       </c>
       <c r="C48" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D48" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12407,10 +12407,10 @@
     <row r="49" ht="34" customHeight="1">
       <c r="A49" s="3"/>
       <c r="B49" s="29" t="str">
-        <v>Skin integrity issue</v>
+        <v>Skin integrity details</v>
       </c>
       <c r="C49" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D49" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12420,10 +12420,10 @@
     <row r="50" ht="34" customHeight="1">
       <c r="A50" s="3"/>
       <c r="B50" s="29" t="str">
-        <v>Skin integrity details</v>
+        <v>Dentures</v>
       </c>
       <c r="C50" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D50" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12433,7 +12433,7 @@
     <row r="51" ht="34" customHeight="1">
       <c r="A51" s="3"/>
       <c r="B51" s="29" t="str">
-        <v>Dentures</v>
+        <v>Hearing aids</v>
       </c>
       <c r="C51" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12446,7 +12446,7 @@
     <row r="52" ht="34" customHeight="1">
       <c r="A52" s="3"/>
       <c r="B52" s="29" t="str">
-        <v>Hearing aids</v>
+        <v>Glasses</v>
       </c>
       <c r="C52" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12459,7 +12459,7 @@
     <row r="53" ht="34" customHeight="1">
       <c r="A53" s="3"/>
       <c r="B53" s="29" t="str">
-        <v>Glasses</v>
+        <v>Oxygen</v>
       </c>
       <c r="C53" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12472,7 +12472,7 @@
     <row r="54" ht="34" customHeight="1">
       <c r="A54" s="3"/>
       <c r="B54" s="29" t="str">
-        <v>Oxygen</v>
+        <v>Hospital bed</v>
       </c>
       <c r="C54" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12485,7 +12485,7 @@
     <row r="55" ht="34" customHeight="1">
       <c r="A55" s="3"/>
       <c r="B55" s="29" t="str">
-        <v>Hospital bed</v>
+        <v>CPAP</v>
       </c>
       <c r="C55" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12498,7 +12498,7 @@
     <row r="56" ht="34" customHeight="1">
       <c r="A56" s="3"/>
       <c r="B56" s="29" t="str">
-        <v>CPAP</v>
+        <v>Catheter care</v>
       </c>
       <c r="C56" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12511,7 +12511,7 @@
     <row r="57" ht="34" customHeight="1">
       <c r="A57" s="3"/>
       <c r="B57" s="29" t="str">
-        <v>Catheter care</v>
+        <v>Colostomy</v>
       </c>
       <c r="C57" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12524,7 +12524,7 @@
     <row r="58" ht="34" customHeight="1">
       <c r="A58" s="3"/>
       <c r="B58" s="29" t="str">
-        <v>Colostomy</v>
+        <v>Ileostomy</v>
       </c>
       <c r="C58" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12537,7 +12537,7 @@
     <row r="59" ht="34" customHeight="1">
       <c r="A59" s="3"/>
       <c r="B59" s="29" t="str">
-        <v>Ileostomy</v>
+        <v>Incontinence issues</v>
       </c>
       <c r="C59" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12547,26 +12547,26 @@
       </c>
       <c r="E59" s="3"/>
     </row>
-    <row r="60" ht="34" customHeight="1">
+    <row r="60" ht="44" customHeight="1">
       <c r="A60" s="3"/>
       <c r="B60" s="29" t="str">
-        <v>Incontinence issues</v>
+        <v>Support</v>
       </c>
       <c r="C60" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Client independently changes briefs; Client needs help changing briefs; Client needs briefs changed</v>
       </c>
       <c r="D60" s="29" t="str">
         <v>04 Health and comfort</v>
       </c>
       <c r="E60" s="3"/>
     </row>
-    <row r="61" ht="44" customHeight="1">
+    <row r="61" ht="34" customHeight="1">
       <c r="A61" s="3"/>
       <c r="B61" s="29" t="str">
-        <v>Support</v>
+        <v>Additional health information</v>
       </c>
       <c r="C61" s="29" t="str">
-        <v>Client independently changes briefs; Client needs help changing briefs; Client needs briefs changed</v>
+        <v>Text or notes</v>
       </c>
       <c r="D61" s="29" t="str">
         <v>04 Health and comfort</v>
@@ -12576,23 +12576,23 @@
     <row r="62" ht="34" customHeight="1">
       <c r="A62" s="3"/>
       <c r="B62" s="29" t="str">
-        <v>Additional health information</v>
+        <v>Medication compliant</v>
       </c>
       <c r="C62" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D62" s="29" t="str">
-        <v>04 Health and comfort</v>
+        <v>05 Medication</v>
       </c>
       <c r="E62" s="3"/>
     </row>
     <row r="63" ht="34" customHeight="1">
       <c r="A63" s="3"/>
       <c r="B63" s="29" t="str">
-        <v>Medication compliant</v>
+        <v>Date of last medication refusal</v>
       </c>
       <c r="C63" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D63" s="29" t="str">
         <v>05 Medication</v>
@@ -12602,10 +12602,10 @@
     <row r="64" ht="34" customHeight="1">
       <c r="A64" s="3"/>
       <c r="B64" s="29" t="str">
-        <v>Date of last medication refusal</v>
+        <v>Medication refused</v>
       </c>
       <c r="C64" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D64" s="29" t="str">
         <v>05 Medication</v>
@@ -12615,10 +12615,10 @@
     <row r="65" ht="34" customHeight="1">
       <c r="A65" s="3"/>
       <c r="B65" s="29" t="str">
-        <v>Medication refused</v>
+        <v>Refusals in the last 30 days</v>
       </c>
       <c r="C65" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D65" s="29" t="str">
         <v>05 Medication</v>
@@ -12628,10 +12628,10 @@
     <row r="66" ht="34" customHeight="1">
       <c r="A66" s="3"/>
       <c r="B66" s="29" t="str">
-        <v>Refusals in the last 30 days</v>
+        <v>Medications at intake</v>
       </c>
       <c r="C66" s="29" t="str">
-        <v>Whole number</v>
+        <v>One item per line</v>
       </c>
       <c r="D66" s="29" t="str">
         <v>05 Medication</v>
@@ -12641,10 +12641,10 @@
     <row r="67" ht="34" customHeight="1">
       <c r="A67" s="3"/>
       <c r="B67" s="29" t="str">
-        <v>Medications at intake</v>
+        <v>PRN patterns</v>
       </c>
       <c r="C67" s="29" t="str">
-        <v>One item per line</v>
+        <v>Text or notes</v>
       </c>
       <c r="D67" s="29" t="str">
         <v>05 Medication</v>
@@ -12654,10 +12654,10 @@
     <row r="68" ht="34" customHeight="1">
       <c r="A68" s="3"/>
       <c r="B68" s="29" t="str">
-        <v>PRN patterns</v>
+        <v>IM injections</v>
       </c>
       <c r="C68" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D68" s="29" t="str">
         <v>05 Medication</v>
@@ -12667,10 +12667,10 @@
     <row r="69" ht="34" customHeight="1">
       <c r="A69" s="3"/>
       <c r="B69" s="29" t="str">
-        <v>IM injections</v>
+        <v>Injection details</v>
       </c>
       <c r="C69" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D69" s="29" t="str">
         <v>05 Medication</v>
@@ -12680,7 +12680,7 @@
     <row r="70" ht="34" customHeight="1">
       <c r="A70" s="3"/>
       <c r="B70" s="29" t="str">
-        <v>Injection details</v>
+        <v>Injection frequency</v>
       </c>
       <c r="C70" s="29" t="str">
         <v>Text or notes</v>
@@ -12693,7 +12693,7 @@
     <row r="71" ht="34" customHeight="1">
       <c r="A71" s="3"/>
       <c r="B71" s="29" t="str">
-        <v>Injection frequency</v>
+        <v>Last injection</v>
       </c>
       <c r="C71" s="29" t="str">
         <v>Text or notes</v>
@@ -12706,7 +12706,7 @@
     <row r="72" ht="34" customHeight="1">
       <c r="A72" s="3"/>
       <c r="B72" s="29" t="str">
-        <v>Last injection</v>
+        <v>Next injection due</v>
       </c>
       <c r="C72" s="29" t="str">
         <v>Text or notes</v>
@@ -12719,7 +12719,7 @@
     <row r="73" ht="34" customHeight="1">
       <c r="A73" s="3"/>
       <c r="B73" s="29" t="str">
-        <v>Next injection due</v>
+        <v>LAI vs oral</v>
       </c>
       <c r="C73" s="29" t="str">
         <v>Text or notes</v>
@@ -12732,36 +12732,36 @@
     <row r="74" ht="34" customHeight="1">
       <c r="A74" s="3"/>
       <c r="B74" s="29" t="str">
-        <v>LAI vs oral</v>
+        <v>County</v>
       </c>
       <c r="C74" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D74" s="29" t="str">
-        <v>05 Medication</v>
+        <v>06 Living situation</v>
       </c>
       <c r="E74" s="3"/>
     </row>
-    <row r="75" ht="34" customHeight="1">
+    <row r="75" ht="76" customHeight="1">
       <c r="A75" s="3"/>
       <c r="B75" s="29" t="str">
-        <v>County</v>
+        <v>Prior setting type</v>
       </c>
       <c r="C75" s="29" t="str">
-        <v>Text or notes</v>
+        <v>State hospital; Acute psychiatric hospital; IMD / MHRC; Skilled nursing facility; Board and care; Residential program; Jail / forensic setting; Independent or family home; Unhoused; Other</v>
       </c>
       <c r="D75" s="29" t="str">
         <v>06 Living situation</v>
       </c>
       <c r="E75" s="3"/>
     </row>
-    <row r="76" ht="76" customHeight="1">
+    <row r="76" ht="34" customHeight="1">
       <c r="A76" s="3"/>
       <c r="B76" s="29" t="str">
-        <v>Prior setting type</v>
+        <v>Prior placement name</v>
       </c>
       <c r="C76" s="29" t="str">
-        <v>State hospital; Acute psychiatric hospital; IMD / MHRC; Skilled nursing facility; Board and care; Residential program; Jail / forensic setting; Independent or family home; Unhoused; Other</v>
+        <v>Text or notes</v>
       </c>
       <c r="D76" s="29" t="str">
         <v>06 Living situation</v>
@@ -12771,10 +12771,10 @@
     <row r="77" ht="34" customHeight="1">
       <c r="A77" s="3"/>
       <c r="B77" s="29" t="str">
-        <v>Prior placement name</v>
+        <v>Admit date</v>
       </c>
       <c r="C77" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D77" s="29" t="str">
         <v>06 Living situation</v>
@@ -12784,20 +12784,20 @@
     <row r="78" ht="34" customHeight="1">
       <c r="A78" s="3"/>
       <c r="B78" s="29" t="str">
-        <v>Admit date</v>
+        <v>Prior placements</v>
       </c>
       <c r="C78" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D78" s="29" t="str">
-        <v>06 Living situation</v>
+        <v>07 Recent care and history</v>
       </c>
       <c r="E78" s="3"/>
     </row>
     <row r="79" ht="34" customHeight="1">
       <c r="A79" s="3"/>
       <c r="B79" s="29" t="str">
-        <v>Prior placements</v>
+        <v>Prior AWOL / failed placements</v>
       </c>
       <c r="C79" s="29" t="str">
         <v>Text or notes</v>
@@ -12810,10 +12810,10 @@
     <row r="80" ht="34" customHeight="1">
       <c r="A80" s="3"/>
       <c r="B80" s="29" t="str">
-        <v>Prior AWOL / failed placements</v>
+        <v>Prior hospitalizations</v>
       </c>
       <c r="C80" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D80" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -12823,10 +12823,10 @@
     <row r="81" ht="34" customHeight="1">
       <c r="A81" s="3"/>
       <c r="B81" s="29" t="str">
-        <v>Prior hospitalizations</v>
+        <v>Most recent hospitalization</v>
       </c>
       <c r="C81" s="29" t="str">
-        <v>Whole number</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D81" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -12836,10 +12836,10 @@
     <row r="82" ht="34" customHeight="1">
       <c r="A82" s="3"/>
       <c r="B82" s="29" t="str">
-        <v>Most recent hospitalization</v>
+        <v>Prior 5150 / 5250 holds</v>
       </c>
       <c r="C82" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D82" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -12849,7 +12849,7 @@
     <row r="83" ht="34" customHeight="1">
       <c r="A83" s="3"/>
       <c r="B83" s="29" t="str">
-        <v>Prior 5150 / 5250 holds</v>
+        <v>Crisis / ER utilization</v>
       </c>
       <c r="C83" s="29" t="str">
         <v>Text or notes</v>
@@ -12862,20 +12862,20 @@
     <row r="84" ht="34" customHeight="1">
       <c r="A84" s="3"/>
       <c r="B84" s="29" t="str">
-        <v>Crisis / ER utilization</v>
+        <v>History of substance abuse</v>
       </c>
       <c r="C84" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D84" s="29" t="str">
-        <v>07 Recent care and history</v>
+        <v>08 Substance use and recovery</v>
       </c>
       <c r="E84" s="3"/>
     </row>
     <row r="85" ht="34" customHeight="1">
       <c r="A85" s="3"/>
       <c r="B85" s="29" t="str">
-        <v>History of substance abuse</v>
+        <v>Active substance use</v>
       </c>
       <c r="C85" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -12888,10 +12888,10 @@
     <row r="86" ht="34" customHeight="1">
       <c r="A86" s="3"/>
       <c r="B86" s="29" t="str">
-        <v>Active substance use</v>
+        <v>Substances</v>
       </c>
       <c r="C86" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Opioids; Amphetamines; Marijuana; Alcohol; Other</v>
       </c>
       <c r="D86" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12901,10 +12901,10 @@
     <row r="87" ht="34" customHeight="1">
       <c r="A87" s="3"/>
       <c r="B87" s="29" t="str">
-        <v>Substances</v>
+        <v>Last substance use</v>
       </c>
       <c r="C87" s="29" t="str">
-        <v>Opioids; Amphetamines; Marijuana; Alcohol; Other</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D87" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12914,10 +12914,10 @@
     <row r="88" ht="34" customHeight="1">
       <c r="A88" s="3"/>
       <c r="B88" s="29" t="str">
-        <v>Last substance use</v>
+        <v>Use pattern</v>
       </c>
       <c r="C88" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Daily; Weekly; Sporadic; Rarely</v>
       </c>
       <c r="D88" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12927,49 +12927,49 @@
     <row r="89" ht="34" customHeight="1">
       <c r="A89" s="3"/>
       <c r="B89" s="29" t="str">
-        <v>Use pattern</v>
+        <v>Effect on baseline behavior</v>
       </c>
       <c r="C89" s="29" t="str">
-        <v>Daily; Weekly; Sporadic; Rarely</v>
+        <v>Text or notes</v>
       </c>
       <c r="D89" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" ht="34" customHeight="1">
+    <row r="90" ht="60" customHeight="1">
       <c r="A90" s="3"/>
       <c r="B90" s="29" t="str">
-        <v>Effect on baseline behavior</v>
+        <v>Longest sobriety in the last five years</v>
       </c>
       <c r="C90" s="29" t="str">
-        <v>Text or notes</v>
+        <v>1 month; 2 months; 3 months; 4 months; 5 months; 6 months; 7 months; 8 months; 9 months; 10 months; 11 months; 1 year; 18 months; 2 years; More than 2 years</v>
       </c>
       <c r="D90" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" ht="60" customHeight="1">
+    <row r="91" ht="44" customHeight="1">
       <c r="A91" s="3"/>
       <c r="B91" s="29" t="str">
-        <v>Longest sobriety in the last five years</v>
+        <v>Acknowledgment of substance-use impact</v>
       </c>
       <c r="C91" s="29" t="str">
-        <v>1 month; 2 months; 3 months; 4 months; 5 months; 6 months; 7 months; 8 months; 9 months; 10 months; 11 months; 1 year; 18 months; 2 years; More than 2 years</v>
+        <v>Acknowledges impact; Partially acknowledges impact; Does not acknowledge impact; Not discussed</v>
       </c>
       <c r="D91" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" ht="44" customHeight="1">
+    <row r="92" ht="34" customHeight="1">
       <c r="A92" s="3"/>
       <c r="B92" s="29" t="str">
-        <v>Acknowledgment of substance-use impact</v>
+        <v>Substance-use impact notes</v>
       </c>
       <c r="C92" s="29" t="str">
-        <v>Acknowledges impact; Partially acknowledges impact; Does not acknowledge impact; Not discussed</v>
+        <v>Text or notes</v>
       </c>
       <c r="D92" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12979,7 +12979,7 @@
     <row r="93" ht="34" customHeight="1">
       <c r="A93" s="3"/>
       <c r="B93" s="29" t="str">
-        <v>Substance-use impact notes</v>
+        <v>Treatment history</v>
       </c>
       <c r="C93" s="29" t="str">
         <v>Text or notes</v>
@@ -12992,10 +12992,10 @@
     <row r="94" ht="34" customHeight="1">
       <c r="A94" s="3"/>
       <c r="B94" s="29" t="str">
-        <v>Treatment history</v>
+        <v>Longest sobriety in the last five years</v>
       </c>
       <c r="C94" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D94" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13005,23 +13005,23 @@
     <row r="95" ht="34" customHeight="1">
       <c r="A95" s="3"/>
       <c r="B95" s="29" t="str">
-        <v>Longest sobriety in the last five years</v>
+        <v>Behavioral history</v>
       </c>
       <c r="C95" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D95" s="29" t="str">
-        <v>08 Substance use and recovery</v>
+        <v>09 Safety and support</v>
       </c>
       <c r="E95" s="3"/>
     </row>
     <row r="96" ht="34" customHeight="1">
       <c r="A96" s="3"/>
       <c r="B96" s="29" t="str">
-        <v>Behavioral history</v>
+        <v>Physical altercations</v>
       </c>
       <c r="C96" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D96" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13031,10 +13031,10 @@
     <row r="97" ht="34" customHeight="1">
       <c r="A97" s="3"/>
       <c r="B97" s="29" t="str">
-        <v>Physical altercations</v>
+        <v>Physical altercation details</v>
       </c>
       <c r="C97" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D97" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13044,10 +13044,10 @@
     <row r="98" ht="34" customHeight="1">
       <c r="A98" s="3"/>
       <c r="B98" s="29" t="str">
-        <v>Physical altercation details</v>
+        <v>History of self-harm</v>
       </c>
       <c r="C98" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D98" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13057,10 +13057,10 @@
     <row r="99" ht="34" customHeight="1">
       <c r="A99" s="3"/>
       <c r="B99" s="29" t="str">
-        <v>History of self-harm</v>
+        <v>Last documented self-harm incident</v>
       </c>
       <c r="C99" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D99" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13070,10 +13070,10 @@
     <row r="100" ht="34" customHeight="1">
       <c r="A100" s="3"/>
       <c r="B100" s="29" t="str">
-        <v>Last documented self-harm incident</v>
+        <v>Current self-harm ideation</v>
       </c>
       <c r="C100" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D100" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13083,10 +13083,10 @@
     <row r="101" ht="34" customHeight="1">
       <c r="A101" s="3"/>
       <c r="B101" s="29" t="str">
-        <v>Current self-harm ideation</v>
+        <v>Current self-harm ideation details</v>
       </c>
       <c r="C101" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D101" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13096,7 +13096,7 @@
     <row r="102" ht="34" customHeight="1">
       <c r="A102" s="3"/>
       <c r="B102" s="29" t="str">
-        <v>Current self-harm ideation details</v>
+        <v>Current safety measures</v>
       </c>
       <c r="C102" s="29" t="str">
         <v>Text or notes</v>
@@ -13109,10 +13109,10 @@
     <row r="103" ht="34" customHeight="1">
       <c r="A103" s="3"/>
       <c r="B103" s="29" t="str">
-        <v>Current safety measures</v>
+        <v>History of assaults</v>
       </c>
       <c r="C103" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D103" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13122,10 +13122,10 @@
     <row r="104" ht="34" customHeight="1">
       <c r="A104" s="3"/>
       <c r="B104" s="29" t="str">
-        <v>History of assaults</v>
+        <v>Most recent assault</v>
       </c>
       <c r="C104" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D104" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13135,10 +13135,10 @@
     <row r="105" ht="34" customHeight="1">
       <c r="A105" s="3"/>
       <c r="B105" s="29" t="str">
-        <v>Most recent assault</v>
+        <v>Assaults in the last two years</v>
       </c>
       <c r="C105" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D105" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13148,10 +13148,10 @@
     <row r="106" ht="34" customHeight="1">
       <c r="A106" s="3"/>
       <c r="B106" s="29" t="str">
-        <v>Assaults in the last two years</v>
+        <v>History of elopement</v>
       </c>
       <c r="C106" s="29" t="str">
-        <v>Whole number</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D106" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13161,10 +13161,10 @@
     <row r="107" ht="34" customHeight="1">
       <c r="A107" s="3"/>
       <c r="B107" s="29" t="str">
-        <v>History of elopement</v>
+        <v>Elopement risk</v>
       </c>
       <c r="C107" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D107" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13174,7 +13174,7 @@
     <row r="108" ht="34" customHeight="1">
       <c r="A108" s="3"/>
       <c r="B108" s="29" t="str">
-        <v>Elopement risk</v>
+        <v>SI / HI history</v>
       </c>
       <c r="C108" s="29" t="str">
         <v>Text or notes</v>
@@ -13187,7 +13187,7 @@
     <row r="109" ht="34" customHeight="1">
       <c r="A109" s="3"/>
       <c r="B109" s="29" t="str">
-        <v>SI / HI history</v>
+        <v>Triggers and what helps</v>
       </c>
       <c r="C109" s="29" t="str">
         <v>Text or notes</v>
@@ -13200,7 +13200,7 @@
     <row r="110" ht="34" customHeight="1">
       <c r="A110" s="3"/>
       <c r="B110" s="29" t="str">
-        <v>Triggers and what helps</v>
+        <v>Aggression risk</v>
       </c>
       <c r="C110" s="29" t="str">
         <v>Text or notes</v>
@@ -13213,7 +13213,7 @@
     <row r="111" ht="34" customHeight="1">
       <c r="A111" s="3"/>
       <c r="B111" s="29" t="str">
-        <v>Aggression risk</v>
+        <v>Responds to internal stimuli</v>
       </c>
       <c r="C111" s="29" t="str">
         <v>Text or notes</v>
@@ -13226,7 +13226,7 @@
     <row r="112" ht="34" customHeight="1">
       <c r="A112" s="3"/>
       <c r="B112" s="29" t="str">
-        <v>Responds to internal stimuli</v>
+        <v>Auditory hallucinations</v>
       </c>
       <c r="C112" s="29" t="str">
         <v>Text or notes</v>
@@ -13239,7 +13239,7 @@
     <row r="113" ht="34" customHeight="1">
       <c r="A113" s="3"/>
       <c r="B113" s="29" t="str">
-        <v>Auditory hallucinations</v>
+        <v>Nature of auditory hallucinations</v>
       </c>
       <c r="C113" s="29" t="str">
         <v>Text or notes</v>
@@ -13252,7 +13252,7 @@
     <row r="114" ht="34" customHeight="1">
       <c r="A114" s="3"/>
       <c r="B114" s="29" t="str">
-        <v>Nature of auditory hallucinations</v>
+        <v>Current auditory frequency</v>
       </c>
       <c r="C114" s="29" t="str">
         <v>Text or notes</v>
@@ -13265,7 +13265,7 @@
     <row r="115" ht="34" customHeight="1">
       <c r="A115" s="3"/>
       <c r="B115" s="29" t="str">
-        <v>Current auditory frequency</v>
+        <v>Auditory triggers</v>
       </c>
       <c r="C115" s="29" t="str">
         <v>Text or notes</v>
@@ -13278,7 +13278,7 @@
     <row r="116" ht="34" customHeight="1">
       <c r="A116" s="3"/>
       <c r="B116" s="29" t="str">
-        <v>Auditory triggers</v>
+        <v>Visual hallucinations</v>
       </c>
       <c r="C116" s="29" t="str">
         <v>Text or notes</v>
@@ -13291,7 +13291,7 @@
     <row r="117" ht="34" customHeight="1">
       <c r="A117" s="3"/>
       <c r="B117" s="29" t="str">
-        <v>Visual hallucinations</v>
+        <v>Nature and frequency of visual hallucinations</v>
       </c>
       <c r="C117" s="29" t="str">
         <v>Text or notes</v>
@@ -13304,7 +13304,7 @@
     <row r="118" ht="34" customHeight="1">
       <c r="A118" s="3"/>
       <c r="B118" s="29" t="str">
-        <v>Nature and frequency of visual hallucinations</v>
+        <v>Recent visual hallucinations</v>
       </c>
       <c r="C118" s="29" t="str">
         <v>Text or notes</v>
@@ -13317,7 +13317,7 @@
     <row r="119" ht="34" customHeight="1">
       <c r="A119" s="3"/>
       <c r="B119" s="29" t="str">
-        <v>Recent visual hallucinations</v>
+        <v>Olfactory hallucinations</v>
       </c>
       <c r="C119" s="29" t="str">
         <v>Text or notes</v>
@@ -13330,7 +13330,7 @@
     <row r="120" ht="34" customHeight="1">
       <c r="A120" s="3"/>
       <c r="B120" s="29" t="str">
-        <v>Olfactory hallucinations</v>
+        <v>Olfactory hallucination details</v>
       </c>
       <c r="C120" s="29" t="str">
         <v>Text or notes</v>
@@ -13343,7 +13343,7 @@
     <row r="121" ht="34" customHeight="1">
       <c r="A121" s="3"/>
       <c r="B121" s="29" t="str">
-        <v>Olfactory hallucination details</v>
+        <v>Impact of olfactory hallucinations</v>
       </c>
       <c r="C121" s="29" t="str">
         <v>Text or notes</v>
@@ -13356,7 +13356,7 @@
     <row r="122" ht="34" customHeight="1">
       <c r="A122" s="3"/>
       <c r="B122" s="29" t="str">
-        <v>Impact of olfactory hallucinations</v>
+        <v>Tactile hallucinations</v>
       </c>
       <c r="C122" s="29" t="str">
         <v>Text or notes</v>
@@ -13369,7 +13369,7 @@
     <row r="123" ht="34" customHeight="1">
       <c r="A123" s="3"/>
       <c r="B123" s="29" t="str">
-        <v>Tactile hallucinations</v>
+        <v>Tactile hallucination details</v>
       </c>
       <c r="C123" s="29" t="str">
         <v>Text or notes</v>
@@ -13382,7 +13382,7 @@
     <row r="124" ht="34" customHeight="1">
       <c r="A124" s="3"/>
       <c r="B124" s="29" t="str">
-        <v>Tactile hallucination details</v>
+        <v>Tactile hallucination frequency</v>
       </c>
       <c r="C124" s="29" t="str">
         <v>Text or notes</v>
@@ -13395,7 +13395,7 @@
     <row r="125" ht="34" customHeight="1">
       <c r="A125" s="3"/>
       <c r="B125" s="29" t="str">
-        <v>Tactile hallucination frequency</v>
+        <v>Gustatory hallucinations</v>
       </c>
       <c r="C125" s="29" t="str">
         <v>Text or notes</v>
@@ -13408,7 +13408,7 @@
     <row r="126" ht="34" customHeight="1">
       <c r="A126" s="3"/>
       <c r="B126" s="29" t="str">
-        <v>Gustatory hallucinations</v>
+        <v>Gustatory hallucination details</v>
       </c>
       <c r="C126" s="29" t="str">
         <v>Text or notes</v>
@@ -13421,7 +13421,7 @@
     <row r="127" ht="34" customHeight="1">
       <c r="A127" s="3"/>
       <c r="B127" s="29" t="str">
-        <v>Gustatory hallucination details</v>
+        <v>Hallucination coping strategies</v>
       </c>
       <c r="C127" s="29" t="str">
         <v>Text or notes</v>
@@ -13434,7 +13434,7 @@
     <row r="128" ht="34" customHeight="1">
       <c r="A128" s="3"/>
       <c r="B128" s="29" t="str">
-        <v>Hallucination coping strategies</v>
+        <v>Hallucination distress or impairment</v>
       </c>
       <c r="C128" s="29" t="str">
         <v>Text or notes</v>
@@ -13447,7 +13447,7 @@
     <row r="129" ht="34" customHeight="1">
       <c r="A129" s="3"/>
       <c r="B129" s="29" t="str">
-        <v>Hallucination distress or impairment</v>
+        <v>Impact on daily functioning</v>
       </c>
       <c r="C129" s="29" t="str">
         <v>Text or notes</v>
@@ -13460,7 +13460,7 @@
     <row r="130" ht="34" customHeight="1">
       <c r="A130" s="3"/>
       <c r="B130" s="29" t="str">
-        <v>Impact on daily functioning</v>
+        <v>Professional discussion and treatment</v>
       </c>
       <c r="C130" s="29" t="str">
         <v>Text or notes</v>
@@ -13473,23 +13473,23 @@
     <row r="131" ht="34" customHeight="1">
       <c r="A131" s="3"/>
       <c r="B131" s="29" t="str">
-        <v>Professional discussion and treatment</v>
+        <v>Conserved status</v>
       </c>
       <c r="C131" s="29" t="str">
-        <v>Text or notes</v>
+        <v>LPS; TCon; Murphy's; Non-Conserved</v>
       </c>
       <c r="D131" s="29" t="str">
-        <v>09 Safety and support</v>
+        <v>10 Decisions and legal support</v>
       </c>
       <c r="E131" s="3"/>
     </row>
     <row r="132" ht="34" customHeight="1">
       <c r="A132" s="3"/>
       <c r="B132" s="29" t="str">
-        <v>Conserved status</v>
+        <v>Conservator name</v>
       </c>
       <c r="C132" s="29" t="str">
-        <v>LPS; TCon; Murphy's; Non-Conserved</v>
+        <v>Text or notes</v>
       </c>
       <c r="D132" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13499,7 +13499,7 @@
     <row r="133" ht="34" customHeight="1">
       <c r="A133" s="3"/>
       <c r="B133" s="29" t="str">
-        <v>Conservator name</v>
+        <v>Conservatorship details</v>
       </c>
       <c r="C133" s="29" t="str">
         <v>Text or notes</v>
@@ -13512,7 +13512,7 @@
     <row r="134" ht="34" customHeight="1">
       <c r="A134" s="3"/>
       <c r="B134" s="29" t="str">
-        <v>Conservatorship details</v>
+        <v>Hold type</v>
       </c>
       <c r="C134" s="29" t="str">
         <v>Text or notes</v>
@@ -13525,10 +13525,10 @@
     <row r="135" ht="34" customHeight="1">
       <c r="A135" s="3"/>
       <c r="B135" s="29" t="str">
-        <v>Hold type</v>
+        <v>Forensic involvement</v>
       </c>
       <c r="C135" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D135" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13538,10 +13538,10 @@
     <row r="136" ht="34" customHeight="1">
       <c r="A136" s="3"/>
       <c r="B136" s="29" t="str">
-        <v>Forensic involvement</v>
+        <v>Forensic involvement details</v>
       </c>
       <c r="C136" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D136" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13551,10 +13551,10 @@
     <row r="137" ht="34" customHeight="1">
       <c r="A137" s="3"/>
       <c r="B137" s="29" t="str">
-        <v>Forensic involvement details</v>
+        <v>History of arrest</v>
       </c>
       <c r="C137" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D137" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13564,10 +13564,10 @@
     <row r="138" ht="34" customHeight="1">
       <c r="A138" s="3"/>
       <c r="B138" s="29" t="str">
-        <v>History of arrest</v>
+        <v>Most recent arrest date</v>
       </c>
       <c r="C138" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D138" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13577,10 +13577,10 @@
     <row r="139" ht="34" customHeight="1">
       <c r="A139" s="3"/>
       <c r="B139" s="29" t="str">
-        <v>Most recent arrest date</v>
+        <v>Most recent arrest charge</v>
       </c>
       <c r="C139" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D139" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13590,7 +13590,7 @@
     <row r="140" ht="34" customHeight="1">
       <c r="A140" s="3"/>
       <c r="B140" s="29" t="str">
-        <v>Most recent arrest charge</v>
+        <v>Time in jail</v>
       </c>
       <c r="C140" s="29" t="str">
         <v>Text or notes</v>
@@ -13603,10 +13603,10 @@
     <row r="141" ht="34" customHeight="1">
       <c r="A141" s="3"/>
       <c r="B141" s="29" t="str">
-        <v>Time in jail</v>
+        <v>Arrest in the last two years</v>
       </c>
       <c r="C141" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D141" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13616,10 +13616,10 @@
     <row r="142" ht="34" customHeight="1">
       <c r="A142" s="3"/>
       <c r="B142" s="29" t="str">
-        <v>Arrest in the last two years</v>
+        <v>Recent arrest details</v>
       </c>
       <c r="C142" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D142" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13629,10 +13629,10 @@
     <row r="143" ht="34" customHeight="1">
       <c r="A143" s="3"/>
       <c r="B143" s="29" t="str">
-        <v>Recent arrest details</v>
+        <v>Total recorded arrests</v>
       </c>
       <c r="C143" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D143" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13642,10 +13642,10 @@
     <row r="144" ht="34" customHeight="1">
       <c r="A144" s="3"/>
       <c r="B144" s="29" t="str">
-        <v>Total recorded arrests</v>
+        <v>PC 290 registration</v>
       </c>
       <c r="C144" s="29" t="str">
-        <v>Whole number</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D144" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13655,7 +13655,7 @@
     <row r="145" ht="34" customHeight="1">
       <c r="A145" s="3"/>
       <c r="B145" s="29" t="str">
-        <v>PC 290 registration</v>
+        <v>Arson history</v>
       </c>
       <c r="C145" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13668,7 +13668,7 @@
     <row r="146" ht="34" customHeight="1">
       <c r="A146" s="3"/>
       <c r="B146" s="29" t="str">
-        <v>Arson history</v>
+        <v>Diversion client</v>
       </c>
       <c r="C146" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13681,10 +13681,10 @@
     <row r="147" ht="34" customHeight="1">
       <c r="A147" s="3"/>
       <c r="B147" s="29" t="str">
-        <v>Diversion client</v>
+        <v>Court requirements</v>
       </c>
       <c r="C147" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D147" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13694,7 +13694,7 @@
     <row r="148" ht="34" customHeight="1">
       <c r="A148" s="3"/>
       <c r="B148" s="29" t="str">
-        <v>Court requirements</v>
+        <v>Court dates</v>
       </c>
       <c r="C148" s="29" t="str">
         <v>Text or notes</v>
@@ -13707,7 +13707,7 @@
     <row r="149" ht="34" customHeight="1">
       <c r="A149" s="3"/>
       <c r="B149" s="29" t="str">
-        <v>Court dates</v>
+        <v>Probation / parole / justice</v>
       </c>
       <c r="C149" s="29" t="str">
         <v>Text or notes</v>
@@ -13720,20 +13720,20 @@
     <row r="150" ht="34" customHeight="1">
       <c r="A150" s="3"/>
       <c r="B150" s="29" t="str">
-        <v>Probation / parole / justice</v>
+        <v>Family involvement</v>
       </c>
       <c r="C150" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D150" s="29" t="str">
-        <v>10 Decisions and legal support</v>
+        <v>11 What matters next</v>
       </c>
       <c r="E150" s="3"/>
     </row>
     <row r="151" ht="34" customHeight="1">
       <c r="A151" s="3"/>
       <c r="B151" s="29" t="str">
-        <v>Family involvement</v>
+        <v>Friendships and social connections</v>
       </c>
       <c r="C151" s="29" t="str">
         <v>Text or notes</v>
@@ -13746,7 +13746,7 @@
     <row r="152" ht="34" customHeight="1">
       <c r="A152" s="3"/>
       <c r="B152" s="29" t="str">
-        <v>Friendships and social connections</v>
+        <v>Prior living situation</v>
       </c>
       <c r="C152" s="29" t="str">
         <v>Text or notes</v>
@@ -13759,7 +13759,7 @@
     <row r="153" ht="34" customHeight="1">
       <c r="A153" s="3"/>
       <c r="B153" s="29" t="str">
-        <v>Prior living situation</v>
+        <v>Housing history</v>
       </c>
       <c r="C153" s="29" t="str">
         <v>Text or notes</v>
@@ -13772,7 +13772,7 @@
     <row r="154" ht="34" customHeight="1">
       <c r="A154" s="3"/>
       <c r="B154" s="29" t="str">
-        <v>Housing history</v>
+        <v>Benefits / income status</v>
       </c>
       <c r="C154" s="29" t="str">
         <v>Text or notes</v>
@@ -13785,7 +13785,7 @@
     <row r="155" ht="34" customHeight="1">
       <c r="A155" s="3"/>
       <c r="B155" s="29" t="str">
-        <v>Benefits / income status</v>
+        <v>Preferred facility characteristics</v>
       </c>
       <c r="C155" s="29" t="str">
         <v>Text or notes</v>
@@ -13798,7 +13798,7 @@
     <row r="156" ht="34" customHeight="1">
       <c r="A156" s="3"/>
       <c r="B156" s="29" t="str">
-        <v>Preferred facility characteristics</v>
+        <v>Discharge planning goals</v>
       </c>
       <c r="C156" s="29" t="str">
         <v>Text or notes</v>
@@ -13811,7 +13811,7 @@
     <row r="157" ht="34" customHeight="1">
       <c r="A157" s="3"/>
       <c r="B157" s="29" t="str">
-        <v>Discharge planning goals</v>
+        <v>Placement preferences and concerns</v>
       </c>
       <c r="C157" s="29" t="str">
         <v>Text or notes</v>
@@ -13824,20 +13824,20 @@
     <row r="158" ht="34" customHeight="1">
       <c r="A158" s="3"/>
       <c r="B158" s="29" t="str">
-        <v>Placement preferences and concerns</v>
+        <v>Additional information</v>
       </c>
       <c r="C158" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D158" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>12 Anything else</v>
       </c>
       <c r="E158" s="3"/>
     </row>
     <row r="159" ht="34" customHeight="1">
       <c r="A159" s="3"/>
       <c r="B159" s="29" t="str">
-        <v>Additional information</v>
+        <v>Placement questions or concerns</v>
       </c>
       <c r="C159" s="29" t="str">
         <v>Text or notes</v>
@@ -13850,7 +13850,7 @@
     <row r="160" ht="34" customHeight="1">
       <c r="A160" s="3"/>
       <c r="B160" s="29" t="str">
-        <v>Placement questions or concerns</v>
+        <v>Assessment notes</v>
       </c>
       <c r="C160" s="29" t="str">
         <v>Text or notes</v>
@@ -13860,17 +13860,11 @@
       </c>
       <c r="E160" s="3"/>
     </row>
-    <row r="161" ht="34" customHeight="1">
+    <row r="161">
       <c r="A161" s="3"/>
-      <c r="B161" s="29" t="str">
-        <v>Assessment notes</v>
-      </c>
-      <c r="C161" s="29" t="str">
-        <v>Text or notes</v>
-      </c>
-      <c r="D161" s="29" t="str">
-        <v>12 Anything else</v>
-      </c>
+      <c r="B161" s="3"/>
+      <c r="C161" s="3"/>
+      <c r="D161" s="3"/>
       <c r="E161" s="3"/>
     </row>
     <row r="162">
@@ -14114,18 +14108,36 @@
         <v>Optional</v>
       </c>
     </row>
-    <row r="15" ht="34" customHeight="1">
+    <row r="15" ht="39" customHeight="1" hidden="1">
       <c r="A15" s="3" t="str">
         <v>resident_number</v>
       </c>
-      <c r="B15" s="13" t="str">
-        <v>Resident number</v>
-      </c>
-      <c r="C15" t="str" s="50"/>
-      <c r="D15" t="str" s="48"/>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="12"/>
+              <color rgb="FF233B32"/>
+            </rPr>
+            <t>Resident number</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="0"/>
+              <sz val="10"/>
+              <color rgb="FF59675F"/>
+            </rPr>
+            <t xml:space="preserve">
+Reference only.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C15" s="23" t="str"/>
+      <c r="D15" s="15" t="str"/>
       <c r="E15" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C15))&gt;0,LEN(TRIM(D15))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D15))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D15))&gt;0)),"Explain why",IF(LEN(TRIM(C15))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
+        <f>"Reference only"</f>
+        <v>Reference only</v>
       </c>
     </row>
     <row r="16" ht="39" customHeight="1">

</xml_diff>

<commit_message>
Condense hospitalization and forensic histories into structured overviews
</commit_message>
<xml_diff>
--- a/public/templates/pipeline-assessment-workbook.xlsx
+++ b/public/templates/pipeline-assessment-workbook.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Raba6eabfa2c0467e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="R6d3c53b35ab2451e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R19ade892a9e9487f"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="R8b151a64b22b4af9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Rbf3a71609d6743d6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="Rfd66ce774fc94e99"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="R387c3a8951cc4843"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="Rf20811a60f024902"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Red12527f76d5406e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R7fbf3f91f3294651"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="R647a55aefa954e92"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="Rc2f47f3707024ecf"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="R78cf9d19b64649d0"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="R5721e6970feb49ce" state="veryHidden"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="Rfcdada3041aa4328"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R2fcb16bfacf74ef7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="R83dcd224a24a4f05"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="Rebc4e9e1c4c54ca0"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="Ra8a42a95b98748cd"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="R5f9921955eb745ef"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="Rf794a62138a74c0c"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="Rf8b55cac3b314109"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="Re7780c6dd2cd4f43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="R386f0510ac0a426b"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R282480e6d0094a89"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="R6983b7cb1a294d1c"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R25c59fc2162549b0"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="R919b6692dd9440fa"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="R7b1b5c4c758446cf" state="veryHidden"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="R666bd830afe64dc1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Confirm the basics'!$B$1:$E$16</definedName>
@@ -31,13 +31,13 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'05 Medication'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'06 Living situation'!$B$1:$E$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'06 Living situation'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="7">'07 Recent care and history'!$B$1:$E$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">'07 Recent care and history'!$B$1:$E$26</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'07 Recent care and history'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'08 Substance use and recovery'!$B$1:$E$29</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'08 Substance use and recovery'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'09 Safety and support'!$B$1:$E$41</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'09 Safety and support'!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="10">'10 Decisions and legal support'!$B$1:$E$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="10">'10 Decisions and legal support'!$B$1:$E$39</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'10 Decisions and legal support'!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="11">'11 What matters next'!$B$1:$E$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="11">'11 What matters next'!$1:$5</definedName>
@@ -395,7 +395,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
-  <dxfs count="381">
+  <dxfs count="386">
     <dxf>
       <font>
         <color rgb="FF68756F"/>
@@ -2320,6 +2320,48 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF68756F"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF1F3F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF70511D"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF0CA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF68756F"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF1F3F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF70511D"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF0CA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF233B32"/>
       </font>
       <fill>
@@ -3461,6 +3503,48 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF68756F"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF1F3F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF70511D"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF0CA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF68756F"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF1F3F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF70511D"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF0CA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF233B32"/>
       </font>
       <fill>
@@ -3492,6 +3576,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF233B32"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF6DF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF68756F"/>
       </font>
       <fill>
@@ -3607,16 +3701,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF233B32"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF6DF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF68756F"/>
       </font>
       <fill>
@@ -3680,16 +3764,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF233B32"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF6DF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF68756F"/>
       </font>
       <fill>
@@ -3711,16 +3785,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF233B32"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF6DF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF68756F"/>
       </font>
       <fill>
@@ -3737,16 +3801,6 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFF0CA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF233B32"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF6DF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4828,11 +4882,11 @@
         <v>7. Recent care and history</v>
       </c>
       <c r="C22" s="31" t="n">
-        <f>COUNTIF('07 Recent care and history'!E6:E11,"Needs answer")+COUNTIF('07 Recent care and history'!E6:E11,"Explain why")</f>
-        <v>1</v>
+        <f>COUNTIF('07 Recent care and history'!E6:E26,"Needs answer")+COUNTIF('07 Recent care and history'!E6:E26,"Explain why")</f>
+        <v>0</v>
       </c>
       <c r="D22" s="31" t="n">
-        <f>COUNTIF('07 Recent care and history'!E6:E11,"Review previous answer")+COUNTIF('07 Recent care and history'!E6:E11,"Review previous reason")</f>
+        <f>COUNTIF('07 Recent care and history'!E6:E26,"Review previous answer")+COUNTIF('07 Recent care and history'!E6:E26,"Review previous reason")</f>
         <v>0</v>
       </c>
       <c r="E22" s="30"/>
@@ -4873,11 +4927,11 @@
         <v>10. Decisions and legal support</v>
       </c>
       <c r="C25" s="31" t="n">
-        <f>COUNTIF('10 Decisions and legal support'!E6:E24,"Needs answer")+COUNTIF('10 Decisions and legal support'!E6:E24,"Explain why")</f>
-        <v>6</v>
+        <f>COUNTIF('10 Decisions and legal support'!E6:E39,"Needs answer")+COUNTIF('10 Decisions and legal support'!E6:E39,"Explain why")</f>
+        <v>4</v>
       </c>
       <c r="D25" s="31" t="n">
-        <f>COUNTIF('10 Decisions and legal support'!E6:E24,"Review previous answer")+COUNTIF('10 Decisions and legal support'!E6:E24,"Review previous reason")</f>
+        <f>COUNTIF('10 Decisions and legal support'!E6:E39,"Review previous answer")+COUNTIF('10 Decisions and legal support'!E6:E39,"Review previous reason")</f>
         <v>0</v>
       </c>
       <c r="E25" s="30"/>
@@ -4939,62 +4993,62 @@
     <mergeCell ref="D27:E27"/>
   </mergeCells>
   <conditionalFormatting sqref="C16:D16">
-    <cfRule type="cellIs" dxfId="357" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="362" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C17:D17">
-    <cfRule type="cellIs" dxfId="358" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="363" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18:D18">
-    <cfRule type="cellIs" dxfId="359" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="364" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19:D19">
-    <cfRule type="cellIs" dxfId="360" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="365" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C20:D20">
-    <cfRule type="cellIs" dxfId="361" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="366" priority="5" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C21:D21">
-    <cfRule type="cellIs" dxfId="362" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="367" priority="6" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C22:D22">
-    <cfRule type="cellIs" dxfId="363" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="368" priority="7" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C23:D23">
-    <cfRule type="cellIs" dxfId="364" priority="8" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="369" priority="8" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C24:D24">
-    <cfRule type="cellIs" dxfId="365" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="370" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C25:D25">
-    <cfRule type="cellIs" dxfId="366" priority="10" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="371" priority="10" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C26:D26">
-    <cfRule type="cellIs" dxfId="367" priority="11" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="372" priority="11" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C27:D27">
-    <cfRule type="cellIs" dxfId="368" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="373" priority="12" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5724,387 +5778,387 @@
     <mergeCell ref="B3:E3"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:E6">
-    <cfRule type="expression" dxfId="206" priority="1">
+    <cfRule type="expression" dxfId="210" priority="1">
       <formula>$E6="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6:E6">
-    <cfRule type="expression" dxfId="207" priority="2">
+    <cfRule type="expression" dxfId="211" priority="2">
       <formula>OR($E6="Needs answer",$E6="Explain why",LEFT($E6,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:E7">
-    <cfRule type="expression" dxfId="208" priority="3">
+    <cfRule type="expression" dxfId="212" priority="3">
       <formula>$E7="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7:E7">
-    <cfRule type="expression" dxfId="209" priority="4">
+    <cfRule type="expression" dxfId="213" priority="4">
       <formula>OR($E7="Needs answer",$E7="Explain why",LEFT($E7,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:D7">
-    <cfRule type="expression" dxfId="210" priority="5">
+    <cfRule type="expression" dxfId="214" priority="5">
       <formula>OR($C7="Unable to assess",$C7="unable_to_assess")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:E8">
-    <cfRule type="expression" dxfId="211" priority="6">
+    <cfRule type="expression" dxfId="215" priority="6">
       <formula>$E8="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8:E8">
-    <cfRule type="expression" dxfId="212" priority="7">
+    <cfRule type="expression" dxfId="216" priority="7">
       <formula>OR($E8="Needs answer",$E8="Explain why",LEFT($E8,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:E9">
-    <cfRule type="expression" dxfId="213" priority="8">
+    <cfRule type="expression" dxfId="217" priority="8">
       <formula>$E9="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9:E9">
-    <cfRule type="expression" dxfId="214" priority="9">
+    <cfRule type="expression" dxfId="218" priority="9">
       <formula>OR($E9="Needs answer",$E9="Explain why",LEFT($E9,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9:D9">
-    <cfRule type="expression" dxfId="215" priority="10">
+    <cfRule type="expression" dxfId="219" priority="10">
       <formula>OR($C9="Unable to assess",$C9="unable_to_assess")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:E10">
-    <cfRule type="expression" dxfId="216" priority="11">
+    <cfRule type="expression" dxfId="220" priority="11">
       <formula>$E10="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10:E10">
-    <cfRule type="expression" dxfId="217" priority="12">
+    <cfRule type="expression" dxfId="221" priority="12">
       <formula>OR($E10="Needs answer",$E10="Explain why",LEFT($E10,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:E11">
-    <cfRule type="expression" dxfId="218" priority="13">
+    <cfRule type="expression" dxfId="222" priority="13">
       <formula>$E11="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11:E11">
-    <cfRule type="expression" dxfId="219" priority="14">
+    <cfRule type="expression" dxfId="223" priority="14">
       <formula>OR($E11="Needs answer",$E11="Explain why",LEFT($E11,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11:D11">
-    <cfRule type="expression" dxfId="220" priority="15">
+    <cfRule type="expression" dxfId="224" priority="15">
       <formula>OR($C11="Unable to assess",$C11="unable_to_assess")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:E12">
-    <cfRule type="expression" dxfId="221" priority="16">
+    <cfRule type="expression" dxfId="225" priority="16">
       <formula>$E12="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E12:E12">
-    <cfRule type="expression" dxfId="222" priority="17">
+    <cfRule type="expression" dxfId="226" priority="17">
       <formula>OR($E12="Needs answer",$E12="Explain why",LEFT($E12,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:E13">
-    <cfRule type="expression" dxfId="223" priority="18">
+    <cfRule type="expression" dxfId="227" priority="18">
       <formula>$E13="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:E13">
-    <cfRule type="expression" dxfId="224" priority="19">
+    <cfRule type="expression" dxfId="228" priority="19">
       <formula>OR($E13="Needs answer",$E13="Explain why",LEFT($E13,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B14:E14">
-    <cfRule type="expression" dxfId="225" priority="20">
+    <cfRule type="expression" dxfId="229" priority="20">
       <formula>$E14="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E14:E14">
-    <cfRule type="expression" dxfId="226" priority="21">
+    <cfRule type="expression" dxfId="230" priority="21">
       <formula>OR($E14="Needs answer",$E14="Explain why",LEFT($E14,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D14:D14">
-    <cfRule type="expression" dxfId="227" priority="22">
+    <cfRule type="expression" dxfId="231" priority="22">
       <formula>OR($C14="Unable to assess",$C14="unable_to_assess")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15:E15">
-    <cfRule type="expression" dxfId="228" priority="23">
+    <cfRule type="expression" dxfId="232" priority="23">
       <formula>$E15="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E15:E15">
-    <cfRule type="expression" dxfId="229" priority="24">
+    <cfRule type="expression" dxfId="233" priority="24">
       <formula>OR($E15="Needs answer",$E15="Explain why",LEFT($E15,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16:E16">
-    <cfRule type="expression" dxfId="230" priority="25">
+    <cfRule type="expression" dxfId="234" priority="25">
       <formula>$E16="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E16:E16">
-    <cfRule type="expression" dxfId="231" priority="26">
+    <cfRule type="expression" dxfId="235" priority="26">
       <formula>OR($E16="Needs answer",$E16="Explain why",LEFT($E16,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17:E17">
-    <cfRule type="expression" dxfId="232" priority="27">
+    <cfRule type="expression" dxfId="236" priority="27">
       <formula>$E17="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E17:E17">
-    <cfRule type="expression" dxfId="233" priority="28">
+    <cfRule type="expression" dxfId="237" priority="28">
       <formula>OR($E17="Needs answer",$E17="Explain why",LEFT($E17,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D17:D17">
-    <cfRule type="expression" dxfId="234" priority="29">
+    <cfRule type="expression" dxfId="238" priority="29">
       <formula>OR($C17="Unable to assess",$C17="unable_to_assess")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:E18">
-    <cfRule type="expression" dxfId="235" priority="30">
+    <cfRule type="expression" dxfId="239" priority="30">
       <formula>$E18="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E18:E18">
-    <cfRule type="expression" dxfId="236" priority="31">
+    <cfRule type="expression" dxfId="240" priority="31">
       <formula>OR($E18="Needs answer",$E18="Explain why",LEFT($E18,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19:E19">
-    <cfRule type="expression" dxfId="237" priority="32">
+    <cfRule type="expression" dxfId="241" priority="32">
       <formula>$E19="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E19:E19">
-    <cfRule type="expression" dxfId="238" priority="33">
+    <cfRule type="expression" dxfId="242" priority="33">
       <formula>OR($E19="Needs answer",$E19="Explain why",LEFT($E19,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:E20">
-    <cfRule type="expression" dxfId="239" priority="34">
+    <cfRule type="expression" dxfId="243" priority="34">
       <formula>$E20="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E20:E20">
-    <cfRule type="expression" dxfId="240" priority="35">
+    <cfRule type="expression" dxfId="244" priority="35">
       <formula>OR($E20="Needs answer",$E20="Explain why",LEFT($E20,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21:E21">
-    <cfRule type="expression" dxfId="241" priority="36">
+    <cfRule type="expression" dxfId="245" priority="36">
       <formula>$E21="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E21:E21">
-    <cfRule type="expression" dxfId="242" priority="37">
+    <cfRule type="expression" dxfId="246" priority="37">
       <formula>OR($E21="Needs answer",$E21="Explain why",LEFT($E21,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:E22">
-    <cfRule type="expression" dxfId="243" priority="38">
+    <cfRule type="expression" dxfId="247" priority="38">
       <formula>$E22="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E22:E22">
-    <cfRule type="expression" dxfId="244" priority="39">
+    <cfRule type="expression" dxfId="248" priority="39">
       <formula>OR($E22="Needs answer",$E22="Explain why",LEFT($E22,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:E23">
-    <cfRule type="expression" dxfId="245" priority="40">
+    <cfRule type="expression" dxfId="249" priority="40">
       <formula>$E23="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E23:E23">
-    <cfRule type="expression" dxfId="246" priority="41">
+    <cfRule type="expression" dxfId="250" priority="41">
       <formula>OR($E23="Needs answer",$E23="Explain why",LEFT($E23,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24:E24">
-    <cfRule type="expression" dxfId="247" priority="42">
+    <cfRule type="expression" dxfId="251" priority="42">
       <formula>$E24="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E24:E24">
-    <cfRule type="expression" dxfId="248" priority="43">
+    <cfRule type="expression" dxfId="252" priority="43">
       <formula>OR($E24="Needs answer",$E24="Explain why",LEFT($E24,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25:E25">
-    <cfRule type="expression" dxfId="249" priority="44">
+    <cfRule type="expression" dxfId="253" priority="44">
       <formula>$E25="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25:E25">
-    <cfRule type="expression" dxfId="250" priority="45">
+    <cfRule type="expression" dxfId="254" priority="45">
       <formula>OR($E25="Needs answer",$E25="Explain why",LEFT($E25,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:E26">
-    <cfRule type="expression" dxfId="251" priority="46">
+    <cfRule type="expression" dxfId="255" priority="46">
       <formula>$E26="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26:E26">
-    <cfRule type="expression" dxfId="252" priority="47">
+    <cfRule type="expression" dxfId="256" priority="47">
       <formula>OR($E26="Needs answer",$E26="Explain why",LEFT($E26,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:E27">
-    <cfRule type="expression" dxfId="253" priority="48">
+    <cfRule type="expression" dxfId="257" priority="48">
       <formula>$E27="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27:E27">
-    <cfRule type="expression" dxfId="254" priority="49">
+    <cfRule type="expression" dxfId="258" priority="49">
       <formula>OR($E27="Needs answer",$E27="Explain why",LEFT($E27,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28:E28">
-    <cfRule type="expression" dxfId="255" priority="50">
+    <cfRule type="expression" dxfId="259" priority="50">
       <formula>$E28="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E28:E28">
-    <cfRule type="expression" dxfId="256" priority="51">
+    <cfRule type="expression" dxfId="260" priority="51">
       <formula>OR($E28="Needs answer",$E28="Explain why",LEFT($E28,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29:E29">
-    <cfRule type="expression" dxfId="257" priority="52">
+    <cfRule type="expression" dxfId="261" priority="52">
       <formula>$E29="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E29:E29">
-    <cfRule type="expression" dxfId="258" priority="53">
+    <cfRule type="expression" dxfId="262" priority="53">
       <formula>OR($E29="Needs answer",$E29="Explain why",LEFT($E29,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:E30">
-    <cfRule type="expression" dxfId="259" priority="54">
+    <cfRule type="expression" dxfId="263" priority="54">
       <formula>$E30="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E30:E30">
-    <cfRule type="expression" dxfId="260" priority="55">
+    <cfRule type="expression" dxfId="264" priority="55">
       <formula>OR($E30="Needs answer",$E30="Explain why",LEFT($E30,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31:E31">
-    <cfRule type="expression" dxfId="261" priority="56">
+    <cfRule type="expression" dxfId="265" priority="56">
       <formula>$E31="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E31:E31">
-    <cfRule type="expression" dxfId="262" priority="57">
+    <cfRule type="expression" dxfId="266" priority="57">
       <formula>OR($E31="Needs answer",$E31="Explain why",LEFT($E31,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32:E32">
-    <cfRule type="expression" dxfId="263" priority="58">
+    <cfRule type="expression" dxfId="267" priority="58">
       <formula>$E32="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E32:E32">
-    <cfRule type="expression" dxfId="264" priority="59">
+    <cfRule type="expression" dxfId="268" priority="59">
       <formula>OR($E32="Needs answer",$E32="Explain why",LEFT($E32,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33:E33">
-    <cfRule type="expression" dxfId="265" priority="60">
+    <cfRule type="expression" dxfId="269" priority="60">
       <formula>$E33="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E33:E33">
-    <cfRule type="expression" dxfId="266" priority="61">
+    <cfRule type="expression" dxfId="270" priority="61">
       <formula>OR($E33="Needs answer",$E33="Explain why",LEFT($E33,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B34:E34">
-    <cfRule type="expression" dxfId="267" priority="62">
+    <cfRule type="expression" dxfId="271" priority="62">
       <formula>$E34="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E34:E34">
-    <cfRule type="expression" dxfId="268" priority="63">
+    <cfRule type="expression" dxfId="272" priority="63">
       <formula>OR($E34="Needs answer",$E34="Explain why",LEFT($E34,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B35:E35">
-    <cfRule type="expression" dxfId="269" priority="64">
+    <cfRule type="expression" dxfId="273" priority="64">
       <formula>$E35="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E35:E35">
-    <cfRule type="expression" dxfId="270" priority="65">
+    <cfRule type="expression" dxfId="274" priority="65">
       <formula>OR($E35="Needs answer",$E35="Explain why",LEFT($E35,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B36:E36">
-    <cfRule type="expression" dxfId="271" priority="66">
+    <cfRule type="expression" dxfId="275" priority="66">
       <formula>$E36="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E36:E36">
-    <cfRule type="expression" dxfId="272" priority="67">
+    <cfRule type="expression" dxfId="276" priority="67">
       <formula>OR($E36="Needs answer",$E36="Explain why",LEFT($E36,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B37:E37">
-    <cfRule type="expression" dxfId="273" priority="68">
+    <cfRule type="expression" dxfId="277" priority="68">
       <formula>$E37="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E37:E37">
-    <cfRule type="expression" dxfId="274" priority="69">
+    <cfRule type="expression" dxfId="278" priority="69">
       <formula>OR($E37="Needs answer",$E37="Explain why",LEFT($E37,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B38:E38">
-    <cfRule type="expression" dxfId="275" priority="70">
+    <cfRule type="expression" dxfId="279" priority="70">
       <formula>$E38="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E38:E38">
-    <cfRule type="expression" dxfId="276" priority="71">
+    <cfRule type="expression" dxfId="280" priority="71">
       <formula>OR($E38="Needs answer",$E38="Explain why",LEFT($E38,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B39:E39">
-    <cfRule type="expression" dxfId="277" priority="72">
+    <cfRule type="expression" dxfId="281" priority="72">
       <formula>$E39="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E39:E39">
-    <cfRule type="expression" dxfId="278" priority="73">
+    <cfRule type="expression" dxfId="282" priority="73">
       <formula>OR($E39="Needs answer",$E39="Explain why",LEFT($E39,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B40:E40">
-    <cfRule type="expression" dxfId="279" priority="74">
+    <cfRule type="expression" dxfId="283" priority="74">
       <formula>$E40="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E40:E40">
-    <cfRule type="expression" dxfId="280" priority="75">
+    <cfRule type="expression" dxfId="284" priority="75">
       <formula>OR($E40="Needs answer",$E40="Explain why",LEFT($E40,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B41:E41">
-    <cfRule type="expression" dxfId="281" priority="76">
+    <cfRule type="expression" dxfId="285" priority="76">
       <formula>$E41="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E41:E41">
-    <cfRule type="expression" dxfId="282" priority="77">
+    <cfRule type="expression" dxfId="286" priority="77">
       <formula>OR($E41="Needs answer",$E41="Explain why",LEFT($E41,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6294,23 +6348,23 @@
         <v>Optional</v>
       </c>
     </row>
-    <row r="10" ht="34" customHeight="1">
+    <row r="10" ht="72" customHeight="1">
       <c r="A10" s="3" t="str">
-        <v>forensic_involvement</v>
+        <v>forensic_history</v>
       </c>
       <c r="B10" s="13" t="str">
-        <v>Forensic involvement</v>
+        <v>Forensic history</v>
       </c>
       <c r="C10" t="str" s="50"/>
       <c r="D10" t="str" s="48"/>
       <c r="E10" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C10))&gt;0,LEN(TRIM(D10))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D10))&gt;0,NOT(OR(LOWER(TRIM(C10))="unable to assess",C10="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C10))="unable to assess",C10="unable_to_assess"),NOT(LEN(TRIM(D10))&gt;0)),"Explain why",IF(LEN(TRIM(C10))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
-        <v>Needs answer</v>
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C10))&gt;0,LEN(TRIM(D10))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D10))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D10))&gt;0)),"Explain why",IF(LEN(TRIM(C10))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
       </c>
     </row>
     <row r="11" ht="72" customHeight="1">
       <c r="A11" s="3" t="str">
-        <v>forensic_involvement_details</v>
+        <v>forensic_timeline</v>
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
@@ -6320,7 +6374,7 @@
               <sz val="12"/>
               <color rgb="FF233B32"/>
             </rPr>
-            <t>Forensic involvement details</t>
+            <t>Forensic timeline</t>
           </r>
           <r>
             <rPr>
@@ -6329,304 +6383,367 @@
               <color rgb="FF59675F"/>
             </rPr>
             <t xml:space="preserve">
-Only if Forensic involvement is Yes.</t>
+Optional. Record an approximate date, event, and outcome in each row.</t>
           </r>
         </is>
       </c>
       <c r="C11" t="str" s="50"/>
       <c r="D11" t="str" s="48"/>
       <c r="E11" s="16" t="str">
-        <f>IF(NOT(AND(OR(LOWER(TRIM('10 Decisions and legal support'!$C$10&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$10&amp;""))="yes"))),IF(OR(LEN(TRIM(C11))&gt;0,LEN(TRIM(D11))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D11))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D11))&gt;0)),"Explain why",IF(LEN(TRIM(C11))&gt;0,"Answered",IF(OR(LOWER(TRIM('10 Decisions and legal support'!$C$10&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$10&amp;""))="yes"),"Needs answer","Optional")))))</f>
-        <v>Not applicable</v>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C11&amp;""&amp;C12&amp;""&amp;C13&amp;""&amp;C14&amp;""&amp;C15&amp;""&amp;C16&amp;""&amp;C17&amp;""&amp;C18&amp;""&amp;C19&amp;""&amp;C20&amp;""&amp;C21&amp;""&amp;C22&amp;""&amp;C23&amp;""&amp;C24))&gt;0,LEN(TRIM(D11))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D11))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D11))&gt;0)),"Explain why",IF(LEN(TRIM(C11&amp;""&amp;C12&amp;""&amp;C13&amp;""&amp;C14&amp;""&amp;C15&amp;""&amp;C16&amp;""&amp;C17&amp;""&amp;C18&amp;""&amp;C19&amp;""&amp;C20&amp;""&amp;C21&amp;""&amp;C22&amp;""&amp;C23&amp;""&amp;C24))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="12" ht="88" customHeight="1" hidden="1">
       <c r="A12" s="3" t="str">
+        <v>forensic_timeline:1</v>
+      </c>
+      <c r="B12" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C12" t="str" s="57"/>
+      <c r="D12" s="3" t="str"/>
+      <c r="E12" s="3"/>
+    </row>
+    <row r="13" ht="88" customHeight="1" hidden="1">
+      <c r="A13" s="3" t="str">
+        <v>forensic_timeline:2</v>
+      </c>
+      <c r="B13" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C13" t="str" s="57"/>
+      <c r="D13" s="3" t="str"/>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" ht="88" customHeight="1" hidden="1">
+      <c r="A14" s="3" t="str">
+        <v>forensic_timeline:3</v>
+      </c>
+      <c r="B14" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C14" t="str" s="57"/>
+      <c r="D14" s="3" t="str"/>
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" ht="88" customHeight="1" hidden="1">
+      <c r="A15" s="3" t="str">
+        <v>forensic_timeline:4</v>
+      </c>
+      <c r="B15" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C15" t="str" s="57"/>
+      <c r="D15" s="3" t="str"/>
+      <c r="E15" s="3"/>
+    </row>
+    <row r="16" ht="88" customHeight="1" hidden="1">
+      <c r="A16" s="3" t="str">
+        <v>forensic_timeline:5</v>
+      </c>
+      <c r="B16" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C16" t="str" s="57"/>
+      <c r="D16" s="3" t="str"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" ht="88" customHeight="1" hidden="1">
+      <c r="A17" s="3" t="str">
+        <v>forensic_timeline:6</v>
+      </c>
+      <c r="B17" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C17" t="str" s="57"/>
+      <c r="D17" s="3" t="str"/>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" ht="88" customHeight="1" hidden="1">
+      <c r="A18" s="3" t="str">
+        <v>forensic_timeline:7</v>
+      </c>
+      <c r="B18" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C18" t="str" s="57"/>
+      <c r="D18" s="3" t="str"/>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" ht="88" customHeight="1" hidden="1">
+      <c r="A19" s="3" t="str">
+        <v>forensic_timeline:8</v>
+      </c>
+      <c r="B19" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C19" t="str" s="57"/>
+      <c r="D19" s="3" t="str"/>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" ht="88" customHeight="1" hidden="1">
+      <c r="A20" s="3" t="str">
+        <v>forensic_timeline:9</v>
+      </c>
+      <c r="B20" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C20" t="str" s="57"/>
+      <c r="D20" s="3" t="str"/>
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" ht="88" customHeight="1" hidden="1">
+      <c r="A21" s="3" t="str">
+        <v>forensic_timeline:10</v>
+      </c>
+      <c r="B21" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C21" t="str" s="57"/>
+      <c r="D21" s="3" t="str"/>
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" ht="88" customHeight="1" hidden="1">
+      <c r="A22" s="3" t="str">
+        <v>forensic_timeline:11</v>
+      </c>
+      <c r="B22" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C22" t="str" s="57"/>
+      <c r="D22" s="3" t="str"/>
+      <c r="E22" s="3"/>
+    </row>
+    <row r="23" ht="88" customHeight="1" hidden="1">
+      <c r="A23" s="3" t="str">
+        <v>forensic_timeline:12</v>
+      </c>
+      <c r="B23" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C23" t="str" s="57"/>
+      <c r="D23" s="3" t="str"/>
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" ht="88" customHeight="1" hidden="1">
+      <c r="A24" s="3" t="str">
+        <v>forensic_timeline:13</v>
+      </c>
+      <c r="B24" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C24" t="str" s="57"/>
+      <c r="D24" s="3" t="str"/>
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="3" t="str">
+        <v>pc290_registration</v>
+      </c>
+      <c r="B25" s="13" t="str">
+        <v>PC 290 registration</v>
+      </c>
+      <c r="C25" t="str" s="50"/>
+      <c r="D25" t="str" s="48"/>
+      <c r="E25" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C25))&gt;0,LEN(TRIM(D25))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D25))&gt;0,NOT(OR(LOWER(TRIM(C25))="unable to assess",C25="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C25))="unable to assess",C25="unable_to_assess"),NOT(LEN(TRIM(D25))&gt;0)),"Explain why",IF(LEN(TRIM(C25))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
+        <v>Needs answer</v>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="3" t="str">
+        <v>arson_history</v>
+      </c>
+      <c r="B26" s="13" t="str">
+        <v>Arson history</v>
+      </c>
+      <c r="C26" t="str" s="50"/>
+      <c r="D26" t="str" s="48"/>
+      <c r="E26" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C26))&gt;0,LEN(TRIM(D26))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D26))&gt;0,NOT(OR(LOWER(TRIM(C26))="unable to assess",C26="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C26))="unable to assess",C26="unable_to_assess"),NOT(LEN(TRIM(D26))&gt;0)),"Explain why",IF(LEN(TRIM(C26))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
+        <v>Needs answer</v>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="3" t="str">
+        <v>diversion_client</v>
+      </c>
+      <c r="B27" s="13" t="str">
+        <v>Diversion client</v>
+      </c>
+      <c r="C27" t="str" s="50"/>
+      <c r="D27" t="str" s="48"/>
+      <c r="E27" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C27))&gt;0,LEN(TRIM(D27))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D27))&gt;0,NOT(OR(LOWER(TRIM(C27))="unable to assess",C27="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C27))="unable to assess",C27="unable_to_assess"),NOT(LEN(TRIM(D27))&gt;0)),"Explain why",IF(LEN(TRIM(C27))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
+        <v>Needs answer</v>
+      </c>
+    </row>
+    <row r="28" ht="72" customHeight="1">
+      <c r="A28" s="3" t="str">
+        <v>court_requirements</v>
+      </c>
+      <c r="B28" s="13" t="str">
+        <v>Court requirements</v>
+      </c>
+      <c r="C28" t="str" s="50"/>
+      <c r="D28" t="str" s="48"/>
+      <c r="E28" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C28))&gt;0,LEN(TRIM(D28))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D28))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D28))&gt;0)),"Explain why",IF(LEN(TRIM(C28))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="29" ht="72" customHeight="1">
+      <c r="A29" s="3" t="str">
+        <v>court_dates</v>
+      </c>
+      <c r="B29" s="13" t="str">
+        <v>Court dates</v>
+      </c>
+      <c r="C29" t="str" s="50"/>
+      <c r="D29" t="str" s="48"/>
+      <c r="E29" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C29))&gt;0,LEN(TRIM(D29))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D29))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D29))&gt;0)),"Explain why",IF(LEN(TRIM(C29))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="30" ht="72" customHeight="1">
+      <c r="A30" s="3" t="str">
+        <v>probation_parole_justice</v>
+      </c>
+      <c r="B30" s="13" t="str">
+        <v>Probation / parole / justice</v>
+      </c>
+      <c r="C30" t="str" s="50"/>
+      <c r="D30" t="str" s="48"/>
+      <c r="E30" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C30))&gt;0,LEN(TRIM(D30))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D30))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D30))&gt;0)),"Explain why",IF(LEN(TRIM(C30))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="31" ht="34" customHeight="1">
+      <c r="A31" s="3" t="str">
+        <v>forensic_involvement</v>
+      </c>
+      <c r="B31" s="13" t="str">
+        <v>Forensic involvement</v>
+      </c>
+      <c r="C31" t="str" s="50"/>
+      <c r="D31" t="str" s="48"/>
+      <c r="E31" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C31))&gt;0,LEN(TRIM(D31))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D31))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D31))&gt;0)),"Explain why",IF(LEN(TRIM(C31))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="3" t="str">
+        <v>forensic_involvement_details</v>
+      </c>
+      <c r="B32" s="13" t="str">
+        <v>Forensic involvement details</v>
+      </c>
+      <c r="C32" t="str" s="50"/>
+      <c r="D32" t="str" s="48"/>
+      <c r="E32" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C32))&gt;0,LEN(TRIM(D32))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D32))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D32))&gt;0)),"Explain why",IF(LEN(TRIM(C32))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="33" ht="34" customHeight="1">
+      <c r="A33" s="3" t="str">
         <v>arrest_history</v>
       </c>
-      <c r="B12" s="13" t="str">
+      <c r="B33" s="13" t="str">
         <v>History of arrest</v>
       </c>
-      <c r="C12" t="str" s="50"/>
-      <c r="D12" t="str" s="48"/>
-      <c r="E12" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C12))&gt;0,LEN(TRIM(D12))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D12))&gt;0,NOT(OR(LOWER(TRIM(C12))="unable to assess",C12="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C12))="unable to assess",C12="unable_to_assess"),NOT(LEN(TRIM(D12))&gt;0)),"Explain why",IF(LEN(TRIM(C12))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
-        <v>Needs answer</v>
-      </c>
-    </row>
-    <row r="13" ht="39" customHeight="1">
-      <c r="A13" s="3" t="str">
+      <c r="C33" t="str" s="50"/>
+      <c r="D33" t="str" s="48"/>
+      <c r="E33" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C33))&gt;0,LEN(TRIM(D33))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D33))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D33))&gt;0)),"Explain why",IF(LEN(TRIM(C33))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="34" ht="34" customHeight="1">
+      <c r="A34" s="3" t="str">
         <v>most_recent_arrest_date</v>
       </c>
-      <c r="B13" s="21" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="12"/>
-              <color rgb="FF233B32"/>
-            </rPr>
-            <t>Most recent arrest date</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="0"/>
-              <sz val="10"/>
-              <color rgb="FF59675F"/>
-            </rPr>
-            <t xml:space="preserve">
-Only if History of arrest is Yes.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C13" t="str" s="51"/>
-      <c r="D13" t="str" s="48"/>
-      <c r="E13" s="16" t="str">
-        <f>IF(NOT(AND(OR(LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes"))),IF(OR(LEN(TRIM(C13))&gt;0,LEN(TRIM(D13))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D13))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D13))&gt;0)),"Explain why",IF(LEN(TRIM(C13))&gt;0,"Answered",IF(OR(LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes"),"Needs answer","Optional")))))</f>
-        <v>Not applicable</v>
-      </c>
-    </row>
-    <row r="14" ht="39" customHeight="1">
-      <c r="A14" s="3" t="str">
+      <c r="B34" s="13" t="str">
+        <v>Most recent arrest date</v>
+      </c>
+      <c r="C34" t="str" s="51"/>
+      <c r="D34" t="str" s="48"/>
+      <c r="E34" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C34))&gt;0,LEN(TRIM(D34))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D34))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D34))&gt;0)),"Explain why",IF(LEN(TRIM(C34))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="35" ht="34" customHeight="1">
+      <c r="A35" s="3" t="str">
         <v>most_recent_arrest_charge</v>
       </c>
-      <c r="B14" s="21" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="12"/>
-              <color rgb="FF233B32"/>
-            </rPr>
-            <t>Most recent arrest charge</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="0"/>
-              <sz val="10"/>
-              <color rgb="FF59675F"/>
-            </rPr>
-            <t xml:space="preserve">
-Only if History of arrest is Yes.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C14" t="str" s="50"/>
-      <c r="D14" t="str" s="48"/>
-      <c r="E14" s="16" t="str">
-        <f>IF(NOT(AND(OR(LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes"))),IF(OR(LEN(TRIM(C14))&gt;0,LEN(TRIM(D14))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D14))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D14))&gt;0)),"Explain why",IF(LEN(TRIM(C14))&gt;0,"Answered",IF(OR(LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes"),"Needs answer","Optional")))))</f>
-        <v>Not applicable</v>
-      </c>
-    </row>
-    <row r="15" ht="39" customHeight="1">
-      <c r="A15" s="3" t="str">
+      <c r="B35" s="13" t="str">
+        <v>Most recent arrest charge</v>
+      </c>
+      <c r="C35" t="str" s="50"/>
+      <c r="D35" t="str" s="48"/>
+      <c r="E35" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C35))&gt;0,LEN(TRIM(D35))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D35))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D35))&gt;0)),"Explain why",IF(LEN(TRIM(C35))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="36" ht="34" customHeight="1">
+      <c r="A36" s="3" t="str">
         <v>most_recent_arrest_jail_time</v>
       </c>
-      <c r="B15" s="21" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="12"/>
-              <color rgb="FF233B32"/>
-            </rPr>
-            <t>Time in jail</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="0"/>
-              <sz val="10"/>
-              <color rgb="FF59675F"/>
-            </rPr>
-            <t xml:space="preserve">
-Only if History of arrest is Yes.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C15" t="str" s="50"/>
-      <c r="D15" t="str" s="48"/>
-      <c r="E15" s="16" t="str">
-        <f>IF(NOT(AND(OR(LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes"))),IF(OR(LEN(TRIM(C15))&gt;0,LEN(TRIM(D15))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D15))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D15))&gt;0)),"Explain why",IF(LEN(TRIM(C15))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Not applicable</v>
-      </c>
-    </row>
-    <row r="16" ht="39" customHeight="1">
-      <c r="A16" s="3" t="str">
+      <c r="B36" s="13" t="str">
+        <v>Time in jail</v>
+      </c>
+      <c r="C36" t="str" s="50"/>
+      <c r="D36" t="str" s="48"/>
+      <c r="E36" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C36))&gt;0,LEN(TRIM(D36))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D36))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D36))&gt;0)),"Explain why",IF(LEN(TRIM(C36))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="37" ht="34" customHeight="1">
+      <c r="A37" s="3" t="str">
         <v>arrest_in_last_two_years</v>
       </c>
-      <c r="B16" s="21" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="12"/>
-              <color rgb="FF233B32"/>
-            </rPr>
-            <t>Arrest in the last two years</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="0"/>
-              <sz val="10"/>
-              <color rgb="FF59675F"/>
-            </rPr>
-            <t xml:space="preserve">
-Only if History of arrest is Yes.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C16" t="str" s="50"/>
-      <c r="D16" t="str" s="48"/>
-      <c r="E16" s="16" t="str">
-        <f>IF(NOT(AND(OR(LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes"))),IF(OR(LEN(TRIM(C16))&gt;0,LEN(TRIM(D16))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D16))&gt;0,NOT(OR(LOWER(TRIM(C16))="unable to assess",C16="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C16))="unable to assess",C16="unable_to_assess"),NOT(LEN(TRIM(D16))&gt;0)),"Explain why",IF(LEN(TRIM(C16))&gt;0,"Answered",IF(OR(LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes"),"Needs answer","Optional")))))</f>
-        <v>Not applicable</v>
-      </c>
-    </row>
-    <row r="17" ht="72" customHeight="1">
-      <c r="A17" s="3" t="str">
+      <c r="B37" s="13" t="str">
+        <v>Arrest in the last two years</v>
+      </c>
+      <c r="C37" t="str" s="50"/>
+      <c r="D37" t="str" s="48"/>
+      <c r="E37" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C37))&gt;0,LEN(TRIM(D37))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D37))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D37))&gt;0)),"Explain why",IF(LEN(TRIM(C37))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="38" ht="34" customHeight="1">
+      <c r="A38" s="3" t="str">
         <v>arrest_last_two_years_details</v>
       </c>
-      <c r="B17" s="21" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="12"/>
-              <color rgb="FF233B32"/>
-            </rPr>
-            <t>Recent arrest details</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="0"/>
-              <sz val="10"/>
-              <color rgb="FF59675F"/>
-            </rPr>
-            <t xml:space="preserve">
-Only if Arrest in the last two years is Yes.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C17" t="str" s="50"/>
-      <c r="D17" t="str" s="48"/>
-      <c r="E17" s="16" t="str">
-        <f>IF(NOT(AND(OR(LOWER(TRIM('10 Decisions and legal support'!$C$16&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$16&amp;""))="yes"),OR(LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes"))),IF(OR(LEN(TRIM(C17))&gt;0,LEN(TRIM(D17))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D17))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D17))&gt;0)),"Explain why",IF(LEN(TRIM(C17))&gt;0,"Answered",IF(OR(LOWER(TRIM('10 Decisions and legal support'!$C$16&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$16&amp;""))="yes"),"Needs answer","Optional")))))</f>
-        <v>Not applicable</v>
-      </c>
-    </row>
-    <row r="18" ht="39" customHeight="1">
-      <c r="A18" s="3" t="str">
+      <c r="B38" s="13" t="str">
+        <v>Recent arrest details</v>
+      </c>
+      <c r="C38" t="str" s="50"/>
+      <c r="D38" t="str" s="48"/>
+      <c r="E38" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C38))&gt;0,LEN(TRIM(D38))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D38))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D38))&gt;0)),"Explain why",IF(LEN(TRIM(C38))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="39" ht="34" customHeight="1">
+      <c r="A39" s="3" t="str">
         <v>total_arrests</v>
       </c>
-      <c r="B18" s="21" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="12"/>
-              <color rgb="FF233B32"/>
-            </rPr>
-            <t>Total recorded arrests</t>
-          </r>
-          <r>
-            <rPr>
-              <b val="0"/>
-              <sz val="10"/>
-              <color rgb="FF59675F"/>
-            </rPr>
-            <t xml:space="preserve">
-Only if History of arrest is Yes.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C18" t="str" s="58"/>
-      <c r="D18" t="str" s="48"/>
-      <c r="E18" s="16" t="str">
-        <f>IF(NOT(AND(OR(LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes"))),IF(OR(LEN(TRIM(C18))&gt;0,LEN(TRIM(D18))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D18))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D18))&gt;0)),"Explain why",IF(LEN(TRIM(C18))&gt;0,"Answered",IF(OR(LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes",LOWER(TRIM('10 Decisions and legal support'!$C$12&amp;""))="yes"),"Needs answer","Optional")))))</f>
-        <v>Not applicable</v>
-      </c>
-    </row>
-    <row r="19" ht="34" customHeight="1">
-      <c r="A19" s="3" t="str">
-        <v>pc290_registration</v>
-      </c>
-      <c r="B19" s="13" t="str">
-        <v>PC 290 registration</v>
-      </c>
-      <c r="C19" t="str" s="50"/>
-      <c r="D19" t="str" s="48"/>
-      <c r="E19" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C19))&gt;0,LEN(TRIM(D19))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D19))&gt;0,NOT(OR(LOWER(TRIM(C19))="unable to assess",C19="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C19))="unable to assess",C19="unable_to_assess"),NOT(LEN(TRIM(D19))&gt;0)),"Explain why",IF(LEN(TRIM(C19))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
-        <v>Needs answer</v>
-      </c>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="3" t="str">
-        <v>arson_history</v>
-      </c>
-      <c r="B20" s="13" t="str">
-        <v>Arson history</v>
-      </c>
-      <c r="C20" t="str" s="50"/>
-      <c r="D20" t="str" s="48"/>
-      <c r="E20" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C20))&gt;0,LEN(TRIM(D20))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D20))&gt;0,NOT(OR(LOWER(TRIM(C20))="unable to assess",C20="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C20))="unable to assess",C20="unable_to_assess"),NOT(LEN(TRIM(D20))&gt;0)),"Explain why",IF(LEN(TRIM(C20))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
-        <v>Needs answer</v>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="3" t="str">
-        <v>diversion_client</v>
-      </c>
-      <c r="B21" s="13" t="str">
-        <v>Diversion client</v>
-      </c>
-      <c r="C21" t="str" s="50"/>
-      <c r="D21" t="str" s="48"/>
-      <c r="E21" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C21))&gt;0,LEN(TRIM(D21))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D21))&gt;0,NOT(OR(LOWER(TRIM(C21))="unable to assess",C21="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C21))="unable to assess",C21="unable_to_assess"),NOT(LEN(TRIM(D21))&gt;0)),"Explain why",IF(LEN(TRIM(C21))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
-        <v>Needs answer</v>
-      </c>
-    </row>
-    <row r="22" ht="72" customHeight="1">
-      <c r="A22" s="3" t="str">
-        <v>court_requirements</v>
-      </c>
-      <c r="B22" s="13" t="str">
-        <v>Court requirements</v>
-      </c>
-      <c r="C22" t="str" s="50"/>
-      <c r="D22" t="str" s="48"/>
-      <c r="E22" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C22))&gt;0,LEN(TRIM(D22))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D22))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D22))&gt;0)),"Explain why",IF(LEN(TRIM(C22))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
-    </row>
-    <row r="23" ht="72" customHeight="1">
-      <c r="A23" s="3" t="str">
-        <v>court_dates</v>
-      </c>
-      <c r="B23" s="13" t="str">
-        <v>Court dates</v>
-      </c>
-      <c r="C23" t="str" s="50"/>
-      <c r="D23" t="str" s="48"/>
-      <c r="E23" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C23))&gt;0,LEN(TRIM(D23))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D23))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D23))&gt;0)),"Explain why",IF(LEN(TRIM(C23))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
-    </row>
-    <row r="24" ht="72" customHeight="1">
-      <c r="A24" s="3" t="str">
-        <v>probation_parole_justice</v>
-      </c>
-      <c r="B24" s="13" t="str">
-        <v>Probation / parole / justice</v>
-      </c>
-      <c r="C24" t="str" s="50"/>
-      <c r="D24" t="str" s="48"/>
-      <c r="E24" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C24))&gt;0,LEN(TRIM(D24))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D24))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D24))&gt;0)),"Explain why",IF(LEN(TRIM(C24))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+      <c r="B39" s="13" t="str">
+        <v>Total recorded arrests</v>
+      </c>
+      <c r="C39" t="str" s="58"/>
+      <c r="D39" t="str" s="48"/>
+      <c r="E39" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C39))&gt;0,LEN(TRIM(D39))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D39))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D39))&gt;0)),"Explain why",IF(LEN(TRIM(C39))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
         <v>Optional</v>
       </c>
     </row>
@@ -6639,249 +6756,241 @@
     <mergeCell ref="B3:E3"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:E6">
-    <cfRule type="expression" dxfId="283" priority="1">
+    <cfRule type="expression" dxfId="287" priority="1">
       <formula>$E6="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6:E6">
-    <cfRule type="expression" dxfId="284" priority="2">
+    <cfRule type="expression" dxfId="288" priority="2">
       <formula>OR($E6="Needs answer",$E6="Explain why",LEFT($E6,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:E7">
-    <cfRule type="expression" dxfId="285" priority="3">
+    <cfRule type="expression" dxfId="289" priority="3">
       <formula>$E7="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7:E7">
-    <cfRule type="expression" dxfId="286" priority="4">
+    <cfRule type="expression" dxfId="290" priority="4">
       <formula>OR($E7="Needs answer",$E7="Explain why",LEFT($E7,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:E8">
-    <cfRule type="expression" dxfId="287" priority="5">
+    <cfRule type="expression" dxfId="291" priority="5">
       <formula>$E8="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8:E8">
-    <cfRule type="expression" dxfId="288" priority="6">
+    <cfRule type="expression" dxfId="292" priority="6">
       <formula>OR($E8="Needs answer",$E8="Explain why",LEFT($E8,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:E9">
-    <cfRule type="expression" dxfId="289" priority="7">
+    <cfRule type="expression" dxfId="293" priority="7">
       <formula>$E9="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9:E9">
-    <cfRule type="expression" dxfId="290" priority="8">
+    <cfRule type="expression" dxfId="294" priority="8">
       <formula>OR($E9="Needs answer",$E9="Explain why",LEFT($E9,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:E10">
-    <cfRule type="expression" dxfId="291" priority="9">
+    <cfRule type="expression" dxfId="295" priority="9">
       <formula>$E10="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10:E10">
-    <cfRule type="expression" dxfId="292" priority="10">
+    <cfRule type="expression" dxfId="296" priority="10">
       <formula>OR($E10="Needs answer",$E10="Explain why",LEFT($E10,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D10:D10">
-    <cfRule type="expression" dxfId="293" priority="11">
-      <formula>OR($C10="Unable to assess",$C10="unable_to_assess")</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B11:E11">
-    <cfRule type="expression" dxfId="294" priority="12">
+    <cfRule type="expression" dxfId="297" priority="11">
       <formula>$E11="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11:E11">
-    <cfRule type="expression" dxfId="295" priority="13">
+    <cfRule type="expression" dxfId="298" priority="12">
       <formula>OR($E11="Needs answer",$E11="Explain why",LEFT($E11,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B12:E12">
-    <cfRule type="expression" dxfId="296" priority="14">
-      <formula>$E12="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E12:E12">
-    <cfRule type="expression" dxfId="297" priority="15">
-      <formula>OR($E12="Needs answer",$E12="Explain why",LEFT($E12,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D12:D12">
-    <cfRule type="expression" dxfId="298" priority="16">
-      <formula>OR($C12="Unable to assess",$C12="unable_to_assess")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13:E13">
-    <cfRule type="expression" dxfId="299" priority="17">
-      <formula>$E13="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E13:E13">
-    <cfRule type="expression" dxfId="300" priority="18">
-      <formula>OR($E13="Needs answer",$E13="Explain why",LEFT($E13,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B14:E14">
-    <cfRule type="expression" dxfId="301" priority="19">
-      <formula>$E14="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E14:E14">
-    <cfRule type="expression" dxfId="302" priority="20">
-      <formula>OR($E14="Needs answer",$E14="Explain why",LEFT($E14,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:E15">
-    <cfRule type="expression" dxfId="303" priority="21">
-      <formula>$E15="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E15:E15">
-    <cfRule type="expression" dxfId="304" priority="22">
-      <formula>OR($E15="Needs answer",$E15="Explain why",LEFT($E15,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B16:E16">
-    <cfRule type="expression" dxfId="305" priority="23">
-      <formula>$E16="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E16:E16">
-    <cfRule type="expression" dxfId="306" priority="24">
-      <formula>OR($E16="Needs answer",$E16="Explain why",LEFT($E16,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D16:D16">
-    <cfRule type="expression" dxfId="307" priority="25">
-      <formula>OR($C16="Unable to assess",$C16="unable_to_assess")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B17:E17">
-    <cfRule type="expression" dxfId="308" priority="26">
-      <formula>$E17="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E17:E17">
-    <cfRule type="expression" dxfId="309" priority="27">
-      <formula>OR($E17="Needs answer",$E17="Explain why",LEFT($E17,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B18:E18">
-    <cfRule type="expression" dxfId="310" priority="28">
-      <formula>$E18="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E18:E18">
-    <cfRule type="expression" dxfId="311" priority="29">
-      <formula>OR($E18="Needs answer",$E18="Explain why",LEFT($E18,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B19:E19">
-    <cfRule type="expression" dxfId="312" priority="30">
-      <formula>$E19="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E19:E19">
-    <cfRule type="expression" dxfId="313" priority="31">
-      <formula>OR($E19="Needs answer",$E19="Explain why",LEFT($E19,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D19:D19">
-    <cfRule type="expression" dxfId="314" priority="32">
-      <formula>OR($C19="Unable to assess",$C19="unable_to_assess")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B20:E20">
-    <cfRule type="expression" dxfId="315" priority="33">
-      <formula>$E20="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E20:E20">
-    <cfRule type="expression" dxfId="316" priority="34">
-      <formula>OR($E20="Needs answer",$E20="Explain why",LEFT($E20,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D20:D20">
-    <cfRule type="expression" dxfId="317" priority="35">
-      <formula>OR($C20="Unable to assess",$C20="unable_to_assess")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B21:E21">
-    <cfRule type="expression" dxfId="318" priority="36">
-      <formula>$E21="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E21:E21">
-    <cfRule type="expression" dxfId="319" priority="37">
-      <formula>OR($E21="Needs answer",$E21="Explain why",LEFT($E21,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D21:D21">
-    <cfRule type="expression" dxfId="320" priority="38">
-      <formula>OR($C21="Unable to assess",$C21="unable_to_assess")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B22:E22">
-    <cfRule type="expression" dxfId="321" priority="39">
-      <formula>$E22="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E22:E22">
-    <cfRule type="expression" dxfId="322" priority="40">
-      <formula>OR($E22="Needs answer",$E22="Explain why",LEFT($E22,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B23:E23">
-    <cfRule type="expression" dxfId="323" priority="41">
-      <formula>$E23="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E23:E23">
-    <cfRule type="expression" dxfId="324" priority="42">
-      <formula>OR($E23="Needs answer",$E23="Explain why",LEFT($E23,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B24:E24">
-    <cfRule type="expression" dxfId="325" priority="43">
-      <formula>$E24="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E24:E24">
-    <cfRule type="expression" dxfId="326" priority="44">
-      <formula>OR($E24="Needs answer",$E24="Explain why",LEFT($E24,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="8">
+  <conditionalFormatting sqref="B25:E25">
+    <cfRule type="expression" dxfId="299" priority="13">
+      <formula>$E25="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25:E25">
+    <cfRule type="expression" dxfId="300" priority="14">
+      <formula>OR($E25="Needs answer",$E25="Explain why",LEFT($E25,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D25:D25">
+    <cfRule type="expression" dxfId="301" priority="15">
+      <formula>OR($C25="Unable to assess",$C25="unable_to_assess")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B26:E26">
+    <cfRule type="expression" dxfId="302" priority="16">
+      <formula>$E26="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26:E26">
+    <cfRule type="expression" dxfId="303" priority="17">
+      <formula>OR($E26="Needs answer",$E26="Explain why",LEFT($E26,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D26:D26">
+    <cfRule type="expression" dxfId="304" priority="18">
+      <formula>OR($C26="Unable to assess",$C26="unable_to_assess")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B27:E27">
+    <cfRule type="expression" dxfId="305" priority="19">
+      <formula>$E27="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E27:E27">
+    <cfRule type="expression" dxfId="306" priority="20">
+      <formula>OR($E27="Needs answer",$E27="Explain why",LEFT($E27,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D27:D27">
+    <cfRule type="expression" dxfId="307" priority="21">
+      <formula>OR($C27="Unable to assess",$C27="unable_to_assess")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B28:E28">
+    <cfRule type="expression" dxfId="308" priority="22">
+      <formula>$E28="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E28:E28">
+    <cfRule type="expression" dxfId="309" priority="23">
+      <formula>OR($E28="Needs answer",$E28="Explain why",LEFT($E28,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29:E29">
+    <cfRule type="expression" dxfId="310" priority="24">
+      <formula>$E29="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E29:E29">
+    <cfRule type="expression" dxfId="311" priority="25">
+      <formula>OR($E29="Needs answer",$E29="Explain why",LEFT($E29,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30:E30">
+    <cfRule type="expression" dxfId="312" priority="26">
+      <formula>$E30="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E30:E30">
+    <cfRule type="expression" dxfId="313" priority="27">
+      <formula>OR($E30="Needs answer",$E30="Explain why",LEFT($E30,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B31:E31">
+    <cfRule type="expression" dxfId="314" priority="28">
+      <formula>$E31="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E31:E31">
+    <cfRule type="expression" dxfId="315" priority="29">
+      <formula>OR($E31="Needs answer",$E31="Explain why",LEFT($E31,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B32:E32">
+    <cfRule type="expression" dxfId="316" priority="30">
+      <formula>$E32="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E32:E32">
+    <cfRule type="expression" dxfId="317" priority="31">
+      <formula>OR($E32="Needs answer",$E32="Explain why",LEFT($E32,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B33:E33">
+    <cfRule type="expression" dxfId="318" priority="32">
+      <formula>$E33="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E33:E33">
+    <cfRule type="expression" dxfId="319" priority="33">
+      <formula>OR($E33="Needs answer",$E33="Explain why",LEFT($E33,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B34:E34">
+    <cfRule type="expression" dxfId="320" priority="34">
+      <formula>$E34="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E34:E34">
+    <cfRule type="expression" dxfId="321" priority="35">
+      <formula>OR($E34="Needs answer",$E34="Explain why",LEFT($E34,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B35:E35">
+    <cfRule type="expression" dxfId="322" priority="36">
+      <formula>$E35="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E35:E35">
+    <cfRule type="expression" dxfId="323" priority="37">
+      <formula>OR($E35="Needs answer",$E35="Explain why",LEFT($E35,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B36:E36">
+    <cfRule type="expression" dxfId="324" priority="38">
+      <formula>$E36="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E36:E36">
+    <cfRule type="expression" dxfId="325" priority="39">
+      <formula>OR($E36="Needs answer",$E36="Explain why",LEFT($E36,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B37:E37">
+    <cfRule type="expression" dxfId="326" priority="40">
+      <formula>$E37="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E37:E37">
+    <cfRule type="expression" dxfId="327" priority="41">
+      <formula>OR($E37="Needs answer",$E37="Explain why",LEFT($E37,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B38:E38">
+    <cfRule type="expression" dxfId="328" priority="42">
+      <formula>$E38="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E38:E38">
+    <cfRule type="expression" dxfId="329" priority="43">
+      <formula>OR($E38="Needs answer",$E38="Explain why",LEFT($E38,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B39:E39">
+    <cfRule type="expression" dxfId="330" priority="44">
+      <formula>$E39="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E39:E39">
+    <cfRule type="expression" dxfId="331" priority="45">
+      <formula>OR($E39="Needs answer",$E39="Explain why",LEFT($E39,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
     <dataValidation type="list" sqref="C6">
       <formula1>"LPS,TCon,Murphy's,Non-Conserved"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C10">
+    <dataValidation type="list" sqref="C25">
       <formula1>"Yes,No,Unable to assess"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C12">
+    <dataValidation type="list" sqref="C26">
       <formula1>"Yes,No,Unable to assess"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C16">
-      <formula1>"Yes,No,Unable to assess"</formula1>
-    </dataValidation>
-    <dataValidation type="whole" operator="between" sqref="C18">
-      <formula1>0</formula1>
-      <formula2>10000</formula2>
-    </dataValidation>
-    <dataValidation type="list" sqref="C19">
-      <formula1>"Yes,No,Unable to assess"</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="C20">
-      <formula1>"Yes,No,Unable to assess"</formula1>
-    </dataValidation>
-    <dataValidation type="list" sqref="C21">
+    <dataValidation type="list" sqref="C27">
       <formula1>"Yes,No,Unable to assess"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7079,82 +7188,82 @@
     <mergeCell ref="B3:E3"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:E6">
-    <cfRule type="expression" dxfId="327" priority="1">
+    <cfRule type="expression" dxfId="332" priority="1">
       <formula>$E6="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6:E6">
-    <cfRule type="expression" dxfId="328" priority="2">
+    <cfRule type="expression" dxfId="333" priority="2">
       <formula>OR($E6="Needs answer",$E6="Explain why",LEFT($E6,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:E7">
-    <cfRule type="expression" dxfId="329" priority="3">
+    <cfRule type="expression" dxfId="334" priority="3">
       <formula>$E7="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7:E7">
-    <cfRule type="expression" dxfId="330" priority="4">
+    <cfRule type="expression" dxfId="335" priority="4">
       <formula>OR($E7="Needs answer",$E7="Explain why",LEFT($E7,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:E8">
-    <cfRule type="expression" dxfId="331" priority="5">
+    <cfRule type="expression" dxfId="336" priority="5">
       <formula>$E8="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8:E8">
-    <cfRule type="expression" dxfId="332" priority="6">
+    <cfRule type="expression" dxfId="337" priority="6">
       <formula>OR($E8="Needs answer",$E8="Explain why",LEFT($E8,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:E9">
-    <cfRule type="expression" dxfId="333" priority="7">
+    <cfRule type="expression" dxfId="338" priority="7">
       <formula>$E9="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9:E9">
-    <cfRule type="expression" dxfId="334" priority="8">
+    <cfRule type="expression" dxfId="339" priority="8">
       <formula>OR($E9="Needs answer",$E9="Explain why",LEFT($E9,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:E10">
-    <cfRule type="expression" dxfId="335" priority="9">
+    <cfRule type="expression" dxfId="340" priority="9">
       <formula>$E10="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10:E10">
-    <cfRule type="expression" dxfId="336" priority="10">
+    <cfRule type="expression" dxfId="341" priority="10">
       <formula>OR($E10="Needs answer",$E10="Explain why",LEFT($E10,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:E11">
-    <cfRule type="expression" dxfId="337" priority="11">
+    <cfRule type="expression" dxfId="342" priority="11">
       <formula>$E11="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11:E11">
-    <cfRule type="expression" dxfId="338" priority="12">
+    <cfRule type="expression" dxfId="343" priority="12">
       <formula>OR($E11="Needs answer",$E11="Explain why",LEFT($E11,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:E12">
-    <cfRule type="expression" dxfId="339" priority="13">
+    <cfRule type="expression" dxfId="344" priority="13">
       <formula>$E12="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E12:E12">
-    <cfRule type="expression" dxfId="340" priority="14">
+    <cfRule type="expression" dxfId="345" priority="14">
       <formula>OR($E12="Needs answer",$E12="Explain why",LEFT($E12,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:E13">
-    <cfRule type="expression" dxfId="341" priority="15">
+    <cfRule type="expression" dxfId="346" priority="15">
       <formula>$E13="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:E13">
-    <cfRule type="expression" dxfId="342" priority="16">
+    <cfRule type="expression" dxfId="347" priority="16">
       <formula>OR($E13="Needs answer",$E13="Explain why",LEFT($E13,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7544,11 +7653,11 @@
         <v>7. Recent care and history</v>
       </c>
       <c r="C24" s="31" t="n">
-        <f>COUNTIF('07 Recent care and history'!E6:E11,"Needs answer")+COUNTIF('07 Recent care and history'!E6:E11,"Explain why")</f>
-        <v>1</v>
+        <f>COUNTIF('07 Recent care and history'!E6:E26,"Needs answer")+COUNTIF('07 Recent care and history'!E6:E26,"Explain why")</f>
+        <v>0</v>
       </c>
       <c r="D24" s="31" t="n">
-        <f>COUNTIF('07 Recent care and history'!E6:E11,"Review previous answer")+COUNTIF('07 Recent care and history'!E6:E11,"Review previous reason")</f>
+        <f>COUNTIF('07 Recent care and history'!E6:E26,"Review previous answer")+COUNTIF('07 Recent care and history'!E6:E26,"Review previous reason")</f>
         <v>0</v>
       </c>
       <c r="E24" s="30"/>
@@ -7589,11 +7698,11 @@
         <v>10. Decisions and legal support</v>
       </c>
       <c r="C27" s="31" t="n">
-        <f>COUNTIF('10 Decisions and legal support'!E6:E24,"Needs answer")+COUNTIF('10 Decisions and legal support'!E6:E24,"Explain why")</f>
-        <v>6</v>
+        <f>COUNTIF('10 Decisions and legal support'!E6:E39,"Needs answer")+COUNTIF('10 Decisions and legal support'!E6:E39,"Explain why")</f>
+        <v>4</v>
       </c>
       <c r="D27" s="31" t="n">
-        <f>COUNTIF('10 Decisions and legal support'!E6:E24,"Review previous answer")+COUNTIF('10 Decisions and legal support'!E6:E24,"Review previous reason")</f>
+        <f>COUNTIF('10 Decisions and legal support'!E6:E39,"Review previous answer")+COUNTIF('10 Decisions and legal support'!E6:E39,"Review previous reason")</f>
         <v>0</v>
       </c>
       <c r="E27" s="30"/>
@@ -7715,132 +7824,132 @@
     <mergeCell ref="B36:E36"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:E6">
-    <cfRule type="expression" dxfId="343" priority="1">
+    <cfRule type="expression" dxfId="348" priority="1">
       <formula>$E6="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6:E6">
-    <cfRule type="expression" dxfId="344" priority="2">
+    <cfRule type="expression" dxfId="349" priority="2">
       <formula>OR($E6="Needs answer",$E6="Explain why",LEFT($E6,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:E7">
-    <cfRule type="expression" dxfId="345" priority="3">
+    <cfRule type="expression" dxfId="350" priority="3">
       <formula>$E7="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7:E7">
-    <cfRule type="expression" dxfId="346" priority="4">
+    <cfRule type="expression" dxfId="351" priority="4">
       <formula>OR($E7="Needs answer",$E7="Explain why",LEFT($E7,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:E8">
-    <cfRule type="expression" dxfId="347" priority="5">
+    <cfRule type="expression" dxfId="352" priority="5">
       <formula>$E8="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8:E8">
-    <cfRule type="expression" dxfId="348" priority="6">
+    <cfRule type="expression" dxfId="353" priority="6">
       <formula>OR($E8="Needs answer",$E8="Explain why",LEFT($E8,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9:E9">
-    <cfRule type="expression" dxfId="349" priority="7">
+    <cfRule type="expression" dxfId="354" priority="7">
       <formula>$E9="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E9:E9">
-    <cfRule type="expression" dxfId="350" priority="8">
+    <cfRule type="expression" dxfId="355" priority="8">
       <formula>OR($E9="Needs answer",$E9="Explain why",LEFT($E9,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:E10">
-    <cfRule type="expression" dxfId="351" priority="9">
+    <cfRule type="expression" dxfId="356" priority="9">
       <formula>$E10="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E10:E10">
-    <cfRule type="expression" dxfId="352" priority="10">
+    <cfRule type="expression" dxfId="357" priority="10">
       <formula>OR($E10="Needs answer",$E10="Explain why",LEFT($E10,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:E11">
-    <cfRule type="expression" dxfId="353" priority="11">
+    <cfRule type="expression" dxfId="358" priority="11">
       <formula>$E11="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11:E11">
-    <cfRule type="expression" dxfId="354" priority="12">
+    <cfRule type="expression" dxfId="359" priority="12">
       <formula>OR($E11="Needs answer",$E11="Explain why",LEFT($E11,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:E13">
-    <cfRule type="expression" dxfId="355" priority="13">
+    <cfRule type="expression" dxfId="360" priority="13">
       <formula>$E13="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:E13">
-    <cfRule type="expression" dxfId="356" priority="14">
+    <cfRule type="expression" dxfId="361" priority="14">
       <formula>OR($E13="Needs answer",$E13="Explain why",LEFT($E13,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18:D18">
-    <cfRule type="cellIs" dxfId="369" priority="15" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="374" priority="15" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19:D19">
-    <cfRule type="cellIs" dxfId="370" priority="16" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="375" priority="16" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C20:D20">
-    <cfRule type="cellIs" dxfId="371" priority="17" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="376" priority="17" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C21:D21">
-    <cfRule type="cellIs" dxfId="372" priority="18" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="377" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C22:D22">
-    <cfRule type="cellIs" dxfId="373" priority="19" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="378" priority="19" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C23:D23">
-    <cfRule type="cellIs" dxfId="374" priority="20" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="379" priority="20" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C24:D24">
-    <cfRule type="cellIs" dxfId="375" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="380" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C25:D25">
-    <cfRule type="cellIs" dxfId="376" priority="22" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="381" priority="22" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C26:D26">
-    <cfRule type="cellIs" dxfId="377" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="382" priority="23" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C27:D27">
-    <cfRule type="cellIs" dxfId="378" priority="24" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="383" priority="24" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:D28">
-    <cfRule type="cellIs" dxfId="379" priority="25" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="384" priority="25" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C29:D29">
-    <cfRule type="cellIs" dxfId="380" priority="26" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="385" priority="26" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7880,7 +7989,7 @@
         <v>Questionnaire fingerprint</v>
       </c>
       <c r="B2" t="str">
-        <v>44ee09c0df7abcd44bc76e520cf2da27dbdbae70d31aef5d40cbd527d55bed9c</v>
+        <v>ceae1f99319c6b47c35e1e3822d9ec6d9ed0a082eb073f9b53612b111faaec6f</v>
       </c>
     </row>
     <row r="3">
@@ -9739,7 +9848,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>prior_hospitalizations_count</v>
+        <v>hospitalization_history</v>
       </c>
       <c r="B83" t="str">
         <v>07 Recent care and history!C8</v>
@@ -9763,7 +9872,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>most_recent_hospitalization</v>
+        <v>hospitalization_timeline</v>
       </c>
       <c r="B84" t="str">
         <v>07 Recent care and history!C9</v>
@@ -9787,10 +9896,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>prior_5150_5250_holds</v>
+        <v>prior_hospitalizations_count</v>
       </c>
       <c r="B85" t="str">
-        <v>07 Recent care and history!C10</v>
+        <v>07 Recent care and history!C23</v>
       </c>
       <c r="C85" t="str"/>
       <c r="D85" t="str"/>
@@ -9811,10 +9920,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>crisis_er_utilization</v>
+        <v>most_recent_hospitalization</v>
       </c>
       <c r="B86" t="str">
-        <v>07 Recent care and history!C11</v>
+        <v>07 Recent care and history!C24</v>
       </c>
       <c r="C86" t="str"/>
       <c r="D86" t="str"/>
@@ -9835,10 +9944,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>substance_abuse_history</v>
+        <v>prior_5150_5250_holds</v>
       </c>
       <c r="B87" t="str">
-        <v>08 Substance use and recovery!C6</v>
+        <v>07 Recent care and history!C25</v>
       </c>
       <c r="C87" t="str"/>
       <c r="D87" t="str"/>
@@ -9859,10 +9968,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>active_substance_use</v>
+        <v>crisis_er_utilization</v>
       </c>
       <c r="B88" t="str">
-        <v>08 Substance use and recovery!C7</v>
+        <v>07 Recent care and history!C26</v>
       </c>
       <c r="C88" t="str"/>
       <c r="D88" t="str"/>
@@ -9883,10 +9992,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>substances</v>
+        <v>substance_abuse_history</v>
       </c>
       <c r="B89" t="str">
-        <v>08 Substance use and recovery!C8</v>
+        <v>08 Substance use and recovery!C6</v>
       </c>
       <c r="C89" t="str"/>
       <c r="D89" t="str"/>
@@ -9907,10 +10016,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>last_substance_use_date</v>
+        <v>active_substance_use</v>
       </c>
       <c r="B90" t="str">
-        <v>08 Substance use and recovery!C22</v>
+        <v>08 Substance use and recovery!C7</v>
       </c>
       <c r="C90" t="str"/>
       <c r="D90" t="str"/>
@@ -9931,10 +10040,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>use_pattern</v>
+        <v>substances</v>
       </c>
       <c r="B91" t="str">
-        <v>08 Substance use and recovery!C23</v>
+        <v>08 Substance use and recovery!C8</v>
       </c>
       <c r="C91" t="str"/>
       <c r="D91" t="str"/>
@@ -9955,10 +10064,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>substance_effect_on_baseline</v>
+        <v>last_substance_use_date</v>
       </c>
       <c r="B92" t="str">
-        <v>08 Substance use and recovery!C24</v>
+        <v>08 Substance use and recovery!C22</v>
       </c>
       <c r="C92" t="str"/>
       <c r="D92" t="str"/>
@@ -9979,10 +10088,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>longest_sobriety_period</v>
+        <v>use_pattern</v>
       </c>
       <c r="B93" t="str">
-        <v>08 Substance use and recovery!C25</v>
+        <v>08 Substance use and recovery!C23</v>
       </c>
       <c r="C93" t="str"/>
       <c r="D93" t="str"/>
@@ -10003,10 +10112,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>substance_use_insight</v>
+        <v>substance_effect_on_baseline</v>
       </c>
       <c r="B94" t="str">
-        <v>08 Substance use and recovery!C26</v>
+        <v>08 Substance use and recovery!C24</v>
       </c>
       <c r="C94" t="str"/>
       <c r="D94" t="str"/>
@@ -10027,10 +10136,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>substance_use_insight_details</v>
+        <v>longest_sobriety_period</v>
       </c>
       <c r="B95" t="str">
-        <v>08 Substance use and recovery!C27</v>
+        <v>08 Substance use and recovery!C25</v>
       </c>
       <c r="C95" t="str"/>
       <c r="D95" t="str"/>
@@ -10051,10 +10160,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>treatment_history</v>
+        <v>substance_use_insight</v>
       </c>
       <c r="B96" t="str">
-        <v>08 Substance use and recovery!C28</v>
+        <v>08 Substance use and recovery!C26</v>
       </c>
       <c r="C96" t="str"/>
       <c r="D96" t="str"/>
@@ -10075,10 +10184,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>longest_sobriety_months</v>
+        <v>substance_use_insight_details</v>
       </c>
       <c r="B97" t="str">
-        <v>08 Substance use and recovery!C29</v>
+        <v>08 Substance use and recovery!C27</v>
       </c>
       <c r="C97" t="str"/>
       <c r="D97" t="str"/>
@@ -10099,10 +10208,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>behavioral_history</v>
+        <v>treatment_history</v>
       </c>
       <c r="B98" t="str">
-        <v>09 Safety and support!C6</v>
+        <v>08 Substance use and recovery!C28</v>
       </c>
       <c r="C98" t="str"/>
       <c r="D98" t="str"/>
@@ -10123,10 +10232,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>physical_altercations</v>
+        <v>longest_sobriety_months</v>
       </c>
       <c r="B99" t="str">
-        <v>09 Safety and support!C7</v>
+        <v>08 Substance use and recovery!C29</v>
       </c>
       <c r="C99" t="str"/>
       <c r="D99" t="str"/>
@@ -10147,10 +10256,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>physical_altercation_details</v>
+        <v>behavioral_history</v>
       </c>
       <c r="B100" t="str">
-        <v>09 Safety and support!C8</v>
+        <v>09 Safety and support!C6</v>
       </c>
       <c r="C100" t="str"/>
       <c r="D100" t="str"/>
@@ -10171,10 +10280,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>self_harm_history</v>
+        <v>physical_altercations</v>
       </c>
       <c r="B101" t="str">
-        <v>09 Safety and support!C9</v>
+        <v>09 Safety and support!C7</v>
       </c>
       <c r="C101" t="str"/>
       <c r="D101" t="str"/>
@@ -10195,10 +10304,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>last_self_harm_incident</v>
+        <v>physical_altercation_details</v>
       </c>
       <c r="B102" t="str">
-        <v>09 Safety and support!C10</v>
+        <v>09 Safety and support!C8</v>
       </c>
       <c r="C102" t="str"/>
       <c r="D102" t="str"/>
@@ -10219,10 +10328,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>current_self_harm_ideation</v>
+        <v>self_harm_history</v>
       </c>
       <c r="B103" t="str">
-        <v>09 Safety and support!C11</v>
+        <v>09 Safety and support!C9</v>
       </c>
       <c r="C103" t="str"/>
       <c r="D103" t="str"/>
@@ -10243,10 +10352,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>current_self_harm_details</v>
+        <v>last_self_harm_incident</v>
       </c>
       <c r="B104" t="str">
-        <v>09 Safety and support!C12</v>
+        <v>09 Safety and support!C10</v>
       </c>
       <c r="C104" t="str"/>
       <c r="D104" t="str"/>
@@ -10267,10 +10376,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>current_safety_measures</v>
+        <v>current_self_harm_ideation</v>
       </c>
       <c r="B105" t="str">
-        <v>09 Safety and support!C13</v>
+        <v>09 Safety and support!C11</v>
       </c>
       <c r="C105" t="str"/>
       <c r="D105" t="str"/>
@@ -10291,10 +10400,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>assault_history</v>
+        <v>current_self_harm_details</v>
       </c>
       <c r="B106" t="str">
-        <v>09 Safety and support!C14</v>
+        <v>09 Safety and support!C12</v>
       </c>
       <c r="C106" t="str"/>
       <c r="D106" t="str"/>
@@ -10315,10 +10424,10 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>last_assault_details</v>
+        <v>current_safety_measures</v>
       </c>
       <c r="B107" t="str">
-        <v>09 Safety and support!C15</v>
+        <v>09 Safety and support!C13</v>
       </c>
       <c r="C107" t="str"/>
       <c r="D107" t="str"/>
@@ -10339,10 +10448,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>assaults_last_two_years_count</v>
+        <v>assault_history</v>
       </c>
       <c r="B108" t="str">
-        <v>09 Safety and support!C16</v>
+        <v>09 Safety and support!C14</v>
       </c>
       <c r="C108" t="str"/>
       <c r="D108" t="str"/>
@@ -10363,10 +10472,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>elopement_history</v>
+        <v>last_assault_details</v>
       </c>
       <c r="B109" t="str">
-        <v>09 Safety and support!C17</v>
+        <v>09 Safety and support!C15</v>
       </c>
       <c r="C109" t="str"/>
       <c r="D109" t="str"/>
@@ -10387,10 +10496,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>elopement_risk</v>
+        <v>assaults_last_two_years_count</v>
       </c>
       <c r="B110" t="str">
-        <v>09 Safety and support!C18</v>
+        <v>09 Safety and support!C16</v>
       </c>
       <c r="C110" t="str"/>
       <c r="D110" t="str"/>
@@ -10411,10 +10520,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>si_hi_history</v>
+        <v>elopement_history</v>
       </c>
       <c r="B111" t="str">
-        <v>09 Safety and support!C19</v>
+        <v>09 Safety and support!C17</v>
       </c>
       <c r="C111" t="str"/>
       <c r="D111" t="str"/>
@@ -10435,10 +10544,10 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>triggers</v>
+        <v>elopement_risk</v>
       </c>
       <c r="B112" t="str">
-        <v>09 Safety and support!C20</v>
+        <v>09 Safety and support!C18</v>
       </c>
       <c r="C112" t="str"/>
       <c r="D112" t="str"/>
@@ -10459,10 +10568,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>aggression_risk</v>
+        <v>si_hi_history</v>
       </c>
       <c r="B113" t="str">
-        <v>09 Safety and support!C21</v>
+        <v>09 Safety and support!C19</v>
       </c>
       <c r="C113" t="str"/>
       <c r="D113" t="str"/>
@@ -10483,10 +10592,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>responds_to_internal_stimuli</v>
+        <v>triggers</v>
       </c>
       <c r="B114" t="str">
-        <v>09 Safety and support!C22</v>
+        <v>09 Safety and support!C20</v>
       </c>
       <c r="C114" t="str"/>
       <c r="D114" t="str"/>
@@ -10507,10 +10616,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>auditory_hallucinations</v>
+        <v>aggression_risk</v>
       </c>
       <c r="B115" t="str">
-        <v>09 Safety and support!C23</v>
+        <v>09 Safety and support!C21</v>
       </c>
       <c r="C115" t="str"/>
       <c r="D115" t="str"/>
@@ -10531,10 +10640,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>auditory_hallucination_nature</v>
+        <v>responds_to_internal_stimuli</v>
       </c>
       <c r="B116" t="str">
-        <v>09 Safety and support!C24</v>
+        <v>09 Safety and support!C22</v>
       </c>
       <c r="C116" t="str"/>
       <c r="D116" t="str"/>
@@ -10555,10 +10664,10 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>auditory_hallucination_frequency</v>
+        <v>auditory_hallucinations</v>
       </c>
       <c r="B117" t="str">
-        <v>09 Safety and support!C25</v>
+        <v>09 Safety and support!C23</v>
       </c>
       <c r="C117" t="str"/>
       <c r="D117" t="str"/>
@@ -10579,10 +10688,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>auditory_hallucination_triggers</v>
+        <v>auditory_hallucination_nature</v>
       </c>
       <c r="B118" t="str">
-        <v>09 Safety and support!C26</v>
+        <v>09 Safety and support!C24</v>
       </c>
       <c r="C118" t="str"/>
       <c r="D118" t="str"/>
@@ -10603,10 +10712,10 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>visual_hallucinations</v>
+        <v>auditory_hallucination_frequency</v>
       </c>
       <c r="B119" t="str">
-        <v>09 Safety and support!C27</v>
+        <v>09 Safety and support!C25</v>
       </c>
       <c r="C119" t="str"/>
       <c r="D119" t="str"/>
@@ -10627,10 +10736,10 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>visual_hallucination_details</v>
+        <v>auditory_hallucination_triggers</v>
       </c>
       <c r="B120" t="str">
-        <v>09 Safety and support!C28</v>
+        <v>09 Safety and support!C26</v>
       </c>
       <c r="C120" t="str"/>
       <c r="D120" t="str"/>
@@ -10651,10 +10760,10 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>visual_hallucination_recent</v>
+        <v>visual_hallucinations</v>
       </c>
       <c r="B121" t="str">
-        <v>09 Safety and support!C29</v>
+        <v>09 Safety and support!C27</v>
       </c>
       <c r="C121" t="str"/>
       <c r="D121" t="str"/>
@@ -10675,10 +10784,10 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>olfactory_hallucinations</v>
+        <v>visual_hallucination_details</v>
       </c>
       <c r="B122" t="str">
-        <v>09 Safety and support!C30</v>
+        <v>09 Safety and support!C28</v>
       </c>
       <c r="C122" t="str"/>
       <c r="D122" t="str"/>
@@ -10699,10 +10808,10 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>olfactory_hallucination_details</v>
+        <v>visual_hallucination_recent</v>
       </c>
       <c r="B123" t="str">
-        <v>09 Safety and support!C31</v>
+        <v>09 Safety and support!C29</v>
       </c>
       <c r="C123" t="str"/>
       <c r="D123" t="str"/>
@@ -10723,10 +10832,10 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>olfactory_hallucination_impact</v>
+        <v>olfactory_hallucinations</v>
       </c>
       <c r="B124" t="str">
-        <v>09 Safety and support!C32</v>
+        <v>09 Safety and support!C30</v>
       </c>
       <c r="C124" t="str"/>
       <c r="D124" t="str"/>
@@ -10747,10 +10856,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>tactile_hallucinations</v>
+        <v>olfactory_hallucination_details</v>
       </c>
       <c r="B125" t="str">
-        <v>09 Safety and support!C33</v>
+        <v>09 Safety and support!C31</v>
       </c>
       <c r="C125" t="str"/>
       <c r="D125" t="str"/>
@@ -10771,10 +10880,10 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>tactile_hallucination_details</v>
+        <v>olfactory_hallucination_impact</v>
       </c>
       <c r="B126" t="str">
-        <v>09 Safety and support!C34</v>
+        <v>09 Safety and support!C32</v>
       </c>
       <c r="C126" t="str"/>
       <c r="D126" t="str"/>
@@ -10795,10 +10904,10 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>tactile_hallucination_frequency</v>
+        <v>tactile_hallucinations</v>
       </c>
       <c r="B127" t="str">
-        <v>09 Safety and support!C35</v>
+        <v>09 Safety and support!C33</v>
       </c>
       <c r="C127" t="str"/>
       <c r="D127" t="str"/>
@@ -10819,10 +10928,10 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>gustatory_hallucinations</v>
+        <v>tactile_hallucination_details</v>
       </c>
       <c r="B128" t="str">
-        <v>09 Safety and support!C36</v>
+        <v>09 Safety and support!C34</v>
       </c>
       <c r="C128" t="str"/>
       <c r="D128" t="str"/>
@@ -10843,10 +10952,10 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>gustatory_hallucination_details</v>
+        <v>tactile_hallucination_frequency</v>
       </c>
       <c r="B129" t="str">
-        <v>09 Safety and support!C37</v>
+        <v>09 Safety and support!C35</v>
       </c>
       <c r="C129" t="str"/>
       <c r="D129" t="str"/>
@@ -10867,10 +10976,10 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>hallucination_coping_strategies</v>
+        <v>gustatory_hallucinations</v>
       </c>
       <c r="B130" t="str">
-        <v>09 Safety and support!C38</v>
+        <v>09 Safety and support!C36</v>
       </c>
       <c r="C130" t="str"/>
       <c r="D130" t="str"/>
@@ -10891,10 +11000,10 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>hallucination_distress_impairment</v>
+        <v>gustatory_hallucination_details</v>
       </c>
       <c r="B131" t="str">
-        <v>09 Safety and support!C39</v>
+        <v>09 Safety and support!C37</v>
       </c>
       <c r="C131" t="str"/>
       <c r="D131" t="str"/>
@@ -10915,10 +11024,10 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>hallucination_functional_impact</v>
+        <v>hallucination_coping_strategies</v>
       </c>
       <c r="B132" t="str">
-        <v>09 Safety and support!C40</v>
+        <v>09 Safety and support!C38</v>
       </c>
       <c r="C132" t="str"/>
       <c r="D132" t="str"/>
@@ -10939,10 +11048,10 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>hallucination_treatment_history</v>
+        <v>hallucination_distress_impairment</v>
       </c>
       <c r="B133" t="str">
-        <v>09 Safety and support!C41</v>
+        <v>09 Safety and support!C39</v>
       </c>
       <c r="C133" t="str"/>
       <c r="D133" t="str"/>
@@ -10963,10 +11072,10 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>conservatorship_type</v>
+        <v>hallucination_functional_impact</v>
       </c>
       <c r="B134" t="str">
-        <v>10 Decisions and legal support!C6</v>
+        <v>09 Safety and support!C40</v>
       </c>
       <c r="C134" t="str"/>
       <c r="D134" t="str"/>
@@ -10987,10 +11096,10 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>conservator_name</v>
+        <v>hallucination_treatment_history</v>
       </c>
       <c r="B135" t="str">
-        <v>10 Decisions and legal support!C7</v>
+        <v>09 Safety and support!C41</v>
       </c>
       <c r="C135" t="str"/>
       <c r="D135" t="str"/>
@@ -11011,10 +11120,10 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>conservatorship_status</v>
+        <v>conservatorship_type</v>
       </c>
       <c r="B136" t="str">
-        <v>10 Decisions and legal support!C8</v>
+        <v>10 Decisions and legal support!C6</v>
       </c>
       <c r="C136" t="str"/>
       <c r="D136" t="str"/>
@@ -11035,10 +11144,10 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>hold_type</v>
+        <v>conservator_name</v>
       </c>
       <c r="B137" t="str">
-        <v>10 Decisions and legal support!C9</v>
+        <v>10 Decisions and legal support!C7</v>
       </c>
       <c r="C137" t="str"/>
       <c r="D137" t="str"/>
@@ -11059,10 +11168,10 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>forensic_involvement</v>
+        <v>conservatorship_status</v>
       </c>
       <c r="B138" t="str">
-        <v>10 Decisions and legal support!C10</v>
+        <v>10 Decisions and legal support!C8</v>
       </c>
       <c r="C138" t="str"/>
       <c r="D138" t="str"/>
@@ -11083,10 +11192,10 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>forensic_involvement_details</v>
+        <v>hold_type</v>
       </c>
       <c r="B139" t="str">
-        <v>10 Decisions and legal support!C11</v>
+        <v>10 Decisions and legal support!C9</v>
       </c>
       <c r="C139" t="str"/>
       <c r="D139" t="str"/>
@@ -11107,10 +11216,10 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>arrest_history</v>
+        <v>forensic_history</v>
       </c>
       <c r="B140" t="str">
-        <v>10 Decisions and legal support!C12</v>
+        <v>10 Decisions and legal support!C10</v>
       </c>
       <c r="C140" t="str"/>
       <c r="D140" t="str"/>
@@ -11131,10 +11240,10 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>most_recent_arrest_date</v>
+        <v>forensic_timeline</v>
       </c>
       <c r="B141" t="str">
-        <v>10 Decisions and legal support!C13</v>
+        <v>10 Decisions and legal support!C11</v>
       </c>
       <c r="C141" t="str"/>
       <c r="D141" t="str"/>
@@ -11155,10 +11264,10 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>most_recent_arrest_charge</v>
+        <v>pc290_registration</v>
       </c>
       <c r="B142" t="str">
-        <v>10 Decisions and legal support!C14</v>
+        <v>10 Decisions and legal support!C25</v>
       </c>
       <c r="C142" t="str"/>
       <c r="D142" t="str"/>
@@ -11179,10 +11288,10 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>most_recent_arrest_jail_time</v>
+        <v>arson_history</v>
       </c>
       <c r="B143" t="str">
-        <v>10 Decisions and legal support!C15</v>
+        <v>10 Decisions and legal support!C26</v>
       </c>
       <c r="C143" t="str"/>
       <c r="D143" t="str"/>
@@ -11203,10 +11312,10 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>arrest_in_last_two_years</v>
+        <v>diversion_client</v>
       </c>
       <c r="B144" t="str">
-        <v>10 Decisions and legal support!C16</v>
+        <v>10 Decisions and legal support!C27</v>
       </c>
       <c r="C144" t="str"/>
       <c r="D144" t="str"/>
@@ -11227,10 +11336,10 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>arrest_last_two_years_details</v>
+        <v>court_requirements</v>
       </c>
       <c r="B145" t="str">
-        <v>10 Decisions and legal support!C17</v>
+        <v>10 Decisions and legal support!C28</v>
       </c>
       <c r="C145" t="str"/>
       <c r="D145" t="str"/>
@@ -11251,10 +11360,10 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>total_arrests</v>
+        <v>court_dates</v>
       </c>
       <c r="B146" t="str">
-        <v>10 Decisions and legal support!C18</v>
+        <v>10 Decisions and legal support!C29</v>
       </c>
       <c r="C146" t="str"/>
       <c r="D146" t="str"/>
@@ -11275,10 +11384,10 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>pc290_registration</v>
+        <v>probation_parole_justice</v>
       </c>
       <c r="B147" t="str">
-        <v>10 Decisions and legal support!C19</v>
+        <v>10 Decisions and legal support!C30</v>
       </c>
       <c r="C147" t="str"/>
       <c r="D147" t="str"/>
@@ -11299,10 +11408,10 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>arson_history</v>
+        <v>forensic_involvement</v>
       </c>
       <c r="B148" t="str">
-        <v>10 Decisions and legal support!C20</v>
+        <v>10 Decisions and legal support!C31</v>
       </c>
       <c r="C148" t="str"/>
       <c r="D148" t="str"/>
@@ -11323,10 +11432,10 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>diversion_client</v>
+        <v>forensic_involvement_details</v>
       </c>
       <c r="B149" t="str">
-        <v>10 Decisions and legal support!C21</v>
+        <v>10 Decisions and legal support!C32</v>
       </c>
       <c r="C149" t="str"/>
       <c r="D149" t="str"/>
@@ -11347,10 +11456,10 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>court_requirements</v>
+        <v>arrest_history</v>
       </c>
       <c r="B150" t="str">
-        <v>10 Decisions and legal support!C22</v>
+        <v>10 Decisions and legal support!C33</v>
       </c>
       <c r="C150" t="str"/>
       <c r="D150" t="str"/>
@@ -11371,10 +11480,10 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>court_dates</v>
+        <v>most_recent_arrest_date</v>
       </c>
       <c r="B151" t="str">
-        <v>10 Decisions and legal support!C23</v>
+        <v>10 Decisions and legal support!C34</v>
       </c>
       <c r="C151" t="str"/>
       <c r="D151" t="str"/>
@@ -11395,10 +11504,10 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>probation_parole_justice</v>
+        <v>most_recent_arrest_charge</v>
       </c>
       <c r="B152" t="str">
-        <v>10 Decisions and legal support!C24</v>
+        <v>10 Decisions and legal support!C35</v>
       </c>
       <c r="C152" t="str"/>
       <c r="D152" t="str"/>
@@ -11419,10 +11528,10 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>family_involvement</v>
+        <v>most_recent_arrest_jail_time</v>
       </c>
       <c r="B153" t="str">
-        <v>11 What matters next!C6</v>
+        <v>10 Decisions and legal support!C36</v>
       </c>
       <c r="C153" t="str"/>
       <c r="D153" t="str"/>
@@ -11443,10 +11552,10 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>friendships_social_connections</v>
+        <v>arrest_in_last_two_years</v>
       </c>
       <c r="B154" t="str">
-        <v>11 What matters next!C7</v>
+        <v>10 Decisions and legal support!C37</v>
       </c>
       <c r="C154" t="str"/>
       <c r="D154" t="str"/>
@@ -11467,10 +11576,10 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>prior_living_situation</v>
+        <v>arrest_last_two_years_details</v>
       </c>
       <c r="B155" t="str">
-        <v>11 What matters next!C8</v>
+        <v>10 Decisions and legal support!C38</v>
       </c>
       <c r="C155" t="str"/>
       <c r="D155" t="str"/>
@@ -11491,10 +11600,10 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>housing_history</v>
+        <v>total_arrests</v>
       </c>
       <c r="B156" t="str">
-        <v>11 What matters next!C9</v>
+        <v>10 Decisions and legal support!C39</v>
       </c>
       <c r="C156" t="str"/>
       <c r="D156" t="str"/>
@@ -11515,10 +11624,10 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>benefits_income_status</v>
+        <v>family_involvement</v>
       </c>
       <c r="B157" t="str">
-        <v>11 What matters next!C10</v>
+        <v>11 What matters next!C6</v>
       </c>
       <c r="C157" t="str"/>
       <c r="D157" t="str"/>
@@ -11539,10 +11648,10 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>preferred_facility_characteristics</v>
+        <v>friendships_social_connections</v>
       </c>
       <c r="B158" t="str">
-        <v>11 What matters next!C11</v>
+        <v>11 What matters next!C7</v>
       </c>
       <c r="C158" t="str"/>
       <c r="D158" t="str"/>
@@ -11563,10 +11672,10 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>discharge_planning_goals</v>
+        <v>prior_living_situation</v>
       </c>
       <c r="B159" t="str">
-        <v>11 What matters next!C12</v>
+        <v>11 What matters next!C8</v>
       </c>
       <c r="C159" t="str"/>
       <c r="D159" t="str"/>
@@ -11587,10 +11696,10 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>placement_preferences_concerns</v>
+        <v>housing_history</v>
       </c>
       <c r="B160" t="str">
-        <v>11 What matters next!C13</v>
+        <v>11 What matters next!C9</v>
       </c>
       <c r="C160" t="str"/>
       <c r="D160" t="str"/>
@@ -11611,10 +11720,10 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>additional_information</v>
+        <v>benefits_income_status</v>
       </c>
       <c r="B161" t="str">
-        <v>12 Anything else!C6</v>
+        <v>11 What matters next!C10</v>
       </c>
       <c r="C161" t="str"/>
       <c r="D161" t="str"/>
@@ -11635,10 +11744,10 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>placement_process_questions</v>
+        <v>preferred_facility_characteristics</v>
       </c>
       <c r="B162" t="str">
-        <v>12 Anything else!C7</v>
+        <v>11 What matters next!C11</v>
       </c>
       <c r="C162" t="str"/>
       <c r="D162" t="str"/>
@@ -11659,10 +11768,10 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>unable_to_assess_reasons</v>
+        <v>discharge_planning_goals</v>
       </c>
       <c r="B163" t="str">
-        <v>12 Anything else!C8</v>
+        <v>11 What matters next!C12</v>
       </c>
       <c r="C163" t="str"/>
       <c r="D163" t="str"/>
@@ -11683,10 +11792,10 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>source_file</v>
+        <v>placement_preferences_concerns</v>
       </c>
       <c r="B164" t="str">
-        <v>12 Anything else!C9</v>
+        <v>11 What matters next!C13</v>
       </c>
       <c r="C164" t="str"/>
       <c r="D164" t="str"/>
@@ -11707,10 +11816,10 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>match_confidence</v>
+        <v>additional_information</v>
       </c>
       <c r="B165" t="str">
-        <v>12 Anything else!C10</v>
+        <v>12 Anything else!C6</v>
       </c>
       <c r="C165" t="str"/>
       <c r="D165" t="str"/>
@@ -11731,10 +11840,10 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>assessment_notes</v>
+        <v>placement_process_questions</v>
       </c>
       <c r="B166" t="str">
-        <v>12 Anything else!C11</v>
+        <v>12 Anything else!C7</v>
       </c>
       <c r="C166" t="str"/>
       <c r="D166" t="str"/>
@@ -11755,10 +11864,10 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>extraction_date</v>
+        <v>unable_to_assess_reasons</v>
       </c>
       <c r="B167" t="str">
-        <v>12 Anything else!C13</v>
+        <v>12 Anything else!C8</v>
       </c>
       <c r="C167" t="str"/>
       <c r="D167" t="str"/>
@@ -11776,6 +11885,102 @@
       <c r="P167" t="str"/>
       <c r="Q167" t="str"/>
       <c r="R167" t="str"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>source_file</v>
+      </c>
+      <c r="B168" t="str">
+        <v>12 Anything else!C9</v>
+      </c>
+      <c r="C168" t="str"/>
+      <c r="D168" t="str"/>
+      <c r="E168" t="str"/>
+      <c r="F168" t="str"/>
+      <c r="G168" t="str"/>
+      <c r="H168" t="str"/>
+      <c r="I168" t="str"/>
+      <c r="J168" t="str"/>
+      <c r="K168" t="str"/>
+      <c r="L168" t="str"/>
+      <c r="M168" t="str"/>
+      <c r="N168" t="str"/>
+      <c r="O168" t="str"/>
+      <c r="P168" t="str"/>
+      <c r="Q168" t="str"/>
+      <c r="R168" t="str"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>match_confidence</v>
+      </c>
+      <c r="B169" t="str">
+        <v>12 Anything else!C10</v>
+      </c>
+      <c r="C169" t="str"/>
+      <c r="D169" t="str"/>
+      <c r="E169" t="str"/>
+      <c r="F169" t="str"/>
+      <c r="G169" t="str"/>
+      <c r="H169" t="str"/>
+      <c r="I169" t="str"/>
+      <c r="J169" t="str"/>
+      <c r="K169" t="str"/>
+      <c r="L169" t="str"/>
+      <c r="M169" t="str"/>
+      <c r="N169" t="str"/>
+      <c r="O169" t="str"/>
+      <c r="P169" t="str"/>
+      <c r="Q169" t="str"/>
+      <c r="R169" t="str"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>assessment_notes</v>
+      </c>
+      <c r="B170" t="str">
+        <v>12 Anything else!C11</v>
+      </c>
+      <c r="C170" t="str"/>
+      <c r="D170" t="str"/>
+      <c r="E170" t="str"/>
+      <c r="F170" t="str"/>
+      <c r="G170" t="str"/>
+      <c r="H170" t="str"/>
+      <c r="I170" t="str"/>
+      <c r="J170" t="str"/>
+      <c r="K170" t="str"/>
+      <c r="L170" t="str"/>
+      <c r="M170" t="str"/>
+      <c r="N170" t="str"/>
+      <c r="O170" t="str"/>
+      <c r="P170" t="str"/>
+      <c r="Q170" t="str"/>
+      <c r="R170" t="str"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>extraction_date</v>
+      </c>
+      <c r="B171" t="str">
+        <v>12 Anything else!C13</v>
+      </c>
+      <c r="C171" t="str"/>
+      <c r="D171" t="str"/>
+      <c r="E171" t="str"/>
+      <c r="F171" t="str"/>
+      <c r="G171" t="str"/>
+      <c r="H171" t="str"/>
+      <c r="I171" t="str"/>
+      <c r="J171" t="str"/>
+      <c r="K171" t="str"/>
+      <c r="L171" t="str"/>
+      <c r="M171" t="str"/>
+      <c r="N171" t="str"/>
+      <c r="O171" t="str"/>
+      <c r="P171" t="str"/>
+      <c r="Q171" t="str"/>
+      <c r="R171" t="str"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12810,10 +13015,10 @@
     <row r="80" ht="34" customHeight="1">
       <c r="A80" s="3"/>
       <c r="B80" s="29" t="str">
-        <v>Prior hospitalizations</v>
+        <v>Hospitalization history</v>
       </c>
       <c r="C80" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D80" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -12823,10 +13028,10 @@
     <row r="81" ht="34" customHeight="1">
       <c r="A81" s="3"/>
       <c r="B81" s="29" t="str">
-        <v>Most recent hospitalization</v>
+        <v>Hospitalization timeline</v>
       </c>
       <c r="C81" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>One item per line</v>
       </c>
       <c r="D81" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -12836,10 +13041,10 @@
     <row r="82" ht="34" customHeight="1">
       <c r="A82" s="3"/>
       <c r="B82" s="29" t="str">
-        <v>Prior 5150 / 5250 holds</v>
+        <v>Prior hospitalizations</v>
       </c>
       <c r="C82" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D82" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -12849,10 +13054,10 @@
     <row r="83" ht="34" customHeight="1">
       <c r="A83" s="3"/>
       <c r="B83" s="29" t="str">
-        <v>Crisis / ER utilization</v>
+        <v>Most recent hospitalization</v>
       </c>
       <c r="C83" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D83" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -12862,36 +13067,36 @@
     <row r="84" ht="34" customHeight="1">
       <c r="A84" s="3"/>
       <c r="B84" s="29" t="str">
-        <v>History of substance abuse</v>
+        <v>Prior 5150 / 5250 holds</v>
       </c>
       <c r="C84" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D84" s="29" t="str">
-        <v>08 Substance use and recovery</v>
+        <v>07 Recent care and history</v>
       </c>
       <c r="E84" s="3"/>
     </row>
     <row r="85" ht="34" customHeight="1">
       <c r="A85" s="3"/>
       <c r="B85" s="29" t="str">
-        <v>Active substance use</v>
+        <v>Crisis / ER utilization</v>
       </c>
       <c r="C85" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D85" s="29" t="str">
-        <v>08 Substance use and recovery</v>
+        <v>07 Recent care and history</v>
       </c>
       <c r="E85" s="3"/>
     </row>
     <row r="86" ht="34" customHeight="1">
       <c r="A86" s="3"/>
       <c r="B86" s="29" t="str">
-        <v>Substances</v>
+        <v>History of substance abuse</v>
       </c>
       <c r="C86" s="29" t="str">
-        <v>Opioids; Amphetamines; Marijuana; Alcohol; Other</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D86" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12901,10 +13106,10 @@
     <row r="87" ht="34" customHeight="1">
       <c r="A87" s="3"/>
       <c r="B87" s="29" t="str">
-        <v>Last substance use</v>
+        <v>Active substance use</v>
       </c>
       <c r="C87" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D87" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12914,10 +13119,10 @@
     <row r="88" ht="34" customHeight="1">
       <c r="A88" s="3"/>
       <c r="B88" s="29" t="str">
-        <v>Use pattern</v>
+        <v>Substances</v>
       </c>
       <c r="C88" s="29" t="str">
-        <v>Daily; Weekly; Sporadic; Rarely</v>
+        <v>Opioids; Amphetamines; Marijuana; Alcohol; Other</v>
       </c>
       <c r="D88" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12927,62 +13132,62 @@
     <row r="89" ht="34" customHeight="1">
       <c r="A89" s="3"/>
       <c r="B89" s="29" t="str">
-        <v>Effect on baseline behavior</v>
+        <v>Last substance use</v>
       </c>
       <c r="C89" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D89" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" ht="60" customHeight="1">
+    <row r="90" ht="34" customHeight="1">
       <c r="A90" s="3"/>
       <c r="B90" s="29" t="str">
-        <v>Longest sobriety in the last five years</v>
+        <v>Use pattern</v>
       </c>
       <c r="C90" s="29" t="str">
-        <v>1 month; 2 months; 3 months; 4 months; 5 months; 6 months; 7 months; 8 months; 9 months; 10 months; 11 months; 1 year; 18 months; 2 years; More than 2 years</v>
+        <v>Daily; Weekly; Sporadic; Rarely</v>
       </c>
       <c r="D90" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" ht="44" customHeight="1">
+    <row r="91" ht="34" customHeight="1">
       <c r="A91" s="3"/>
       <c r="B91" s="29" t="str">
-        <v>Acknowledgment of substance-use impact</v>
+        <v>Effect on baseline behavior</v>
       </c>
       <c r="C91" s="29" t="str">
-        <v>Acknowledges impact; Partially acknowledges impact; Does not acknowledge impact; Not discussed</v>
+        <v>Text or notes</v>
       </c>
       <c r="D91" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" ht="34" customHeight="1">
+    <row r="92" ht="60" customHeight="1">
       <c r="A92" s="3"/>
       <c r="B92" s="29" t="str">
-        <v>Substance-use impact notes</v>
+        <v>Longest sobriety in the last five years</v>
       </c>
       <c r="C92" s="29" t="str">
-        <v>Text or notes</v>
+        <v>1 month; 2 months; 3 months; 4 months; 5 months; 6 months; 7 months; 8 months; 9 months; 10 months; 11 months; 1 year; 18 months; 2 years; More than 2 years</v>
       </c>
       <c r="D92" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E92" s="3"/>
     </row>
-    <row r="93" ht="34" customHeight="1">
+    <row r="93" ht="44" customHeight="1">
       <c r="A93" s="3"/>
       <c r="B93" s="29" t="str">
-        <v>Treatment history</v>
+        <v>Acknowledgment of substance-use impact</v>
       </c>
       <c r="C93" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Acknowledges impact; Partially acknowledges impact; Does not acknowledge impact; Not discussed</v>
       </c>
       <c r="D93" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -12992,10 +13197,10 @@
     <row r="94" ht="34" customHeight="1">
       <c r="A94" s="3"/>
       <c r="B94" s="29" t="str">
-        <v>Longest sobriety in the last five years</v>
+        <v>Substance-use impact notes</v>
       </c>
       <c r="C94" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D94" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13005,33 +13210,33 @@
     <row r="95" ht="34" customHeight="1">
       <c r="A95" s="3"/>
       <c r="B95" s="29" t="str">
-        <v>Behavioral history</v>
+        <v>Treatment history</v>
       </c>
       <c r="C95" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D95" s="29" t="str">
-        <v>09 Safety and support</v>
+        <v>08 Substance use and recovery</v>
       </c>
       <c r="E95" s="3"/>
     </row>
     <row r="96" ht="34" customHeight="1">
       <c r="A96" s="3"/>
       <c r="B96" s="29" t="str">
-        <v>Physical altercations</v>
+        <v>Longest sobriety in the last five years</v>
       </c>
       <c r="C96" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Whole number</v>
       </c>
       <c r="D96" s="29" t="str">
-        <v>09 Safety and support</v>
+        <v>08 Substance use and recovery</v>
       </c>
       <c r="E96" s="3"/>
     </row>
     <row r="97" ht="34" customHeight="1">
       <c r="A97" s="3"/>
       <c r="B97" s="29" t="str">
-        <v>Physical altercation details</v>
+        <v>Behavioral history</v>
       </c>
       <c r="C97" s="29" t="str">
         <v>Text or notes</v>
@@ -13044,7 +13249,7 @@
     <row r="98" ht="34" customHeight="1">
       <c r="A98" s="3"/>
       <c r="B98" s="29" t="str">
-        <v>History of self-harm</v>
+        <v>Physical altercations</v>
       </c>
       <c r="C98" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13057,7 +13262,7 @@
     <row r="99" ht="34" customHeight="1">
       <c r="A99" s="3"/>
       <c r="B99" s="29" t="str">
-        <v>Last documented self-harm incident</v>
+        <v>Physical altercation details</v>
       </c>
       <c r="C99" s="29" t="str">
         <v>Text or notes</v>
@@ -13070,7 +13275,7 @@
     <row r="100" ht="34" customHeight="1">
       <c r="A100" s="3"/>
       <c r="B100" s="29" t="str">
-        <v>Current self-harm ideation</v>
+        <v>History of self-harm</v>
       </c>
       <c r="C100" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13083,7 +13288,7 @@
     <row r="101" ht="34" customHeight="1">
       <c r="A101" s="3"/>
       <c r="B101" s="29" t="str">
-        <v>Current self-harm ideation details</v>
+        <v>Last documented self-harm incident</v>
       </c>
       <c r="C101" s="29" t="str">
         <v>Text or notes</v>
@@ -13096,10 +13301,10 @@
     <row r="102" ht="34" customHeight="1">
       <c r="A102" s="3"/>
       <c r="B102" s="29" t="str">
-        <v>Current safety measures</v>
+        <v>Current self-harm ideation</v>
       </c>
       <c r="C102" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D102" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13109,10 +13314,10 @@
     <row r="103" ht="34" customHeight="1">
       <c r="A103" s="3"/>
       <c r="B103" s="29" t="str">
-        <v>History of assaults</v>
+        <v>Current self-harm ideation details</v>
       </c>
       <c r="C103" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D103" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13122,7 +13327,7 @@
     <row r="104" ht="34" customHeight="1">
       <c r="A104" s="3"/>
       <c r="B104" s="29" t="str">
-        <v>Most recent assault</v>
+        <v>Current safety measures</v>
       </c>
       <c r="C104" s="29" t="str">
         <v>Text or notes</v>
@@ -13135,10 +13340,10 @@
     <row r="105" ht="34" customHeight="1">
       <c r="A105" s="3"/>
       <c r="B105" s="29" t="str">
-        <v>Assaults in the last two years</v>
+        <v>History of assaults</v>
       </c>
       <c r="C105" s="29" t="str">
-        <v>Whole number</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D105" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13148,10 +13353,10 @@
     <row r="106" ht="34" customHeight="1">
       <c r="A106" s="3"/>
       <c r="B106" s="29" t="str">
-        <v>History of elopement</v>
+        <v>Most recent assault</v>
       </c>
       <c r="C106" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D106" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13161,10 +13366,10 @@
     <row r="107" ht="34" customHeight="1">
       <c r="A107" s="3"/>
       <c r="B107" s="29" t="str">
-        <v>Elopement risk</v>
+        <v>Assaults in the last two years</v>
       </c>
       <c r="C107" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D107" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13174,10 +13379,10 @@
     <row r="108" ht="34" customHeight="1">
       <c r="A108" s="3"/>
       <c r="B108" s="29" t="str">
-        <v>SI / HI history</v>
+        <v>History of elopement</v>
       </c>
       <c r="C108" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D108" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13187,7 +13392,7 @@
     <row r="109" ht="34" customHeight="1">
       <c r="A109" s="3"/>
       <c r="B109" s="29" t="str">
-        <v>Triggers and what helps</v>
+        <v>Elopement risk</v>
       </c>
       <c r="C109" s="29" t="str">
         <v>Text or notes</v>
@@ -13200,7 +13405,7 @@
     <row r="110" ht="34" customHeight="1">
       <c r="A110" s="3"/>
       <c r="B110" s="29" t="str">
-        <v>Aggression risk</v>
+        <v>SI / HI history</v>
       </c>
       <c r="C110" s="29" t="str">
         <v>Text or notes</v>
@@ -13213,7 +13418,7 @@
     <row r="111" ht="34" customHeight="1">
       <c r="A111" s="3"/>
       <c r="B111" s="29" t="str">
-        <v>Responds to internal stimuli</v>
+        <v>Triggers and what helps</v>
       </c>
       <c r="C111" s="29" t="str">
         <v>Text or notes</v>
@@ -13226,7 +13431,7 @@
     <row r="112" ht="34" customHeight="1">
       <c r="A112" s="3"/>
       <c r="B112" s="29" t="str">
-        <v>Auditory hallucinations</v>
+        <v>Aggression risk</v>
       </c>
       <c r="C112" s="29" t="str">
         <v>Text or notes</v>
@@ -13239,7 +13444,7 @@
     <row r="113" ht="34" customHeight="1">
       <c r="A113" s="3"/>
       <c r="B113" s="29" t="str">
-        <v>Nature of auditory hallucinations</v>
+        <v>Responds to internal stimuli</v>
       </c>
       <c r="C113" s="29" t="str">
         <v>Text or notes</v>
@@ -13252,7 +13457,7 @@
     <row r="114" ht="34" customHeight="1">
       <c r="A114" s="3"/>
       <c r="B114" s="29" t="str">
-        <v>Current auditory frequency</v>
+        <v>Auditory hallucinations</v>
       </c>
       <c r="C114" s="29" t="str">
         <v>Text or notes</v>
@@ -13265,7 +13470,7 @@
     <row r="115" ht="34" customHeight="1">
       <c r="A115" s="3"/>
       <c r="B115" s="29" t="str">
-        <v>Auditory triggers</v>
+        <v>Nature of auditory hallucinations</v>
       </c>
       <c r="C115" s="29" t="str">
         <v>Text or notes</v>
@@ -13278,7 +13483,7 @@
     <row r="116" ht="34" customHeight="1">
       <c r="A116" s="3"/>
       <c r="B116" s="29" t="str">
-        <v>Visual hallucinations</v>
+        <v>Current auditory frequency</v>
       </c>
       <c r="C116" s="29" t="str">
         <v>Text or notes</v>
@@ -13291,7 +13496,7 @@
     <row r="117" ht="34" customHeight="1">
       <c r="A117" s="3"/>
       <c r="B117" s="29" t="str">
-        <v>Nature and frequency of visual hallucinations</v>
+        <v>Auditory triggers</v>
       </c>
       <c r="C117" s="29" t="str">
         <v>Text or notes</v>
@@ -13304,7 +13509,7 @@
     <row r="118" ht="34" customHeight="1">
       <c r="A118" s="3"/>
       <c r="B118" s="29" t="str">
-        <v>Recent visual hallucinations</v>
+        <v>Visual hallucinations</v>
       </c>
       <c r="C118" s="29" t="str">
         <v>Text or notes</v>
@@ -13317,7 +13522,7 @@
     <row r="119" ht="34" customHeight="1">
       <c r="A119" s="3"/>
       <c r="B119" s="29" t="str">
-        <v>Olfactory hallucinations</v>
+        <v>Nature and frequency of visual hallucinations</v>
       </c>
       <c r="C119" s="29" t="str">
         <v>Text or notes</v>
@@ -13330,7 +13535,7 @@
     <row r="120" ht="34" customHeight="1">
       <c r="A120" s="3"/>
       <c r="B120" s="29" t="str">
-        <v>Olfactory hallucination details</v>
+        <v>Recent visual hallucinations</v>
       </c>
       <c r="C120" s="29" t="str">
         <v>Text or notes</v>
@@ -13343,7 +13548,7 @@
     <row r="121" ht="34" customHeight="1">
       <c r="A121" s="3"/>
       <c r="B121" s="29" t="str">
-        <v>Impact of olfactory hallucinations</v>
+        <v>Olfactory hallucinations</v>
       </c>
       <c r="C121" s="29" t="str">
         <v>Text or notes</v>
@@ -13356,7 +13561,7 @@
     <row r="122" ht="34" customHeight="1">
       <c r="A122" s="3"/>
       <c r="B122" s="29" t="str">
-        <v>Tactile hallucinations</v>
+        <v>Olfactory hallucination details</v>
       </c>
       <c r="C122" s="29" t="str">
         <v>Text or notes</v>
@@ -13369,7 +13574,7 @@
     <row r="123" ht="34" customHeight="1">
       <c r="A123" s="3"/>
       <c r="B123" s="29" t="str">
-        <v>Tactile hallucination details</v>
+        <v>Impact of olfactory hallucinations</v>
       </c>
       <c r="C123" s="29" t="str">
         <v>Text or notes</v>
@@ -13382,7 +13587,7 @@
     <row r="124" ht="34" customHeight="1">
       <c r="A124" s="3"/>
       <c r="B124" s="29" t="str">
-        <v>Tactile hallucination frequency</v>
+        <v>Tactile hallucinations</v>
       </c>
       <c r="C124" s="29" t="str">
         <v>Text or notes</v>
@@ -13395,7 +13600,7 @@
     <row r="125" ht="34" customHeight="1">
       <c r="A125" s="3"/>
       <c r="B125" s="29" t="str">
-        <v>Gustatory hallucinations</v>
+        <v>Tactile hallucination details</v>
       </c>
       <c r="C125" s="29" t="str">
         <v>Text or notes</v>
@@ -13408,7 +13613,7 @@
     <row r="126" ht="34" customHeight="1">
       <c r="A126" s="3"/>
       <c r="B126" s="29" t="str">
-        <v>Gustatory hallucination details</v>
+        <v>Tactile hallucination frequency</v>
       </c>
       <c r="C126" s="29" t="str">
         <v>Text or notes</v>
@@ -13421,7 +13626,7 @@
     <row r="127" ht="34" customHeight="1">
       <c r="A127" s="3"/>
       <c r="B127" s="29" t="str">
-        <v>Hallucination coping strategies</v>
+        <v>Gustatory hallucinations</v>
       </c>
       <c r="C127" s="29" t="str">
         <v>Text or notes</v>
@@ -13434,7 +13639,7 @@
     <row r="128" ht="34" customHeight="1">
       <c r="A128" s="3"/>
       <c r="B128" s="29" t="str">
-        <v>Hallucination distress or impairment</v>
+        <v>Gustatory hallucination details</v>
       </c>
       <c r="C128" s="29" t="str">
         <v>Text or notes</v>
@@ -13447,7 +13652,7 @@
     <row r="129" ht="34" customHeight="1">
       <c r="A129" s="3"/>
       <c r="B129" s="29" t="str">
-        <v>Impact on daily functioning</v>
+        <v>Hallucination coping strategies</v>
       </c>
       <c r="C129" s="29" t="str">
         <v>Text or notes</v>
@@ -13460,7 +13665,7 @@
     <row r="130" ht="34" customHeight="1">
       <c r="A130" s="3"/>
       <c r="B130" s="29" t="str">
-        <v>Professional discussion and treatment</v>
+        <v>Hallucination distress or impairment</v>
       </c>
       <c r="C130" s="29" t="str">
         <v>Text or notes</v>
@@ -13473,36 +13678,36 @@
     <row r="131" ht="34" customHeight="1">
       <c r="A131" s="3"/>
       <c r="B131" s="29" t="str">
-        <v>Conserved status</v>
+        <v>Impact on daily functioning</v>
       </c>
       <c r="C131" s="29" t="str">
-        <v>LPS; TCon; Murphy's; Non-Conserved</v>
+        <v>Text or notes</v>
       </c>
       <c r="D131" s="29" t="str">
-        <v>10 Decisions and legal support</v>
+        <v>09 Safety and support</v>
       </c>
       <c r="E131" s="3"/>
     </row>
     <row r="132" ht="34" customHeight="1">
       <c r="A132" s="3"/>
       <c r="B132" s="29" t="str">
-        <v>Conservator name</v>
+        <v>Professional discussion and treatment</v>
       </c>
       <c r="C132" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D132" s="29" t="str">
-        <v>10 Decisions and legal support</v>
+        <v>09 Safety and support</v>
       </c>
       <c r="E132" s="3"/>
     </row>
     <row r="133" ht="34" customHeight="1">
       <c r="A133" s="3"/>
       <c r="B133" s="29" t="str">
-        <v>Conservatorship details</v>
+        <v>Conserved status</v>
       </c>
       <c r="C133" s="29" t="str">
-        <v>Text or notes</v>
+        <v>LPS; TCon; Murphy's; Non-Conserved</v>
       </c>
       <c r="D133" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13512,7 +13717,7 @@
     <row r="134" ht="34" customHeight="1">
       <c r="A134" s="3"/>
       <c r="B134" s="29" t="str">
-        <v>Hold type</v>
+        <v>Conservator name</v>
       </c>
       <c r="C134" s="29" t="str">
         <v>Text or notes</v>
@@ -13525,10 +13730,10 @@
     <row r="135" ht="34" customHeight="1">
       <c r="A135" s="3"/>
       <c r="B135" s="29" t="str">
-        <v>Forensic involvement</v>
+        <v>Conservatorship details</v>
       </c>
       <c r="C135" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D135" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13538,7 +13743,7 @@
     <row r="136" ht="34" customHeight="1">
       <c r="A136" s="3"/>
       <c r="B136" s="29" t="str">
-        <v>Forensic involvement details</v>
+        <v>Hold type</v>
       </c>
       <c r="C136" s="29" t="str">
         <v>Text or notes</v>
@@ -13551,10 +13756,10 @@
     <row r="137" ht="34" customHeight="1">
       <c r="A137" s="3"/>
       <c r="B137" s="29" t="str">
-        <v>History of arrest</v>
+        <v>Forensic history</v>
       </c>
       <c r="C137" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D137" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13564,10 +13769,10 @@
     <row r="138" ht="34" customHeight="1">
       <c r="A138" s="3"/>
       <c r="B138" s="29" t="str">
-        <v>Most recent arrest date</v>
+        <v>Forensic timeline</v>
       </c>
       <c r="C138" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>One item per line</v>
       </c>
       <c r="D138" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13577,10 +13782,10 @@
     <row r="139" ht="34" customHeight="1">
       <c r="A139" s="3"/>
       <c r="B139" s="29" t="str">
-        <v>Most recent arrest charge</v>
+        <v>PC 290 registration</v>
       </c>
       <c r="C139" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D139" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13590,10 +13795,10 @@
     <row r="140" ht="34" customHeight="1">
       <c r="A140" s="3"/>
       <c r="B140" s="29" t="str">
-        <v>Time in jail</v>
+        <v>Arson history</v>
       </c>
       <c r="C140" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D140" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13603,7 +13808,7 @@
     <row r="141" ht="34" customHeight="1">
       <c r="A141" s="3"/>
       <c r="B141" s="29" t="str">
-        <v>Arrest in the last two years</v>
+        <v>Diversion client</v>
       </c>
       <c r="C141" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13616,7 +13821,7 @@
     <row r="142" ht="34" customHeight="1">
       <c r="A142" s="3"/>
       <c r="B142" s="29" t="str">
-        <v>Recent arrest details</v>
+        <v>Court requirements</v>
       </c>
       <c r="C142" s="29" t="str">
         <v>Text or notes</v>
@@ -13629,10 +13834,10 @@
     <row r="143" ht="34" customHeight="1">
       <c r="A143" s="3"/>
       <c r="B143" s="29" t="str">
-        <v>Total recorded arrests</v>
+        <v>Court dates</v>
       </c>
       <c r="C143" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D143" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13642,10 +13847,10 @@
     <row r="144" ht="34" customHeight="1">
       <c r="A144" s="3"/>
       <c r="B144" s="29" t="str">
-        <v>PC 290 registration</v>
+        <v>Probation / parole / justice</v>
       </c>
       <c r="C144" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D144" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13655,10 +13860,10 @@
     <row r="145" ht="34" customHeight="1">
       <c r="A145" s="3"/>
       <c r="B145" s="29" t="str">
-        <v>Arson history</v>
+        <v>Forensic involvement</v>
       </c>
       <c r="C145" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D145" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13668,10 +13873,10 @@
     <row r="146" ht="34" customHeight="1">
       <c r="A146" s="3"/>
       <c r="B146" s="29" t="str">
-        <v>Diversion client</v>
+        <v>Forensic involvement details</v>
       </c>
       <c r="C146" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D146" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13681,7 +13886,7 @@
     <row r="147" ht="34" customHeight="1">
       <c r="A147" s="3"/>
       <c r="B147" s="29" t="str">
-        <v>Court requirements</v>
+        <v>History of arrest</v>
       </c>
       <c r="C147" s="29" t="str">
         <v>Text or notes</v>
@@ -13694,10 +13899,10 @@
     <row r="148" ht="34" customHeight="1">
       <c r="A148" s="3"/>
       <c r="B148" s="29" t="str">
-        <v>Court dates</v>
+        <v>Most recent arrest date</v>
       </c>
       <c r="C148" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D148" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13707,7 +13912,7 @@
     <row r="149" ht="34" customHeight="1">
       <c r="A149" s="3"/>
       <c r="B149" s="29" t="str">
-        <v>Probation / parole / justice</v>
+        <v>Most recent arrest charge</v>
       </c>
       <c r="C149" s="29" t="str">
         <v>Text or notes</v>
@@ -13720,59 +13925,59 @@
     <row r="150" ht="34" customHeight="1">
       <c r="A150" s="3"/>
       <c r="B150" s="29" t="str">
-        <v>Family involvement</v>
+        <v>Time in jail</v>
       </c>
       <c r="C150" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D150" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>10 Decisions and legal support</v>
       </c>
       <c r="E150" s="3"/>
     </row>
     <row r="151" ht="34" customHeight="1">
       <c r="A151" s="3"/>
       <c r="B151" s="29" t="str">
-        <v>Friendships and social connections</v>
+        <v>Arrest in the last two years</v>
       </c>
       <c r="C151" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D151" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>10 Decisions and legal support</v>
       </c>
       <c r="E151" s="3"/>
     </row>
     <row r="152" ht="34" customHeight="1">
       <c r="A152" s="3"/>
       <c r="B152" s="29" t="str">
-        <v>Prior living situation</v>
+        <v>Recent arrest details</v>
       </c>
       <c r="C152" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D152" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>10 Decisions and legal support</v>
       </c>
       <c r="E152" s="3"/>
     </row>
     <row r="153" ht="34" customHeight="1">
       <c r="A153" s="3"/>
       <c r="B153" s="29" t="str">
-        <v>Housing history</v>
+        <v>Total recorded arrests</v>
       </c>
       <c r="C153" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D153" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>10 Decisions and legal support</v>
       </c>
       <c r="E153" s="3"/>
     </row>
     <row r="154" ht="34" customHeight="1">
       <c r="A154" s="3"/>
       <c r="B154" s="29" t="str">
-        <v>Benefits / income status</v>
+        <v>Family involvement</v>
       </c>
       <c r="C154" s="29" t="str">
         <v>Text or notes</v>
@@ -13785,7 +13990,7 @@
     <row r="155" ht="34" customHeight="1">
       <c r="A155" s="3"/>
       <c r="B155" s="29" t="str">
-        <v>Preferred facility characteristics</v>
+        <v>Friendships and social connections</v>
       </c>
       <c r="C155" s="29" t="str">
         <v>Text or notes</v>
@@ -13798,7 +14003,7 @@
     <row r="156" ht="34" customHeight="1">
       <c r="A156" s="3"/>
       <c r="B156" s="29" t="str">
-        <v>Discharge planning goals</v>
+        <v>Prior living situation</v>
       </c>
       <c r="C156" s="29" t="str">
         <v>Text or notes</v>
@@ -13811,7 +14016,7 @@
     <row r="157" ht="34" customHeight="1">
       <c r="A157" s="3"/>
       <c r="B157" s="29" t="str">
-        <v>Placement preferences and concerns</v>
+        <v>Housing history</v>
       </c>
       <c r="C157" s="29" t="str">
         <v>Text or notes</v>
@@ -13824,68 +14029,92 @@
     <row r="158" ht="34" customHeight="1">
       <c r="A158" s="3"/>
       <c r="B158" s="29" t="str">
-        <v>Additional information</v>
+        <v>Benefits / income status</v>
       </c>
       <c r="C158" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D158" s="29" t="str">
-        <v>12 Anything else</v>
+        <v>11 What matters next</v>
       </c>
       <c r="E158" s="3"/>
     </row>
     <row r="159" ht="34" customHeight="1">
       <c r="A159" s="3"/>
       <c r="B159" s="29" t="str">
-        <v>Placement questions or concerns</v>
+        <v>Preferred facility characteristics</v>
       </c>
       <c r="C159" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D159" s="29" t="str">
-        <v>12 Anything else</v>
+        <v>11 What matters next</v>
       </c>
       <c r="E159" s="3"/>
     </row>
     <row r="160" ht="34" customHeight="1">
       <c r="A160" s="3"/>
       <c r="B160" s="29" t="str">
-        <v>Assessment notes</v>
+        <v>Discharge planning goals</v>
       </c>
       <c r="C160" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D160" s="29" t="str">
+        <v>11 What matters next</v>
+      </c>
+      <c r="E160" s="3"/>
+    </row>
+    <row r="161" ht="34" customHeight="1">
+      <c r="A161" s="3"/>
+      <c r="B161" s="29" t="str">
+        <v>Placement preferences and concerns</v>
+      </c>
+      <c r="C161" s="29" t="str">
+        <v>Text or notes</v>
+      </c>
+      <c r="D161" s="29" t="str">
+        <v>11 What matters next</v>
+      </c>
+      <c r="E161" s="3"/>
+    </row>
+    <row r="162" ht="34" customHeight="1">
+      <c r="A162" s="3"/>
+      <c r="B162" s="29" t="str">
+        <v>Additional information</v>
+      </c>
+      <c r="C162" s="29" t="str">
+        <v>Text or notes</v>
+      </c>
+      <c r="D162" s="29" t="str">
         <v>12 Anything else</v>
       </c>
-      <c r="E160" s="3"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="3"/>
-      <c r="B161" s="3"/>
-      <c r="C161" s="3"/>
-      <c r="D161" s="3"/>
-      <c r="E161" s="3"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="3"/>
-      <c r="B162" s="3"/>
-      <c r="C162" s="3"/>
-      <c r="D162" s="3"/>
       <c r="E162" s="3"/>
     </row>
-    <row r="163">
+    <row r="163" ht="34" customHeight="1">
       <c r="A163" s="3"/>
-      <c r="B163" s="3"/>
-      <c r="C163" s="3"/>
-      <c r="D163" s="3"/>
+      <c r="B163" s="29" t="str">
+        <v>Placement questions or concerns</v>
+      </c>
+      <c r="C163" s="29" t="str">
+        <v>Text or notes</v>
+      </c>
+      <c r="D163" s="29" t="str">
+        <v>12 Anything else</v>
+      </c>
       <c r="E163" s="3"/>
     </row>
-    <row r="164">
+    <row r="164" ht="34" customHeight="1">
       <c r="A164" s="3"/>
-      <c r="B164" s="3"/>
-      <c r="C164" s="3"/>
-      <c r="D164" s="3"/>
+      <c r="B164" s="29" t="str">
+        <v>Assessment notes</v>
+      </c>
+      <c r="C164" s="29" t="str">
+        <v>Text or notes</v>
+      </c>
+      <c r="D164" s="29" t="str">
+        <v>12 Anything else</v>
+      </c>
       <c r="E164" s="3"/>
     </row>
     <row r="165">
@@ -13908,6 +14137,34 @@
       <c r="C167" s="3"/>
       <c r="D167" s="3"/>
       <c r="E167" s="3"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="3"/>
+      <c r="B168" s="3"/>
+      <c r="C168" s="3"/>
+      <c r="D168" s="3"/>
+      <c r="E168" s="3"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="3"/>
+      <c r="B169" s="3"/>
+      <c r="C169" s="3"/>
+      <c r="D169" s="3"/>
+      <c r="E169" s="3"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="3"/>
+      <c r="B170" s="3"/>
+      <c r="C170" s="3"/>
+      <c r="D170" s="3"/>
+      <c r="E170" s="3"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="3"/>
+      <c r="B171" s="3"/>
+      <c r="C171" s="3"/>
+      <c r="D171" s="3"/>
+      <c r="E171" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17356,59 +17613,248 @@
         <v>Optional</v>
       </c>
     </row>
-    <row r="8" ht="34" customHeight="1">
+    <row r="8" ht="72" customHeight="1">
       <c r="A8" s="3" t="str">
-        <v>prior_hospitalizations_count</v>
+        <v>hospitalization_history</v>
       </c>
       <c r="B8" s="13" t="str">
-        <v>Prior hospitalizations</v>
-      </c>
-      <c r="C8" t="str" s="58"/>
+        <v>Hospitalization history</v>
+      </c>
+      <c r="C8" t="str" s="50"/>
       <c r="D8" t="str" s="48"/>
       <c r="E8" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C8))&gt;0,LEN(TRIM(D8))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D8))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D8))&gt;0)),"Explain why",IF(LEN(TRIM(C8))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
-        <v>Needs answer</v>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C8))&gt;0,LEN(TRIM(D8))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D8))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D8))&gt;0)),"Explain why",IF(LEN(TRIM(C8))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="3" t="str">
-        <v>most_recent_hospitalization</v>
-      </c>
-      <c r="B9" s="13" t="str">
-        <v>Most recent hospitalization</v>
-      </c>
-      <c r="C9" t="str" s="51"/>
+        <v>hospitalization_timeline</v>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="12"/>
+              <color rgb="FF233B32"/>
+            </rPr>
+            <t>Hospitalization timeline</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="0"/>
+              <sz val="10"/>
+              <color rgb="FF59675F"/>
+            </rPr>
+            <t xml:space="preserve">
+Optional. Add an event only when you know enough to describe it; approximate timing is fine.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C9" t="str" s="50"/>
       <c r="D9" t="str" s="48"/>
       <c r="E9" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C9))&gt;0,LEN(TRIM(D9))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D9))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D9))&gt;0)),"Explain why",IF(LEN(TRIM(C9))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C9&amp;""&amp;C10&amp;""&amp;C11&amp;""&amp;C12&amp;""&amp;C13&amp;""&amp;C14&amp;""&amp;C15&amp;""&amp;C16&amp;""&amp;C17&amp;""&amp;C18&amp;""&amp;C19&amp;""&amp;C20&amp;""&amp;C21&amp;""&amp;C22))&gt;0,LEN(TRIM(D9))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D9))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D9))&gt;0)),"Explain why",IF(LEN(TRIM(C9&amp;""&amp;C10&amp;""&amp;C11&amp;""&amp;C12&amp;""&amp;C13&amp;""&amp;C14&amp;""&amp;C15&amp;""&amp;C16&amp;""&amp;C17&amp;""&amp;C18&amp;""&amp;C19&amp;""&amp;C20&amp;""&amp;C21&amp;""&amp;C22))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
         <v>Optional</v>
       </c>
     </row>
-    <row r="10" ht="72" customHeight="1">
+    <row r="10" ht="88" customHeight="1" hidden="1">
       <c r="A10" s="3" t="str">
+        <v>hospitalization_timeline:1</v>
+      </c>
+      <c r="B10" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C10" t="str" s="57"/>
+      <c r="D10" s="3" t="str"/>
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" ht="88" customHeight="1" hidden="1">
+      <c r="A11" s="3" t="str">
+        <v>hospitalization_timeline:2</v>
+      </c>
+      <c r="B11" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C11" t="str" s="57"/>
+      <c r="D11" s="3" t="str"/>
+      <c r="E11" s="3"/>
+    </row>
+    <row r="12" ht="88" customHeight="1" hidden="1">
+      <c r="A12" s="3" t="str">
+        <v>hospitalization_timeline:3</v>
+      </c>
+      <c r="B12" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C12" t="str" s="57"/>
+      <c r="D12" s="3" t="str"/>
+      <c r="E12" s="3"/>
+    </row>
+    <row r="13" ht="88" customHeight="1" hidden="1">
+      <c r="A13" s="3" t="str">
+        <v>hospitalization_timeline:4</v>
+      </c>
+      <c r="B13" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C13" t="str" s="57"/>
+      <c r="D13" s="3" t="str"/>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" ht="88" customHeight="1" hidden="1">
+      <c r="A14" s="3" t="str">
+        <v>hospitalization_timeline:5</v>
+      </c>
+      <c r="B14" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C14" t="str" s="57"/>
+      <c r="D14" s="3" t="str"/>
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" ht="88" customHeight="1" hidden="1">
+      <c r="A15" s="3" t="str">
+        <v>hospitalization_timeline:6</v>
+      </c>
+      <c r="B15" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C15" t="str" s="57"/>
+      <c r="D15" s="3" t="str"/>
+      <c r="E15" s="3"/>
+    </row>
+    <row r="16" ht="88" customHeight="1" hidden="1">
+      <c r="A16" s="3" t="str">
+        <v>hospitalization_timeline:7</v>
+      </c>
+      <c r="B16" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C16" t="str" s="57"/>
+      <c r="D16" s="3" t="str"/>
+      <c r="E16" s="3"/>
+    </row>
+    <row r="17" ht="88" customHeight="1" hidden="1">
+      <c r="A17" s="3" t="str">
+        <v>hospitalization_timeline:8</v>
+      </c>
+      <c r="B17" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C17" t="str" s="57"/>
+      <c r="D17" s="3" t="str"/>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" ht="88" customHeight="1" hidden="1">
+      <c r="A18" s="3" t="str">
+        <v>hospitalization_timeline:9</v>
+      </c>
+      <c r="B18" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C18" t="str" s="57"/>
+      <c r="D18" s="3" t="str"/>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" ht="88" customHeight="1" hidden="1">
+      <c r="A19" s="3" t="str">
+        <v>hospitalization_timeline:10</v>
+      </c>
+      <c r="B19" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C19" t="str" s="57"/>
+      <c r="D19" s="3" t="str"/>
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" ht="88" customHeight="1" hidden="1">
+      <c r="A20" s="3" t="str">
+        <v>hospitalization_timeline:11</v>
+      </c>
+      <c r="B20" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C20" t="str" s="57"/>
+      <c r="D20" s="3" t="str"/>
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" ht="88" customHeight="1" hidden="1">
+      <c r="A21" s="3" t="str">
+        <v>hospitalization_timeline:12</v>
+      </c>
+      <c r="B21" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C21" t="str" s="57"/>
+      <c r="D21" s="3" t="str"/>
+      <c r="E21" s="3"/>
+    </row>
+    <row r="22" ht="88" customHeight="1" hidden="1">
+      <c r="A22" s="3" t="str">
+        <v>hospitalization_timeline:13</v>
+      </c>
+      <c r="B22" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C22" t="str" s="57"/>
+      <c r="D22" s="3" t="str"/>
+      <c r="E22" s="3"/>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="3" t="str">
+        <v>prior_hospitalizations_count</v>
+      </c>
+      <c r="B23" s="13" t="str">
+        <v>Prior hospitalizations</v>
+      </c>
+      <c r="C23" t="str" s="58"/>
+      <c r="D23" t="str" s="48"/>
+      <c r="E23" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C23))&gt;0,LEN(TRIM(D23))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D23))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D23))&gt;0)),"Explain why",IF(LEN(TRIM(C23))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="3" t="str">
+        <v>most_recent_hospitalization</v>
+      </c>
+      <c r="B24" s="13" t="str">
+        <v>Most recent hospitalization</v>
+      </c>
+      <c r="C24" t="str" s="51"/>
+      <c r="D24" t="str" s="48"/>
+      <c r="E24" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C24))&gt;0,LEN(TRIM(D24))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D24))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D24))&gt;0)),"Explain why",IF(LEN(TRIM(C24))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="3" t="str">
         <v>prior_5150_5250_holds</v>
       </c>
-      <c r="B10" s="13" t="str">
+      <c r="B25" s="13" t="str">
         <v>Prior 5150 / 5250 holds</v>
       </c>
-      <c r="C10" t="str" s="50"/>
-      <c r="D10" t="str" s="48"/>
-      <c r="E10" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C10))&gt;0,LEN(TRIM(D10))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D10))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D10))&gt;0)),"Explain why",IF(LEN(TRIM(C10))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+      <c r="C25" t="str" s="50"/>
+      <c r="D25" t="str" s="48"/>
+      <c r="E25" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C25))&gt;0,LEN(TRIM(D25))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D25))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D25))&gt;0)),"Explain why",IF(LEN(TRIM(C25))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
         <v>Optional</v>
       </c>
     </row>
-    <row r="11" ht="72" customHeight="1">
-      <c r="A11" s="3" t="str">
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="3" t="str">
         <v>crisis_er_utilization</v>
       </c>
-      <c r="B11" s="13" t="str">
+      <c r="B26" s="13" t="str">
         <v>Crisis / ER utilization</v>
       </c>
-      <c r="C11" t="str" s="50"/>
-      <c r="D11" t="str" s="48"/>
-      <c r="E11" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C11))&gt;0,LEN(TRIM(D11))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D11))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D11))&gt;0)),"Explain why",IF(LEN(TRIM(C11))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+      <c r="C26" t="str" s="50"/>
+      <c r="D26" t="str" s="48"/>
+      <c r="E26" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C26))&gt;0,LEN(TRIM(D26))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D26))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D26))&gt;0)),"Explain why",IF(LEN(TRIM(C26))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
         <v>Optional</v>
       </c>
     </row>
@@ -17460,32 +17906,46 @@
       <formula>OR($E9="Needs answer",$E9="Explain why",LEFT($E9,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B10:E10">
+  <conditionalFormatting sqref="B23:E23">
     <cfRule type="expression" dxfId="178" priority="9">
-      <formula>$E10="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E10:E10">
+      <formula>$E23="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E23:E23">
     <cfRule type="expression" dxfId="179" priority="10">
-      <formula>OR($E10="Needs answer",$E10="Explain why",LEFT($E10,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B11:E11">
+      <formula>OR($E23="Needs answer",$E23="Explain why",LEFT($E23,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B24:E24">
     <cfRule type="expression" dxfId="180" priority="11">
-      <formula>$E11="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E11:E11">
+      <formula>$E24="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E24:E24">
     <cfRule type="expression" dxfId="181" priority="12">
-      <formula>OR($E11="Needs answer",$E11="Explain why",LEFT($E11,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation type="whole" operator="between" sqref="C8">
-      <formula1>0</formula1>
-      <formula2>10000</formula2>
-    </dataValidation>
-  </dataValidations>
+      <formula>OR($E24="Needs answer",$E24="Explain why",LEFT($E24,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B25:E25">
+    <cfRule type="expression" dxfId="182" priority="13">
+      <formula>$E25="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E25:E25">
+    <cfRule type="expression" dxfId="183" priority="14">
+      <formula>OR($E25="Needs answer",$E25="Explain why",LEFT($E25,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B26:E26">
+    <cfRule type="expression" dxfId="184" priority="15">
+      <formula>$E26="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E26:E26">
+    <cfRule type="expression" dxfId="185" priority="16">
+      <formula>OR($E26="Needs answer",$E26="Explain why",LEFT($E26,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -18011,122 +18471,122 @@
     <mergeCell ref="B3:E3"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:E6">
-    <cfRule type="expression" dxfId="182" priority="1">
+    <cfRule type="expression" dxfId="186" priority="1">
       <formula>$E6="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6:E6">
-    <cfRule type="expression" dxfId="183" priority="2">
+    <cfRule type="expression" dxfId="187" priority="2">
       <formula>OR($E6="Needs answer",$E6="Explain why",LEFT($E6,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6:D6">
-    <cfRule type="expression" dxfId="184" priority="3">
+    <cfRule type="expression" dxfId="188" priority="3">
       <formula>OR($C6="Unable to assess",$C6="unable_to_assess")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:E7">
-    <cfRule type="expression" dxfId="185" priority="4">
+    <cfRule type="expression" dxfId="189" priority="4">
       <formula>$E7="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E7:E7">
-    <cfRule type="expression" dxfId="186" priority="5">
+    <cfRule type="expression" dxfId="190" priority="5">
       <formula>OR($E7="Needs answer",$E7="Explain why",LEFT($E7,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:D7">
-    <cfRule type="expression" dxfId="187" priority="6">
+    <cfRule type="expression" dxfId="191" priority="6">
       <formula>OR($C7="Unable to assess",$C7="unable_to_assess")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:E8">
-    <cfRule type="expression" dxfId="188" priority="7">
+    <cfRule type="expression" dxfId="192" priority="7">
       <formula>$E8="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8:E8">
-    <cfRule type="expression" dxfId="189" priority="8">
+    <cfRule type="expression" dxfId="193" priority="8">
       <formula>OR($E8="Needs answer",$E8="Explain why",LEFT($E8,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:E22">
-    <cfRule type="expression" dxfId="190" priority="9">
+    <cfRule type="expression" dxfId="194" priority="9">
       <formula>$E22="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E22:E22">
-    <cfRule type="expression" dxfId="191" priority="10">
+    <cfRule type="expression" dxfId="195" priority="10">
       <formula>OR($E22="Needs answer",$E22="Explain why",LEFT($E22,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23:E23">
-    <cfRule type="expression" dxfId="192" priority="11">
+    <cfRule type="expression" dxfId="196" priority="11">
       <formula>$E23="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E23:E23">
-    <cfRule type="expression" dxfId="193" priority="12">
+    <cfRule type="expression" dxfId="197" priority="12">
       <formula>OR($E23="Needs answer",$E23="Explain why",LEFT($E23,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24:E24">
-    <cfRule type="expression" dxfId="194" priority="13">
+    <cfRule type="expression" dxfId="198" priority="13">
       <formula>$E24="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E24:E24">
-    <cfRule type="expression" dxfId="195" priority="14">
+    <cfRule type="expression" dxfId="199" priority="14">
       <formula>OR($E24="Needs answer",$E24="Explain why",LEFT($E24,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25:E25">
-    <cfRule type="expression" dxfId="196" priority="15">
+    <cfRule type="expression" dxfId="200" priority="15">
       <formula>$E25="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25:E25">
-    <cfRule type="expression" dxfId="197" priority="16">
+    <cfRule type="expression" dxfId="201" priority="16">
       <formula>OR($E25="Needs answer",$E25="Explain why",LEFT($E25,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:E26">
-    <cfRule type="expression" dxfId="198" priority="17">
+    <cfRule type="expression" dxfId="202" priority="17">
       <formula>$E26="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E26:E26">
-    <cfRule type="expression" dxfId="199" priority="18">
+    <cfRule type="expression" dxfId="203" priority="18">
       <formula>OR($E26="Needs answer",$E26="Explain why",LEFT($E26,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:E27">
-    <cfRule type="expression" dxfId="200" priority="19">
+    <cfRule type="expression" dxfId="204" priority="19">
       <formula>$E27="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E27:E27">
-    <cfRule type="expression" dxfId="201" priority="20">
+    <cfRule type="expression" dxfId="205" priority="20">
       <formula>OR($E27="Needs answer",$E27="Explain why",LEFT($E27,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28:E28">
-    <cfRule type="expression" dxfId="202" priority="21">
+    <cfRule type="expression" dxfId="206" priority="21">
       <formula>$E28="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E28:E28">
-    <cfRule type="expression" dxfId="203" priority="22">
+    <cfRule type="expression" dxfId="207" priority="22">
       <formula>OR($E28="Needs answer",$E28="Explain why",LEFT($E28,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29:E29">
-    <cfRule type="expression" dxfId="204" priority="23">
+    <cfRule type="expression" dxfId="208" priority="23">
       <formula>$E29="Not applicable"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E29:E29">
-    <cfRule type="expression" dxfId="205" priority="24">
+    <cfRule type="expression" dxfId="209" priority="24">
       <formula>OR($E29="Needs answer",$E29="Explain why",LEFT($E29,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Simplify intake medication reference and placement history
(cherry picked from commit 15e02fe301feb2bf1312727467e084070bb4c201)
</commit_message>
<xml_diff>
--- a/public/templates/pipeline-assessment-workbook.xlsx
+++ b/public/templates/pipeline-assessment-workbook.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R2fcb16bfacf74ef7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="R83dcd224a24a4f05"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="Rebc4e9e1c4c54ca0"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="Ra8a42a95b98748cd"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="R5f9921955eb745ef"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="Rf794a62138a74c0c"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="Rf8b55cac3b314109"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="Re7780c6dd2cd4f43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="R386f0510ac0a426b"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R282480e6d0094a89"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="R6983b7cb1a294d1c"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R25c59fc2162549b0"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="R919b6692dd9440fa"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="R7b1b5c4c758446cf" state="veryHidden"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="R666bd830afe64dc1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rea505e774e45403c"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="R0c0157dd3bfb4404"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R613c4939346946e5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="Rd4cdafd37d674dcc"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Re49e3869eecc4849"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="Ra7a741e3af554825"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="Rb6f7ae69db834e53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="R229fa0a170c64755"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="R31a37d5ce5d14959"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R1110fc44b1e94567"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="R01ce2b7e25c84ec2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R8e7cbcc449b04976"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="R9cae6c060a474f4f"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="Rb861b1ec397245fa" state="veryHidden"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="R9b58ee9f9cd34eaa"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Confirm the basics'!$B$1:$E$16</definedName>
@@ -7099,14 +7099,32 @@
       <c r="A8" s="3" t="str">
         <v>prior_living_situation</v>
       </c>
-      <c r="B8" s="13" t="str">
-        <v>Prior living situation</v>
-      </c>
-      <c r="C8" t="str" s="50"/>
-      <c r="D8" t="str" s="48"/>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="12"/>
+              <color rgb="FF233B32"/>
+            </rPr>
+            <t>Earlier living-situation answer</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="0"/>
+              <sz val="10"/>
+              <color rgb="FF59675F"/>
+            </rPr>
+            <t xml:space="preserve">
+Reference only.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C8" s="23" t="str"/>
+      <c r="D8" s="15" t="str"/>
       <c r="E8" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C8))&gt;0,LEN(TRIM(D8))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D8))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D8))&gt;0)),"Explain why",IF(LEN(TRIM(C8))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
+        <f>"Reference only"</f>
+        <v>Reference only</v>
       </c>
     </row>
     <row r="9" ht="72" customHeight="1">
@@ -7114,7 +7132,7 @@
         <v>housing_history</v>
       </c>
       <c r="B9" s="13" t="str">
-        <v>Housing history</v>
+        <v>Home and housing history</v>
       </c>
       <c r="C9" t="str" s="50"/>
       <c r="D9" t="str" s="48"/>
@@ -7989,7 +8007,7 @@
         <v>Questionnaire fingerprint</v>
       </c>
       <c r="B2" t="str">
-        <v>ceae1f99319c6b47c35e1e3822d9ec6d9ed0a082eb073f9b53612b111faaec6f</v>
+        <v>a411199d0450c15c3e8fce1cba5e44bb4ace2fe3931c189ead5e4f7a7bec55c7</v>
       </c>
     </row>
     <row r="3">
@@ -12131,7 +12149,7 @@
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="3"/>
       <c r="B12" s="29" t="str">
-        <v>Current location</v>
+        <v>Where the client is now</v>
       </c>
       <c r="C12" s="29" t="str">
         <v>Text or notes</v>
@@ -12833,10 +12851,10 @@
     <row r="66" ht="34" customHeight="1">
       <c r="A66" s="3"/>
       <c r="B66" s="29" t="str">
-        <v>Medications at intake</v>
+        <v>PRN patterns</v>
       </c>
       <c r="C66" s="29" t="str">
-        <v>One item per line</v>
+        <v>Text or notes</v>
       </c>
       <c r="D66" s="29" t="str">
         <v>05 Medication</v>
@@ -12846,10 +12864,10 @@
     <row r="67" ht="34" customHeight="1">
       <c r="A67" s="3"/>
       <c r="B67" s="29" t="str">
-        <v>PRN patterns</v>
+        <v>IM injections</v>
       </c>
       <c r="C67" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D67" s="29" t="str">
         <v>05 Medication</v>
@@ -12859,10 +12877,10 @@
     <row r="68" ht="34" customHeight="1">
       <c r="A68" s="3"/>
       <c r="B68" s="29" t="str">
-        <v>IM injections</v>
+        <v>Injection details</v>
       </c>
       <c r="C68" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D68" s="29" t="str">
         <v>05 Medication</v>
@@ -12872,7 +12890,7 @@
     <row r="69" ht="34" customHeight="1">
       <c r="A69" s="3"/>
       <c r="B69" s="29" t="str">
-        <v>Injection details</v>
+        <v>Injection frequency</v>
       </c>
       <c r="C69" s="29" t="str">
         <v>Text or notes</v>
@@ -12885,7 +12903,7 @@
     <row r="70" ht="34" customHeight="1">
       <c r="A70" s="3"/>
       <c r="B70" s="29" t="str">
-        <v>Injection frequency</v>
+        <v>Last injection</v>
       </c>
       <c r="C70" s="29" t="str">
         <v>Text or notes</v>
@@ -12898,7 +12916,7 @@
     <row r="71" ht="34" customHeight="1">
       <c r="A71" s="3"/>
       <c r="B71" s="29" t="str">
-        <v>Last injection</v>
+        <v>Next injection due</v>
       </c>
       <c r="C71" s="29" t="str">
         <v>Text or notes</v>
@@ -12911,7 +12929,7 @@
     <row r="72" ht="34" customHeight="1">
       <c r="A72" s="3"/>
       <c r="B72" s="29" t="str">
-        <v>Next injection due</v>
+        <v>LAI vs oral</v>
       </c>
       <c r="C72" s="29" t="str">
         <v>Text or notes</v>
@@ -12924,36 +12942,36 @@
     <row r="73" ht="34" customHeight="1">
       <c r="A73" s="3"/>
       <c r="B73" s="29" t="str">
-        <v>LAI vs oral</v>
+        <v>County</v>
       </c>
       <c r="C73" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D73" s="29" t="str">
-        <v>05 Medication</v>
+        <v>06 Living situation</v>
       </c>
       <c r="E73" s="3"/>
     </row>
-    <row r="74" ht="34" customHeight="1">
+    <row r="74" ht="76" customHeight="1">
       <c r="A74" s="3"/>
       <c r="B74" s="29" t="str">
-        <v>County</v>
+        <v>Most recent setting type</v>
       </c>
       <c r="C74" s="29" t="str">
-        <v>Text or notes</v>
+        <v>State hospital; Acute psychiatric hospital; IMD / MHRC; Skilled nursing facility; Board and care; Residential program; Jail / forensic setting; Independent or family home; Unhoused; Other</v>
       </c>
       <c r="D74" s="29" t="str">
         <v>06 Living situation</v>
       </c>
       <c r="E74" s="3"/>
     </row>
-    <row r="75" ht="76" customHeight="1">
+    <row r="75" ht="34" customHeight="1">
       <c r="A75" s="3"/>
       <c r="B75" s="29" t="str">
-        <v>Prior setting type</v>
+        <v>Most recent facility or program</v>
       </c>
       <c r="C75" s="29" t="str">
-        <v>State hospital; Acute psychiatric hospital; IMD / MHRC; Skilled nursing facility; Board and care; Residential program; Jail / forensic setting; Independent or family home; Unhoused; Other</v>
+        <v>Text or notes</v>
       </c>
       <c r="D75" s="29" t="str">
         <v>06 Living situation</v>
@@ -12963,10 +12981,10 @@
     <row r="76" ht="34" customHeight="1">
       <c r="A76" s="3"/>
       <c r="B76" s="29" t="str">
-        <v>Prior placement name</v>
+        <v>Admit date</v>
       </c>
       <c r="C76" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D76" s="29" t="str">
         <v>06 Living situation</v>
@@ -12976,20 +12994,20 @@
     <row r="77" ht="34" customHeight="1">
       <c r="A77" s="3"/>
       <c r="B77" s="29" t="str">
-        <v>Admit date</v>
+        <v>Earlier care placements</v>
       </c>
       <c r="C77" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D77" s="29" t="str">
-        <v>06 Living situation</v>
+        <v>07 Recent care and history</v>
       </c>
       <c r="E77" s="3"/>
     </row>
     <row r="78" ht="34" customHeight="1">
       <c r="A78" s="3"/>
       <c r="B78" s="29" t="str">
-        <v>Prior placements</v>
+        <v>Prior AWOL / failed placements</v>
       </c>
       <c r="C78" s="29" t="str">
         <v>Text or notes</v>
@@ -13002,7 +13020,7 @@
     <row r="79" ht="34" customHeight="1">
       <c r="A79" s="3"/>
       <c r="B79" s="29" t="str">
-        <v>Prior AWOL / failed placements</v>
+        <v>Hospitalization history</v>
       </c>
       <c r="C79" s="29" t="str">
         <v>Text or notes</v>
@@ -13015,10 +13033,10 @@
     <row r="80" ht="34" customHeight="1">
       <c r="A80" s="3"/>
       <c r="B80" s="29" t="str">
-        <v>Hospitalization history</v>
+        <v>Hospitalization timeline</v>
       </c>
       <c r="C80" s="29" t="str">
-        <v>Text or notes</v>
+        <v>One item per line</v>
       </c>
       <c r="D80" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -13028,10 +13046,10 @@
     <row r="81" ht="34" customHeight="1">
       <c r="A81" s="3"/>
       <c r="B81" s="29" t="str">
-        <v>Hospitalization timeline</v>
+        <v>Prior hospitalizations</v>
       </c>
       <c r="C81" s="29" t="str">
-        <v>One item per line</v>
+        <v>Whole number</v>
       </c>
       <c r="D81" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -13041,10 +13059,10 @@
     <row r="82" ht="34" customHeight="1">
       <c r="A82" s="3"/>
       <c r="B82" s="29" t="str">
-        <v>Prior hospitalizations</v>
+        <v>Most recent hospitalization</v>
       </c>
       <c r="C82" s="29" t="str">
-        <v>Whole number</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D82" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -13054,10 +13072,10 @@
     <row r="83" ht="34" customHeight="1">
       <c r="A83" s="3"/>
       <c r="B83" s="29" t="str">
-        <v>Most recent hospitalization</v>
+        <v>Prior 5150 / 5250 holds</v>
       </c>
       <c r="C83" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D83" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -13067,7 +13085,7 @@
     <row r="84" ht="34" customHeight="1">
       <c r="A84" s="3"/>
       <c r="B84" s="29" t="str">
-        <v>Prior 5150 / 5250 holds</v>
+        <v>Crisis / ER utilization</v>
       </c>
       <c r="C84" s="29" t="str">
         <v>Text or notes</v>
@@ -13080,20 +13098,20 @@
     <row r="85" ht="34" customHeight="1">
       <c r="A85" s="3"/>
       <c r="B85" s="29" t="str">
-        <v>Crisis / ER utilization</v>
+        <v>History of substance abuse</v>
       </c>
       <c r="C85" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D85" s="29" t="str">
-        <v>07 Recent care and history</v>
+        <v>08 Substance use and recovery</v>
       </c>
       <c r="E85" s="3"/>
     </row>
     <row r="86" ht="34" customHeight="1">
       <c r="A86" s="3"/>
       <c r="B86" s="29" t="str">
-        <v>History of substance abuse</v>
+        <v>Active substance use</v>
       </c>
       <c r="C86" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13106,10 +13124,10 @@
     <row r="87" ht="34" customHeight="1">
       <c r="A87" s="3"/>
       <c r="B87" s="29" t="str">
-        <v>Active substance use</v>
+        <v>Substances</v>
       </c>
       <c r="C87" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Opioids; Amphetamines; Marijuana; Alcohol; Other</v>
       </c>
       <c r="D87" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13119,10 +13137,10 @@
     <row r="88" ht="34" customHeight="1">
       <c r="A88" s="3"/>
       <c r="B88" s="29" t="str">
-        <v>Substances</v>
+        <v>Last substance use</v>
       </c>
       <c r="C88" s="29" t="str">
-        <v>Opioids; Amphetamines; Marijuana; Alcohol; Other</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D88" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13132,10 +13150,10 @@
     <row r="89" ht="34" customHeight="1">
       <c r="A89" s="3"/>
       <c r="B89" s="29" t="str">
-        <v>Last substance use</v>
+        <v>Use pattern</v>
       </c>
       <c r="C89" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Daily; Weekly; Sporadic; Rarely</v>
       </c>
       <c r="D89" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13145,49 +13163,49 @@
     <row r="90" ht="34" customHeight="1">
       <c r="A90" s="3"/>
       <c r="B90" s="29" t="str">
-        <v>Use pattern</v>
+        <v>Effect on baseline behavior</v>
       </c>
       <c r="C90" s="29" t="str">
-        <v>Daily; Weekly; Sporadic; Rarely</v>
+        <v>Text or notes</v>
       </c>
       <c r="D90" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" ht="34" customHeight="1">
+    <row r="91" ht="60" customHeight="1">
       <c r="A91" s="3"/>
       <c r="B91" s="29" t="str">
-        <v>Effect on baseline behavior</v>
+        <v>Longest sobriety in the last five years</v>
       </c>
       <c r="C91" s="29" t="str">
-        <v>Text or notes</v>
+        <v>1 month; 2 months; 3 months; 4 months; 5 months; 6 months; 7 months; 8 months; 9 months; 10 months; 11 months; 1 year; 18 months; 2 years; More than 2 years</v>
       </c>
       <c r="D91" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" ht="60" customHeight="1">
+    <row r="92" ht="44" customHeight="1">
       <c r="A92" s="3"/>
       <c r="B92" s="29" t="str">
-        <v>Longest sobriety in the last five years</v>
+        <v>Acknowledgment of substance-use impact</v>
       </c>
       <c r="C92" s="29" t="str">
-        <v>1 month; 2 months; 3 months; 4 months; 5 months; 6 months; 7 months; 8 months; 9 months; 10 months; 11 months; 1 year; 18 months; 2 years; More than 2 years</v>
+        <v>Acknowledges impact; Partially acknowledges impact; Does not acknowledge impact; Not discussed</v>
       </c>
       <c r="D92" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E92" s="3"/>
     </row>
-    <row r="93" ht="44" customHeight="1">
+    <row r="93" ht="34" customHeight="1">
       <c r="A93" s="3"/>
       <c r="B93" s="29" t="str">
-        <v>Acknowledgment of substance-use impact</v>
+        <v>Substance-use impact notes</v>
       </c>
       <c r="C93" s="29" t="str">
-        <v>Acknowledges impact; Partially acknowledges impact; Does not acknowledge impact; Not discussed</v>
+        <v>Text or notes</v>
       </c>
       <c r="D93" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13197,7 +13215,7 @@
     <row r="94" ht="34" customHeight="1">
       <c r="A94" s="3"/>
       <c r="B94" s="29" t="str">
-        <v>Substance-use impact notes</v>
+        <v>Treatment history</v>
       </c>
       <c r="C94" s="29" t="str">
         <v>Text or notes</v>
@@ -13210,10 +13228,10 @@
     <row r="95" ht="34" customHeight="1">
       <c r="A95" s="3"/>
       <c r="B95" s="29" t="str">
-        <v>Treatment history</v>
+        <v>Longest sobriety in the last five years</v>
       </c>
       <c r="C95" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D95" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13223,23 +13241,23 @@
     <row r="96" ht="34" customHeight="1">
       <c r="A96" s="3"/>
       <c r="B96" s="29" t="str">
-        <v>Longest sobriety in the last five years</v>
+        <v>Behavioral history</v>
       </c>
       <c r="C96" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D96" s="29" t="str">
-        <v>08 Substance use and recovery</v>
+        <v>09 Safety and support</v>
       </c>
       <c r="E96" s="3"/>
     </row>
     <row r="97" ht="34" customHeight="1">
       <c r="A97" s="3"/>
       <c r="B97" s="29" t="str">
-        <v>Behavioral history</v>
+        <v>Physical altercations</v>
       </c>
       <c r="C97" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D97" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13249,10 +13267,10 @@
     <row r="98" ht="34" customHeight="1">
       <c r="A98" s="3"/>
       <c r="B98" s="29" t="str">
-        <v>Physical altercations</v>
+        <v>Physical altercation details</v>
       </c>
       <c r="C98" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D98" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13262,10 +13280,10 @@
     <row r="99" ht="34" customHeight="1">
       <c r="A99" s="3"/>
       <c r="B99" s="29" t="str">
-        <v>Physical altercation details</v>
+        <v>History of self-harm</v>
       </c>
       <c r="C99" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D99" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13275,10 +13293,10 @@
     <row r="100" ht="34" customHeight="1">
       <c r="A100" s="3"/>
       <c r="B100" s="29" t="str">
-        <v>History of self-harm</v>
+        <v>Last documented self-harm incident</v>
       </c>
       <c r="C100" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D100" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13288,10 +13306,10 @@
     <row r="101" ht="34" customHeight="1">
       <c r="A101" s="3"/>
       <c r="B101" s="29" t="str">
-        <v>Last documented self-harm incident</v>
+        <v>Current self-harm ideation</v>
       </c>
       <c r="C101" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D101" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13301,10 +13319,10 @@
     <row r="102" ht="34" customHeight="1">
       <c r="A102" s="3"/>
       <c r="B102" s="29" t="str">
-        <v>Current self-harm ideation</v>
+        <v>Current self-harm ideation details</v>
       </c>
       <c r="C102" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D102" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13314,7 +13332,7 @@
     <row r="103" ht="34" customHeight="1">
       <c r="A103" s="3"/>
       <c r="B103" s="29" t="str">
-        <v>Current self-harm ideation details</v>
+        <v>Current safety measures</v>
       </c>
       <c r="C103" s="29" t="str">
         <v>Text or notes</v>
@@ -13327,10 +13345,10 @@
     <row r="104" ht="34" customHeight="1">
       <c r="A104" s="3"/>
       <c r="B104" s="29" t="str">
-        <v>Current safety measures</v>
+        <v>History of assaults</v>
       </c>
       <c r="C104" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D104" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13340,10 +13358,10 @@
     <row r="105" ht="34" customHeight="1">
       <c r="A105" s="3"/>
       <c r="B105" s="29" t="str">
-        <v>History of assaults</v>
+        <v>Most recent assault</v>
       </c>
       <c r="C105" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D105" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13353,10 +13371,10 @@
     <row r="106" ht="34" customHeight="1">
       <c r="A106" s="3"/>
       <c r="B106" s="29" t="str">
-        <v>Most recent assault</v>
+        <v>Assaults in the last two years</v>
       </c>
       <c r="C106" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D106" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13366,10 +13384,10 @@
     <row r="107" ht="34" customHeight="1">
       <c r="A107" s="3"/>
       <c r="B107" s="29" t="str">
-        <v>Assaults in the last two years</v>
+        <v>History of elopement</v>
       </c>
       <c r="C107" s="29" t="str">
-        <v>Whole number</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D107" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13379,10 +13397,10 @@
     <row r="108" ht="34" customHeight="1">
       <c r="A108" s="3"/>
       <c r="B108" s="29" t="str">
-        <v>History of elopement</v>
+        <v>Elopement risk</v>
       </c>
       <c r="C108" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D108" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13392,7 +13410,7 @@
     <row r="109" ht="34" customHeight="1">
       <c r="A109" s="3"/>
       <c r="B109" s="29" t="str">
-        <v>Elopement risk</v>
+        <v>SI / HI history</v>
       </c>
       <c r="C109" s="29" t="str">
         <v>Text or notes</v>
@@ -13405,7 +13423,7 @@
     <row r="110" ht="34" customHeight="1">
       <c r="A110" s="3"/>
       <c r="B110" s="29" t="str">
-        <v>SI / HI history</v>
+        <v>Triggers and what helps</v>
       </c>
       <c r="C110" s="29" t="str">
         <v>Text or notes</v>
@@ -13418,7 +13436,7 @@
     <row r="111" ht="34" customHeight="1">
       <c r="A111" s="3"/>
       <c r="B111" s="29" t="str">
-        <v>Triggers and what helps</v>
+        <v>Aggression risk</v>
       </c>
       <c r="C111" s="29" t="str">
         <v>Text or notes</v>
@@ -13431,7 +13449,7 @@
     <row r="112" ht="34" customHeight="1">
       <c r="A112" s="3"/>
       <c r="B112" s="29" t="str">
-        <v>Aggression risk</v>
+        <v>Responds to internal stimuli</v>
       </c>
       <c r="C112" s="29" t="str">
         <v>Text or notes</v>
@@ -13444,7 +13462,7 @@
     <row r="113" ht="34" customHeight="1">
       <c r="A113" s="3"/>
       <c r="B113" s="29" t="str">
-        <v>Responds to internal stimuli</v>
+        <v>Auditory hallucinations</v>
       </c>
       <c r="C113" s="29" t="str">
         <v>Text or notes</v>
@@ -13457,7 +13475,7 @@
     <row r="114" ht="34" customHeight="1">
       <c r="A114" s="3"/>
       <c r="B114" s="29" t="str">
-        <v>Auditory hallucinations</v>
+        <v>Nature of auditory hallucinations</v>
       </c>
       <c r="C114" s="29" t="str">
         <v>Text or notes</v>
@@ -13470,7 +13488,7 @@
     <row r="115" ht="34" customHeight="1">
       <c r="A115" s="3"/>
       <c r="B115" s="29" t="str">
-        <v>Nature of auditory hallucinations</v>
+        <v>Current auditory frequency</v>
       </c>
       <c r="C115" s="29" t="str">
         <v>Text or notes</v>
@@ -13483,7 +13501,7 @@
     <row r="116" ht="34" customHeight="1">
       <c r="A116" s="3"/>
       <c r="B116" s="29" t="str">
-        <v>Current auditory frequency</v>
+        <v>Auditory triggers</v>
       </c>
       <c r="C116" s="29" t="str">
         <v>Text or notes</v>
@@ -13496,7 +13514,7 @@
     <row r="117" ht="34" customHeight="1">
       <c r="A117" s="3"/>
       <c r="B117" s="29" t="str">
-        <v>Auditory triggers</v>
+        <v>Visual hallucinations</v>
       </c>
       <c r="C117" s="29" t="str">
         <v>Text or notes</v>
@@ -13509,7 +13527,7 @@
     <row r="118" ht="34" customHeight="1">
       <c r="A118" s="3"/>
       <c r="B118" s="29" t="str">
-        <v>Visual hallucinations</v>
+        <v>Nature and frequency of visual hallucinations</v>
       </c>
       <c r="C118" s="29" t="str">
         <v>Text or notes</v>
@@ -13522,7 +13540,7 @@
     <row r="119" ht="34" customHeight="1">
       <c r="A119" s="3"/>
       <c r="B119" s="29" t="str">
-        <v>Nature and frequency of visual hallucinations</v>
+        <v>Recent visual hallucinations</v>
       </c>
       <c r="C119" s="29" t="str">
         <v>Text or notes</v>
@@ -13535,7 +13553,7 @@
     <row r="120" ht="34" customHeight="1">
       <c r="A120" s="3"/>
       <c r="B120" s="29" t="str">
-        <v>Recent visual hallucinations</v>
+        <v>Olfactory hallucinations</v>
       </c>
       <c r="C120" s="29" t="str">
         <v>Text or notes</v>
@@ -13548,7 +13566,7 @@
     <row r="121" ht="34" customHeight="1">
       <c r="A121" s="3"/>
       <c r="B121" s="29" t="str">
-        <v>Olfactory hallucinations</v>
+        <v>Olfactory hallucination details</v>
       </c>
       <c r="C121" s="29" t="str">
         <v>Text or notes</v>
@@ -13561,7 +13579,7 @@
     <row r="122" ht="34" customHeight="1">
       <c r="A122" s="3"/>
       <c r="B122" s="29" t="str">
-        <v>Olfactory hallucination details</v>
+        <v>Impact of olfactory hallucinations</v>
       </c>
       <c r="C122" s="29" t="str">
         <v>Text or notes</v>
@@ -13574,7 +13592,7 @@
     <row r="123" ht="34" customHeight="1">
       <c r="A123" s="3"/>
       <c r="B123" s="29" t="str">
-        <v>Impact of olfactory hallucinations</v>
+        <v>Tactile hallucinations</v>
       </c>
       <c r="C123" s="29" t="str">
         <v>Text or notes</v>
@@ -13587,7 +13605,7 @@
     <row r="124" ht="34" customHeight="1">
       <c r="A124" s="3"/>
       <c r="B124" s="29" t="str">
-        <v>Tactile hallucinations</v>
+        <v>Tactile hallucination details</v>
       </c>
       <c r="C124" s="29" t="str">
         <v>Text or notes</v>
@@ -13600,7 +13618,7 @@
     <row r="125" ht="34" customHeight="1">
       <c r="A125" s="3"/>
       <c r="B125" s="29" t="str">
-        <v>Tactile hallucination details</v>
+        <v>Tactile hallucination frequency</v>
       </c>
       <c r="C125" s="29" t="str">
         <v>Text or notes</v>
@@ -13613,7 +13631,7 @@
     <row r="126" ht="34" customHeight="1">
       <c r="A126" s="3"/>
       <c r="B126" s="29" t="str">
-        <v>Tactile hallucination frequency</v>
+        <v>Gustatory hallucinations</v>
       </c>
       <c r="C126" s="29" t="str">
         <v>Text or notes</v>
@@ -13626,7 +13644,7 @@
     <row r="127" ht="34" customHeight="1">
       <c r="A127" s="3"/>
       <c r="B127" s="29" t="str">
-        <v>Gustatory hallucinations</v>
+        <v>Gustatory hallucination details</v>
       </c>
       <c r="C127" s="29" t="str">
         <v>Text or notes</v>
@@ -13639,7 +13657,7 @@
     <row r="128" ht="34" customHeight="1">
       <c r="A128" s="3"/>
       <c r="B128" s="29" t="str">
-        <v>Gustatory hallucination details</v>
+        <v>Hallucination coping strategies</v>
       </c>
       <c r="C128" s="29" t="str">
         <v>Text or notes</v>
@@ -13652,7 +13670,7 @@
     <row r="129" ht="34" customHeight="1">
       <c r="A129" s="3"/>
       <c r="B129" s="29" t="str">
-        <v>Hallucination coping strategies</v>
+        <v>Hallucination distress or impairment</v>
       </c>
       <c r="C129" s="29" t="str">
         <v>Text or notes</v>
@@ -13665,7 +13683,7 @@
     <row r="130" ht="34" customHeight="1">
       <c r="A130" s="3"/>
       <c r="B130" s="29" t="str">
-        <v>Hallucination distress or impairment</v>
+        <v>Impact on daily functioning</v>
       </c>
       <c r="C130" s="29" t="str">
         <v>Text or notes</v>
@@ -13678,7 +13696,7 @@
     <row r="131" ht="34" customHeight="1">
       <c r="A131" s="3"/>
       <c r="B131" s="29" t="str">
-        <v>Impact on daily functioning</v>
+        <v>Professional discussion and treatment</v>
       </c>
       <c r="C131" s="29" t="str">
         <v>Text or notes</v>
@@ -13691,23 +13709,23 @@
     <row r="132" ht="34" customHeight="1">
       <c r="A132" s="3"/>
       <c r="B132" s="29" t="str">
-        <v>Professional discussion and treatment</v>
+        <v>Conserved status</v>
       </c>
       <c r="C132" s="29" t="str">
-        <v>Text or notes</v>
+        <v>LPS; TCon; Murphy's; Non-Conserved</v>
       </c>
       <c r="D132" s="29" t="str">
-        <v>09 Safety and support</v>
+        <v>10 Decisions and legal support</v>
       </c>
       <c r="E132" s="3"/>
     </row>
     <row r="133" ht="34" customHeight="1">
       <c r="A133" s="3"/>
       <c r="B133" s="29" t="str">
-        <v>Conserved status</v>
+        <v>Conservator name</v>
       </c>
       <c r="C133" s="29" t="str">
-        <v>LPS; TCon; Murphy's; Non-Conserved</v>
+        <v>Text or notes</v>
       </c>
       <c r="D133" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13717,7 +13735,7 @@
     <row r="134" ht="34" customHeight="1">
       <c r="A134" s="3"/>
       <c r="B134" s="29" t="str">
-        <v>Conservator name</v>
+        <v>Conservatorship details</v>
       </c>
       <c r="C134" s="29" t="str">
         <v>Text or notes</v>
@@ -13730,7 +13748,7 @@
     <row r="135" ht="34" customHeight="1">
       <c r="A135" s="3"/>
       <c r="B135" s="29" t="str">
-        <v>Conservatorship details</v>
+        <v>Hold type</v>
       </c>
       <c r="C135" s="29" t="str">
         <v>Text or notes</v>
@@ -13743,7 +13761,7 @@
     <row r="136" ht="34" customHeight="1">
       <c r="A136" s="3"/>
       <c r="B136" s="29" t="str">
-        <v>Hold type</v>
+        <v>Forensic history</v>
       </c>
       <c r="C136" s="29" t="str">
         <v>Text or notes</v>
@@ -13756,10 +13774,10 @@
     <row r="137" ht="34" customHeight="1">
       <c r="A137" s="3"/>
       <c r="B137" s="29" t="str">
-        <v>Forensic history</v>
+        <v>Forensic timeline</v>
       </c>
       <c r="C137" s="29" t="str">
-        <v>Text or notes</v>
+        <v>One item per line</v>
       </c>
       <c r="D137" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13769,10 +13787,10 @@
     <row r="138" ht="34" customHeight="1">
       <c r="A138" s="3"/>
       <c r="B138" s="29" t="str">
-        <v>Forensic timeline</v>
+        <v>PC 290 registration</v>
       </c>
       <c r="C138" s="29" t="str">
-        <v>One item per line</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D138" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13782,7 +13800,7 @@
     <row r="139" ht="34" customHeight="1">
       <c r="A139" s="3"/>
       <c r="B139" s="29" t="str">
-        <v>PC 290 registration</v>
+        <v>Arson history</v>
       </c>
       <c r="C139" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13795,7 +13813,7 @@
     <row r="140" ht="34" customHeight="1">
       <c r="A140" s="3"/>
       <c r="B140" s="29" t="str">
-        <v>Arson history</v>
+        <v>Diversion client</v>
       </c>
       <c r="C140" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13808,10 +13826,10 @@
     <row r="141" ht="34" customHeight="1">
       <c r="A141" s="3"/>
       <c r="B141" s="29" t="str">
-        <v>Diversion client</v>
+        <v>Court requirements</v>
       </c>
       <c r="C141" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D141" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13821,7 +13839,7 @@
     <row r="142" ht="34" customHeight="1">
       <c r="A142" s="3"/>
       <c r="B142" s="29" t="str">
-        <v>Court requirements</v>
+        <v>Court dates</v>
       </c>
       <c r="C142" s="29" t="str">
         <v>Text or notes</v>
@@ -13834,7 +13852,7 @@
     <row r="143" ht="34" customHeight="1">
       <c r="A143" s="3"/>
       <c r="B143" s="29" t="str">
-        <v>Court dates</v>
+        <v>Probation / parole / justice</v>
       </c>
       <c r="C143" s="29" t="str">
         <v>Text or notes</v>
@@ -13847,7 +13865,7 @@
     <row r="144" ht="34" customHeight="1">
       <c r="A144" s="3"/>
       <c r="B144" s="29" t="str">
-        <v>Probation / parole / justice</v>
+        <v>Forensic involvement</v>
       </c>
       <c r="C144" s="29" t="str">
         <v>Text or notes</v>
@@ -13860,7 +13878,7 @@
     <row r="145" ht="34" customHeight="1">
       <c r="A145" s="3"/>
       <c r="B145" s="29" t="str">
-        <v>Forensic involvement</v>
+        <v>Forensic involvement details</v>
       </c>
       <c r="C145" s="29" t="str">
         <v>Text or notes</v>
@@ -13873,7 +13891,7 @@
     <row r="146" ht="34" customHeight="1">
       <c r="A146" s="3"/>
       <c r="B146" s="29" t="str">
-        <v>Forensic involvement details</v>
+        <v>History of arrest</v>
       </c>
       <c r="C146" s="29" t="str">
         <v>Text or notes</v>
@@ -13886,10 +13904,10 @@
     <row r="147" ht="34" customHeight="1">
       <c r="A147" s="3"/>
       <c r="B147" s="29" t="str">
-        <v>History of arrest</v>
+        <v>Most recent arrest date</v>
       </c>
       <c r="C147" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D147" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13899,10 +13917,10 @@
     <row r="148" ht="34" customHeight="1">
       <c r="A148" s="3"/>
       <c r="B148" s="29" t="str">
-        <v>Most recent arrest date</v>
+        <v>Most recent arrest charge</v>
       </c>
       <c r="C148" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D148" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13912,7 +13930,7 @@
     <row r="149" ht="34" customHeight="1">
       <c r="A149" s="3"/>
       <c r="B149" s="29" t="str">
-        <v>Most recent arrest charge</v>
+        <v>Time in jail</v>
       </c>
       <c r="C149" s="29" t="str">
         <v>Text or notes</v>
@@ -13925,7 +13943,7 @@
     <row r="150" ht="34" customHeight="1">
       <c r="A150" s="3"/>
       <c r="B150" s="29" t="str">
-        <v>Time in jail</v>
+        <v>Arrest in the last two years</v>
       </c>
       <c r="C150" s="29" t="str">
         <v>Text or notes</v>
@@ -13938,7 +13956,7 @@
     <row r="151" ht="34" customHeight="1">
       <c r="A151" s="3"/>
       <c r="B151" s="29" t="str">
-        <v>Arrest in the last two years</v>
+        <v>Recent arrest details</v>
       </c>
       <c r="C151" s="29" t="str">
         <v>Text or notes</v>
@@ -13951,10 +13969,10 @@
     <row r="152" ht="34" customHeight="1">
       <c r="A152" s="3"/>
       <c r="B152" s="29" t="str">
-        <v>Recent arrest details</v>
+        <v>Total recorded arrests</v>
       </c>
       <c r="C152" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D152" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13964,20 +13982,20 @@
     <row r="153" ht="34" customHeight="1">
       <c r="A153" s="3"/>
       <c r="B153" s="29" t="str">
-        <v>Total recorded arrests</v>
+        <v>Family involvement</v>
       </c>
       <c r="C153" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D153" s="29" t="str">
-        <v>10 Decisions and legal support</v>
+        <v>11 What matters next</v>
       </c>
       <c r="E153" s="3"/>
     </row>
     <row r="154" ht="34" customHeight="1">
       <c r="A154" s="3"/>
       <c r="B154" s="29" t="str">
-        <v>Family involvement</v>
+        <v>Friendships and social connections</v>
       </c>
       <c r="C154" s="29" t="str">
         <v>Text or notes</v>
@@ -13990,7 +14008,7 @@
     <row r="155" ht="34" customHeight="1">
       <c r="A155" s="3"/>
       <c r="B155" s="29" t="str">
-        <v>Friendships and social connections</v>
+        <v>Home and housing history</v>
       </c>
       <c r="C155" s="29" t="str">
         <v>Text or notes</v>
@@ -14003,7 +14021,7 @@
     <row r="156" ht="34" customHeight="1">
       <c r="A156" s="3"/>
       <c r="B156" s="29" t="str">
-        <v>Prior living situation</v>
+        <v>Benefits / income status</v>
       </c>
       <c r="C156" s="29" t="str">
         <v>Text or notes</v>
@@ -14016,7 +14034,7 @@
     <row r="157" ht="34" customHeight="1">
       <c r="A157" s="3"/>
       <c r="B157" s="29" t="str">
-        <v>Housing history</v>
+        <v>Preferred facility characteristics</v>
       </c>
       <c r="C157" s="29" t="str">
         <v>Text or notes</v>
@@ -14029,7 +14047,7 @@
     <row r="158" ht="34" customHeight="1">
       <c r="A158" s="3"/>
       <c r="B158" s="29" t="str">
-        <v>Benefits / income status</v>
+        <v>Discharge planning goals</v>
       </c>
       <c r="C158" s="29" t="str">
         <v>Text or notes</v>
@@ -14042,7 +14060,7 @@
     <row r="159" ht="34" customHeight="1">
       <c r="A159" s="3"/>
       <c r="B159" s="29" t="str">
-        <v>Preferred facility characteristics</v>
+        <v>Placement preferences and concerns</v>
       </c>
       <c r="C159" s="29" t="str">
         <v>Text or notes</v>
@@ -14055,33 +14073,33 @@
     <row r="160" ht="34" customHeight="1">
       <c r="A160" s="3"/>
       <c r="B160" s="29" t="str">
-        <v>Discharge planning goals</v>
+        <v>Additional information</v>
       </c>
       <c r="C160" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D160" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>12 Anything else</v>
       </c>
       <c r="E160" s="3"/>
     </row>
     <row r="161" ht="34" customHeight="1">
       <c r="A161" s="3"/>
       <c r="B161" s="29" t="str">
-        <v>Placement preferences and concerns</v>
+        <v>Placement questions or concerns</v>
       </c>
       <c r="C161" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D161" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>12 Anything else</v>
       </c>
       <c r="E161" s="3"/>
     </row>
     <row r="162" ht="34" customHeight="1">
       <c r="A162" s="3"/>
       <c r="B162" s="29" t="str">
-        <v>Additional information</v>
+        <v>Assessment notes</v>
       </c>
       <c r="C162" s="29" t="str">
         <v>Text or notes</v>
@@ -14091,30 +14109,18 @@
       </c>
       <c r="E162" s="3"/>
     </row>
-    <row r="163" ht="34" customHeight="1">
+    <row r="163">
       <c r="A163" s="3"/>
-      <c r="B163" s="29" t="str">
-        <v>Placement questions or concerns</v>
-      </c>
-      <c r="C163" s="29" t="str">
-        <v>Text or notes</v>
-      </c>
-      <c r="D163" s="29" t="str">
-        <v>12 Anything else</v>
-      </c>
+      <c r="B163" s="3"/>
+      <c r="C163" s="3"/>
+      <c r="D163" s="3"/>
       <c r="E163" s="3"/>
     </row>
-    <row r="164" ht="34" customHeight="1">
+    <row r="164">
       <c r="A164" s="3"/>
-      <c r="B164" s="29" t="str">
-        <v>Assessment notes</v>
-      </c>
-      <c r="C164" s="29" t="str">
-        <v>Text or notes</v>
-      </c>
-      <c r="D164" s="29" t="str">
-        <v>12 Anything else</v>
-      </c>
+      <c r="B164" s="3"/>
+      <c r="C164" s="3"/>
+      <c r="D164" s="3"/>
       <c r="E164" s="3"/>
     </row>
     <row r="165">
@@ -14342,7 +14348,7 @@
         <v>current_location</v>
       </c>
       <c r="B13" s="13" t="str">
-        <v>Current location</v>
+        <v>Where the client is now</v>
       </c>
       <c r="C13" t="str" s="50"/>
       <c r="D13" t="str" s="48"/>
@@ -16832,7 +16838,7 @@
         <v>Not applicable</v>
       </c>
     </row>
-    <row r="10" ht="72" customHeight="1">
+    <row r="10" ht="75" customHeight="1">
       <c r="A10" s="3" t="str">
         <v>medications_at_intake</v>
       </c>
@@ -16853,15 +16859,16 @@
               <color rgb="FF59675F"/>
             </rPr>
             <t xml:space="preserve">
-Enter one medication per line.</t>
+Earlier entered medication history. Attach the current medication list in Files for the community handoff.
+Reference only.</t>
           </r>
         </is>
       </c>
-      <c r="C10" t="str" s="50"/>
-      <c r="D10" t="str" s="48"/>
+      <c r="C10" s="23" t="str"/>
+      <c r="D10" s="15" t="str"/>
       <c r="E10" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C10&amp;""&amp;C11&amp;""&amp;C12&amp;""&amp;C13&amp;""&amp;C14&amp;""&amp;C15&amp;""&amp;C16&amp;""&amp;C17&amp;""&amp;C18&amp;""&amp;C19&amp;""&amp;C20&amp;""&amp;C21&amp;""&amp;C22&amp;""&amp;C23))&gt;0,LEN(TRIM(D10))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D10))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D10))&gt;0)),"Explain why",IF(LEN(TRIM(C10&amp;""&amp;C11&amp;""&amp;C12&amp;""&amp;C13&amp;""&amp;C14&amp;""&amp;C15&amp;""&amp;C16&amp;""&amp;C17&amp;""&amp;C18&amp;""&amp;C19&amp;""&amp;C20&amp;""&amp;C21&amp;""&amp;C22&amp;""&amp;C23))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
+        <f>"Reference only"</f>
+        <v>Reference only</v>
       </c>
     </row>
     <row r="11" ht="88" customHeight="1" hidden="1">
@@ -16871,7 +16878,7 @@
       <c r="B11" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C11" t="str" s="57"/>
+      <c r="C11" s="24" t="str"/>
       <c r="D11" s="3" t="str"/>
       <c r="E11" s="3"/>
     </row>
@@ -16882,7 +16889,7 @@
       <c r="B12" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C12" t="str" s="57"/>
+      <c r="C12" s="24" t="str"/>
       <c r="D12" s="3" t="str"/>
       <c r="E12" s="3"/>
     </row>
@@ -16893,7 +16900,7 @@
       <c r="B13" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C13" t="str" s="57"/>
+      <c r="C13" s="24" t="str"/>
       <c r="D13" s="3" t="str"/>
       <c r="E13" s="3"/>
     </row>
@@ -16904,7 +16911,7 @@
       <c r="B14" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C14" t="str" s="57"/>
+      <c r="C14" s="24" t="str"/>
       <c r="D14" s="3" t="str"/>
       <c r="E14" s="3"/>
     </row>
@@ -16915,7 +16922,7 @@
       <c r="B15" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C15" t="str" s="57"/>
+      <c r="C15" s="24" t="str"/>
       <c r="D15" s="3" t="str"/>
       <c r="E15" s="3"/>
     </row>
@@ -16926,7 +16933,7 @@
       <c r="B16" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C16" t="str" s="57"/>
+      <c r="C16" s="24" t="str"/>
       <c r="D16" s="3" t="str"/>
       <c r="E16" s="3"/>
     </row>
@@ -16937,7 +16944,7 @@
       <c r="B17" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C17" t="str" s="57"/>
+      <c r="C17" s="24" t="str"/>
       <c r="D17" s="3" t="str"/>
       <c r="E17" s="3"/>
     </row>
@@ -16948,7 +16955,7 @@
       <c r="B18" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C18" t="str" s="57"/>
+      <c r="C18" s="24" t="str"/>
       <c r="D18" s="3" t="str"/>
       <c r="E18" s="3"/>
     </row>
@@ -16959,7 +16966,7 @@
       <c r="B19" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C19" t="str" s="57"/>
+      <c r="C19" s="24" t="str"/>
       <c r="D19" s="3" t="str"/>
       <c r="E19" s="3"/>
     </row>
@@ -16970,7 +16977,7 @@
       <c r="B20" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C20" t="str" s="57"/>
+      <c r="C20" s="24" t="str"/>
       <c r="D20" s="3" t="str"/>
       <c r="E20" s="3"/>
     </row>
@@ -16981,7 +16988,7 @@
       <c r="B21" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C21" t="str" s="57"/>
+      <c r="C21" s="24" t="str"/>
       <c r="D21" s="3" t="str"/>
       <c r="E21" s="3"/>
     </row>
@@ -16992,7 +16999,7 @@
       <c r="B22" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C22" t="str" s="57"/>
+      <c r="C22" s="24" t="str"/>
       <c r="D22" s="3" t="str"/>
       <c r="E22" s="3"/>
     </row>
@@ -17003,7 +17010,7 @@
       <c r="B23" s="3" t="str">
         <v>Medications at intake (continued)</v>
       </c>
-      <c r="C23" t="str" s="57"/>
+      <c r="C23" s="24" t="str"/>
       <c r="D23" s="3" t="str"/>
       <c r="E23" s="3"/>
     </row>
@@ -17417,12 +17424,30 @@
         <v>Optional</v>
       </c>
     </row>
-    <row r="7" ht="34" customHeight="1">
+    <row r="7" ht="51" customHeight="1">
       <c r="A7" s="3" t="str">
         <v>prior_setting_bucket</v>
       </c>
-      <c r="B7" s="13" t="str">
-        <v>Prior setting type</v>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="12"/>
+              <color rgb="FF233B32"/>
+            </rPr>
+            <t>Most recent setting type</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="0"/>
+              <sz val="10"/>
+              <color rgb="FF59675F"/>
+            </rPr>
+            <t xml:space="preserve">
+Choose the setting the client is coming from for this referral.</t>
+          </r>
+        </is>
       </c>
       <c r="C7" t="str" s="50"/>
       <c r="D7" t="str" s="48"/>
@@ -17436,7 +17461,7 @@
         <v>referring_facility</v>
       </c>
       <c r="B8" s="13" t="str">
-        <v>Prior placement name</v>
+        <v>Most recent facility or program</v>
       </c>
       <c r="C8" t="str" s="50"/>
       <c r="D8" t="str" s="48"/>
@@ -17590,7 +17615,7 @@
         <v>prior_placements</v>
       </c>
       <c r="B6" s="13" t="str">
-        <v>Prior placements</v>
+        <v>Earlier care placements</v>
       </c>
       <c r="C6" t="str" s="50"/>
       <c r="D6" t="str" s="48"/>

</xml_diff>

<commit_message>
Consolidate repeated assessment history and placement prompts
(cherry picked from commit 8ace96ccb9d6358dbe2e0e85762a41c861bd95c9)
</commit_message>
<xml_diff>
--- a/public/templates/pipeline-assessment-workbook.xlsx
+++ b/public/templates/pipeline-assessment-workbook.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rea505e774e45403c"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="R0c0157dd3bfb4404"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R613c4939346946e5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="Rd4cdafd37d674dcc"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Re49e3869eecc4849"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="Ra7a741e3af554825"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="Rb6f7ae69db834e53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="R229fa0a170c64755"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="R31a37d5ce5d14959"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R1110fc44b1e94567"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="R01ce2b7e25c84ec2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R8e7cbcc449b04976"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="R9cae6c060a474f4f"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="Rb861b1ec397245fa" state="veryHidden"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="R9b58ee9f9cd34eaa"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Re56b9b25da424454"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="Rb8877295a23342e9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R5792cea647164f84"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="R8adede638d3b48a0"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Recf645d799044eef"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="R7f05fc8c83b04708"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="Re5e59df1ad974e31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="Rb4d5de57739849d5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Rb6ac36abfee240bb"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R5f1f749efc254059"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="R01d5c1a26d264a9e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R9e31f31815b14ef9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="R8b6b6ea4958b4d38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="R5748b07ebda94d82" state="veryHidden"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="R99a8451577a8493e"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Confirm the basics'!$B$1:$E$16</definedName>
@@ -3524,6 +3524,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF233B32"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF6DF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF68756F"/>
       </font>
       <fill>
@@ -3602,16 +3612,6 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFF0CA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF233B32"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF6DF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6362,11 +6362,123 @@
         <v>Optional</v>
       </c>
     </row>
-    <row r="11" ht="72" customHeight="1">
+    <row r="11" ht="34" customHeight="1">
       <c r="A11" s="3" t="str">
+        <v>pc290_registration</v>
+      </c>
+      <c r="B11" s="13" t="str">
+        <v>PC 290 registration</v>
+      </c>
+      <c r="C11" t="str" s="50"/>
+      <c r="D11" t="str" s="48"/>
+      <c r="E11" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C11))&gt;0,LEN(TRIM(D11))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D11))&gt;0,NOT(OR(LOWER(TRIM(C11))="unable to assess",C11="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C11))="unable to assess",C11="unable_to_assess"),NOT(LEN(TRIM(D11))&gt;0)),"Explain why",IF(LEN(TRIM(C11))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
+        <v>Needs answer</v>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="3" t="str">
+        <v>arson_history</v>
+      </c>
+      <c r="B12" s="13" t="str">
+        <v>Arson history</v>
+      </c>
+      <c r="C12" t="str" s="50"/>
+      <c r="D12" t="str" s="48"/>
+      <c r="E12" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C12))&gt;0,LEN(TRIM(D12))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D12))&gt;0,NOT(OR(LOWER(TRIM(C12))="unable to assess",C12="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C12))="unable to assess",C12="unable_to_assess"),NOT(LEN(TRIM(D12))&gt;0)),"Explain why",IF(LEN(TRIM(C12))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
+        <v>Needs answer</v>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="3" t="str">
+        <v>diversion_client</v>
+      </c>
+      <c r="B13" s="13" t="str">
+        <v>Diversion client</v>
+      </c>
+      <c r="C13" t="str" s="50"/>
+      <c r="D13" t="str" s="48"/>
+      <c r="E13" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C13))&gt;0,LEN(TRIM(D13))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D13))&gt;0,NOT(OR(LOWER(TRIM(C13))="unable to assess",C13="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C13))="unable to assess",C13="unable_to_assess"),NOT(LEN(TRIM(D13))&gt;0)),"Explain why",IF(LEN(TRIM(C13))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
+        <v>Needs answer</v>
+      </c>
+    </row>
+    <row r="14" ht="72" customHeight="1">
+      <c r="A14" s="3" t="str">
+        <v>court_requirements</v>
+      </c>
+      <c r="B14" s="13" t="str">
+        <v>Court requirements</v>
+      </c>
+      <c r="C14" t="str" s="50"/>
+      <c r="D14" t="str" s="48"/>
+      <c r="E14" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C14))&gt;0,LEN(TRIM(D14))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D14))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D14))&gt;0)),"Explain why",IF(LEN(TRIM(C14))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="3" t="str">
+        <v>court_dates</v>
+      </c>
+      <c r="B15" s="13" t="str">
+        <v>Court dates</v>
+      </c>
+      <c r="C15" t="str" s="50"/>
+      <c r="D15" t="str" s="48"/>
+      <c r="E15" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C15))&gt;0,LEN(TRIM(D15))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D15))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D15))&gt;0)),"Explain why",IF(LEN(TRIM(C15))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1">
+      <c r="A16" s="3" t="str">
+        <v>probation_parole_justice</v>
+      </c>
+      <c r="B16" s="13" t="str">
+        <v>Probation / parole / justice</v>
+      </c>
+      <c r="C16" t="str" s="50"/>
+      <c r="D16" t="str" s="48"/>
+      <c r="E16" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C16))&gt;0,LEN(TRIM(D16))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D16))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D16))&gt;0)),"Explain why",IF(LEN(TRIM(C16))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="3" t="str">
+        <v>forensic_involvement</v>
+      </c>
+      <c r="B17" s="13" t="str">
+        <v>Forensic involvement</v>
+      </c>
+      <c r="C17" t="str" s="50"/>
+      <c r="D17" t="str" s="48"/>
+      <c r="E17" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C17))&gt;0,LEN(TRIM(D17))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D17))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D17))&gt;0)),"Explain why",IF(LEN(TRIM(C17))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="3" t="str">
+        <v>forensic_involvement_details</v>
+      </c>
+      <c r="B18" s="13" t="str">
+        <v>Forensic involvement details</v>
+      </c>
+      <c r="C18" t="str" s="50"/>
+      <c r="D18" t="str" s="48"/>
+      <c r="E18" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C18))&gt;0,LEN(TRIM(D18))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D18))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D18))&gt;0)),"Explain why",IF(LEN(TRIM(C18))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="19" ht="72" customHeight="1">
+      <c r="A19" s="3" t="str">
         <v>forensic_timeline</v>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -6383,271 +6495,159 @@
               <color rgb="FF59675F"/>
             </rPr>
             <t xml:space="preserve">
-Optional. Record an approximate date, event, and outcome in each row.</t>
+Reference only.</t>
           </r>
         </is>
       </c>
-      <c r="C11" t="str" s="50"/>
-      <c r="D11" t="str" s="48"/>
-      <c r="E11" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C11&amp;""&amp;C12&amp;""&amp;C13&amp;""&amp;C14&amp;""&amp;C15&amp;""&amp;C16&amp;""&amp;C17&amp;""&amp;C18&amp;""&amp;C19&amp;""&amp;C20&amp;""&amp;C21&amp;""&amp;C22&amp;""&amp;C23&amp;""&amp;C24))&gt;0,LEN(TRIM(D11))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D11))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D11))&gt;0)),"Explain why",IF(LEN(TRIM(C11&amp;""&amp;C12&amp;""&amp;C13&amp;""&amp;C14&amp;""&amp;C15&amp;""&amp;C16&amp;""&amp;C17&amp;""&amp;C18&amp;""&amp;C19&amp;""&amp;C20&amp;""&amp;C21&amp;""&amp;C22&amp;""&amp;C23&amp;""&amp;C24))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
-    </row>
-    <row r="12" ht="88" customHeight="1" hidden="1">
-      <c r="A12" s="3" t="str">
-        <v>forensic_timeline:1</v>
-      </c>
-      <c r="B12" s="3" t="str">
-        <v>Forensic timeline (continued)</v>
-      </c>
-      <c r="C12" t="str" s="57"/>
-      <c r="D12" s="3" t="str"/>
-      <c r="E12" s="3"/>
-    </row>
-    <row r="13" ht="88" customHeight="1" hidden="1">
-      <c r="A13" s="3" t="str">
-        <v>forensic_timeline:2</v>
-      </c>
-      <c r="B13" s="3" t="str">
-        <v>Forensic timeline (continued)</v>
-      </c>
-      <c r="C13" t="str" s="57"/>
-      <c r="D13" s="3" t="str"/>
-      <c r="E13" s="3"/>
-    </row>
-    <row r="14" ht="88" customHeight="1" hidden="1">
-      <c r="A14" s="3" t="str">
-        <v>forensic_timeline:3</v>
-      </c>
-      <c r="B14" s="3" t="str">
-        <v>Forensic timeline (continued)</v>
-      </c>
-      <c r="C14" t="str" s="57"/>
-      <c r="D14" s="3" t="str"/>
-      <c r="E14" s="3"/>
-    </row>
-    <row r="15" ht="88" customHeight="1" hidden="1">
-      <c r="A15" s="3" t="str">
-        <v>forensic_timeline:4</v>
-      </c>
-      <c r="B15" s="3" t="str">
-        <v>Forensic timeline (continued)</v>
-      </c>
-      <c r="C15" t="str" s="57"/>
-      <c r="D15" s="3" t="str"/>
-      <c r="E15" s="3"/>
-    </row>
-    <row r="16" ht="88" customHeight="1" hidden="1">
-      <c r="A16" s="3" t="str">
-        <v>forensic_timeline:5</v>
-      </c>
-      <c r="B16" s="3" t="str">
-        <v>Forensic timeline (continued)</v>
-      </c>
-      <c r="C16" t="str" s="57"/>
-      <c r="D16" s="3" t="str"/>
-      <c r="E16" s="3"/>
-    </row>
-    <row r="17" ht="88" customHeight="1" hidden="1">
-      <c r="A17" s="3" t="str">
-        <v>forensic_timeline:6</v>
-      </c>
-      <c r="B17" s="3" t="str">
-        <v>Forensic timeline (continued)</v>
-      </c>
-      <c r="C17" t="str" s="57"/>
-      <c r="D17" s="3" t="str"/>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" ht="88" customHeight="1" hidden="1">
-      <c r="A18" s="3" t="str">
-        <v>forensic_timeline:7</v>
-      </c>
-      <c r="B18" s="3" t="str">
-        <v>Forensic timeline (continued)</v>
-      </c>
-      <c r="C18" t="str" s="57"/>
-      <c r="D18" s="3" t="str"/>
-      <c r="E18" s="3"/>
-    </row>
-    <row r="19" ht="88" customHeight="1" hidden="1">
-      <c r="A19" s="3" t="str">
-        <v>forensic_timeline:8</v>
-      </c>
-      <c r="B19" s="3" t="str">
-        <v>Forensic timeline (continued)</v>
-      </c>
-      <c r="C19" t="str" s="57"/>
-      <c r="D19" s="3" t="str"/>
-      <c r="E19" s="3"/>
+      <c r="C19" s="23" t="str"/>
+      <c r="D19" s="15" t="str"/>
+      <c r="E19" s="16" t="str">
+        <f>"Reference only"</f>
+        <v>Reference only</v>
+      </c>
     </row>
     <row r="20" ht="88" customHeight="1" hidden="1">
       <c r="A20" s="3" t="str">
-        <v>forensic_timeline:9</v>
+        <v>forensic_timeline:1</v>
       </c>
       <c r="B20" s="3" t="str">
         <v>Forensic timeline (continued)</v>
       </c>
-      <c r="C20" t="str" s="57"/>
+      <c r="C20" s="24" t="str"/>
       <c r="D20" s="3" t="str"/>
       <c r="E20" s="3"/>
     </row>
     <row r="21" ht="88" customHeight="1" hidden="1">
       <c r="A21" s="3" t="str">
-        <v>forensic_timeline:10</v>
+        <v>forensic_timeline:2</v>
       </c>
       <c r="B21" s="3" t="str">
         <v>Forensic timeline (continued)</v>
       </c>
-      <c r="C21" t="str" s="57"/>
+      <c r="C21" s="24" t="str"/>
       <c r="D21" s="3" t="str"/>
       <c r="E21" s="3"/>
     </row>
     <row r="22" ht="88" customHeight="1" hidden="1">
       <c r="A22" s="3" t="str">
-        <v>forensic_timeline:11</v>
+        <v>forensic_timeline:3</v>
       </c>
       <c r="B22" s="3" t="str">
         <v>Forensic timeline (continued)</v>
       </c>
-      <c r="C22" t="str" s="57"/>
+      <c r="C22" s="24" t="str"/>
       <c r="D22" s="3" t="str"/>
       <c r="E22" s="3"/>
     </row>
     <row r="23" ht="88" customHeight="1" hidden="1">
       <c r="A23" s="3" t="str">
-        <v>forensic_timeline:12</v>
+        <v>forensic_timeline:4</v>
       </c>
       <c r="B23" s="3" t="str">
         <v>Forensic timeline (continued)</v>
       </c>
-      <c r="C23" t="str" s="57"/>
+      <c r="C23" s="24" t="str"/>
       <c r="D23" s="3" t="str"/>
       <c r="E23" s="3"/>
     </row>
     <row r="24" ht="88" customHeight="1" hidden="1">
       <c r="A24" s="3" t="str">
-        <v>forensic_timeline:13</v>
+        <v>forensic_timeline:5</v>
       </c>
       <c r="B24" s="3" t="str">
         <v>Forensic timeline (continued)</v>
       </c>
-      <c r="C24" t="str" s="57"/>
+      <c r="C24" s="24" t="str"/>
       <c r="D24" s="3" t="str"/>
       <c r="E24" s="3"/>
     </row>
-    <row r="25" ht="34" customHeight="1">
+    <row r="25" ht="88" customHeight="1" hidden="1">
       <c r="A25" s="3" t="str">
-        <v>pc290_registration</v>
-      </c>
-      <c r="B25" s="13" t="str">
-        <v>PC 290 registration</v>
-      </c>
-      <c r="C25" t="str" s="50"/>
-      <c r="D25" t="str" s="48"/>
-      <c r="E25" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C25))&gt;0,LEN(TRIM(D25))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D25))&gt;0,NOT(OR(LOWER(TRIM(C25))="unable to assess",C25="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C25))="unable to assess",C25="unable_to_assess"),NOT(LEN(TRIM(D25))&gt;0)),"Explain why",IF(LEN(TRIM(C25))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
-        <v>Needs answer</v>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
+        <v>forensic_timeline:6</v>
+      </c>
+      <c r="B25" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C25" s="24" t="str"/>
+      <c r="D25" s="3" t="str"/>
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" ht="88" customHeight="1" hidden="1">
       <c r="A26" s="3" t="str">
-        <v>arson_history</v>
-      </c>
-      <c r="B26" s="13" t="str">
-        <v>Arson history</v>
-      </c>
-      <c r="C26" t="str" s="50"/>
-      <c r="D26" t="str" s="48"/>
-      <c r="E26" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C26))&gt;0,LEN(TRIM(D26))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D26))&gt;0,NOT(OR(LOWER(TRIM(C26))="unable to assess",C26="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C26))="unable to assess",C26="unable_to_assess"),NOT(LEN(TRIM(D26))&gt;0)),"Explain why",IF(LEN(TRIM(C26))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
-        <v>Needs answer</v>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
+        <v>forensic_timeline:7</v>
+      </c>
+      <c r="B26" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C26" s="24" t="str"/>
+      <c r="D26" s="3" t="str"/>
+      <c r="E26" s="3"/>
+    </row>
+    <row r="27" ht="88" customHeight="1" hidden="1">
       <c r="A27" s="3" t="str">
-        <v>diversion_client</v>
-      </c>
-      <c r="B27" s="13" t="str">
-        <v>Diversion client</v>
-      </c>
-      <c r="C27" t="str" s="50"/>
-      <c r="D27" t="str" s="48"/>
-      <c r="E27" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C27))&gt;0,LEN(TRIM(D27))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D27))&gt;0,NOT(OR(LOWER(TRIM(C27))="unable to assess",C27="unable_to_assess"))),"Review previous reason",IF(AND(OR(LOWER(TRIM(C27))="unable to assess",C27="unable_to_assess"),NOT(LEN(TRIM(D27))&gt;0)),"Explain why",IF(LEN(TRIM(C27))&gt;0,"Answered",IF(TRUE,"Needs answer","Optional")))))</f>
-        <v>Needs answer</v>
-      </c>
-    </row>
-    <row r="28" ht="72" customHeight="1">
+        <v>forensic_timeline:8</v>
+      </c>
+      <c r="B27" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C27" s="24" t="str"/>
+      <c r="D27" s="3" t="str"/>
+      <c r="E27" s="3"/>
+    </row>
+    <row r="28" ht="88" customHeight="1" hidden="1">
       <c r="A28" s="3" t="str">
-        <v>court_requirements</v>
-      </c>
-      <c r="B28" s="13" t="str">
-        <v>Court requirements</v>
-      </c>
-      <c r="C28" t="str" s="50"/>
-      <c r="D28" t="str" s="48"/>
-      <c r="E28" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C28))&gt;0,LEN(TRIM(D28))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D28))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D28))&gt;0)),"Explain why",IF(LEN(TRIM(C28))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
-    </row>
-    <row r="29" ht="72" customHeight="1">
+        <v>forensic_timeline:9</v>
+      </c>
+      <c r="B28" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C28" s="24" t="str"/>
+      <c r="D28" s="3" t="str"/>
+      <c r="E28" s="3"/>
+    </row>
+    <row r="29" ht="88" customHeight="1" hidden="1">
       <c r="A29" s="3" t="str">
-        <v>court_dates</v>
-      </c>
-      <c r="B29" s="13" t="str">
-        <v>Court dates</v>
-      </c>
-      <c r="C29" t="str" s="50"/>
-      <c r="D29" t="str" s="48"/>
-      <c r="E29" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C29))&gt;0,LEN(TRIM(D29))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D29))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D29))&gt;0)),"Explain why",IF(LEN(TRIM(C29))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
-    </row>
-    <row r="30" ht="72" customHeight="1">
+        <v>forensic_timeline:10</v>
+      </c>
+      <c r="B29" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C29" s="24" t="str"/>
+      <c r="D29" s="3" t="str"/>
+      <c r="E29" s="3"/>
+    </row>
+    <row r="30" ht="88" customHeight="1" hidden="1">
       <c r="A30" s="3" t="str">
-        <v>probation_parole_justice</v>
-      </c>
-      <c r="B30" s="13" t="str">
-        <v>Probation / parole / justice</v>
-      </c>
-      <c r="C30" t="str" s="50"/>
-      <c r="D30" t="str" s="48"/>
-      <c r="E30" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C30))&gt;0,LEN(TRIM(D30))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D30))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D30))&gt;0)),"Explain why",IF(LEN(TRIM(C30))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
-    </row>
-    <row r="31" ht="34" customHeight="1">
+        <v>forensic_timeline:11</v>
+      </c>
+      <c r="B30" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C30" s="24" t="str"/>
+      <c r="D30" s="3" t="str"/>
+      <c r="E30" s="3"/>
+    </row>
+    <row r="31" ht="88" customHeight="1" hidden="1">
       <c r="A31" s="3" t="str">
-        <v>forensic_involvement</v>
-      </c>
-      <c r="B31" s="13" t="str">
-        <v>Forensic involvement</v>
-      </c>
-      <c r="C31" t="str" s="50"/>
-      <c r="D31" t="str" s="48"/>
-      <c r="E31" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C31))&gt;0,LEN(TRIM(D31))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D31))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D31))&gt;0)),"Explain why",IF(LEN(TRIM(C31))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
-    </row>
-    <row r="32" ht="34" customHeight="1">
+        <v>forensic_timeline:12</v>
+      </c>
+      <c r="B31" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C31" s="24" t="str"/>
+      <c r="D31" s="3" t="str"/>
+      <c r="E31" s="3"/>
+    </row>
+    <row r="32" ht="88" customHeight="1" hidden="1">
       <c r="A32" s="3" t="str">
-        <v>forensic_involvement_details</v>
-      </c>
-      <c r="B32" s="13" t="str">
-        <v>Forensic involvement details</v>
-      </c>
-      <c r="C32" t="str" s="50"/>
-      <c r="D32" t="str" s="48"/>
-      <c r="E32" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C32))&gt;0,LEN(TRIM(D32))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D32))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D32))&gt;0)),"Explain why",IF(LEN(TRIM(C32))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
+        <v>forensic_timeline:13</v>
+      </c>
+      <c r="B32" s="3" t="str">
+        <v>Forensic timeline (continued)</v>
+      </c>
+      <c r="C32" s="24" t="str"/>
+      <c r="D32" s="3" t="str"/>
+      <c r="E32" s="3"/>
     </row>
     <row r="33" ht="34" customHeight="1">
       <c r="A33" s="3" t="str">
@@ -6815,99 +6815,99 @@
       <formula>OR($E11="Needs answer",$E11="Explain why",LEFT($E11,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B25:E25">
+  <conditionalFormatting sqref="D11:D11">
     <cfRule type="expression" dxfId="299" priority="13">
-      <formula>$E25="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E25:E25">
+      <formula>OR($C11="Unable to assess",$C11="unable_to_assess")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B12:E12">
     <cfRule type="expression" dxfId="300" priority="14">
-      <formula>OR($E25="Needs answer",$E25="Explain why",LEFT($E25,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D25:D25">
+      <formula>$E12="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12:E12">
     <cfRule type="expression" dxfId="301" priority="15">
-      <formula>OR($C25="Unable to assess",$C25="unable_to_assess")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B26:E26">
+      <formula>OR($E12="Needs answer",$E12="Explain why",LEFT($E12,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12:D12">
     <cfRule type="expression" dxfId="302" priority="16">
-      <formula>$E26="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E26:E26">
+      <formula>OR($C12="Unable to assess",$C12="unable_to_assess")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B13:E13">
     <cfRule type="expression" dxfId="303" priority="17">
-      <formula>OR($E26="Needs answer",$E26="Explain why",LEFT($E26,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D26:D26">
+      <formula>$E13="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E13:E13">
     <cfRule type="expression" dxfId="304" priority="18">
-      <formula>OR($C26="Unable to assess",$C26="unable_to_assess")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B27:E27">
+      <formula>OR($E13="Needs answer",$E13="Explain why",LEFT($E13,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D13:D13">
     <cfRule type="expression" dxfId="305" priority="19">
-      <formula>$E27="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E27:E27">
+      <formula>OR($C13="Unable to assess",$C13="unable_to_assess")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B14:E14">
     <cfRule type="expression" dxfId="306" priority="20">
-      <formula>OR($E27="Needs answer",$E27="Explain why",LEFT($E27,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D27:D27">
+      <formula>$E14="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E14:E14">
     <cfRule type="expression" dxfId="307" priority="21">
-      <formula>OR($C27="Unable to assess",$C27="unable_to_assess")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B28:E28">
+      <formula>OR($E14="Needs answer",$E14="Explain why",LEFT($E14,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15:E15">
     <cfRule type="expression" dxfId="308" priority="22">
-      <formula>$E28="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E28:E28">
+      <formula>$E15="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E15:E15">
     <cfRule type="expression" dxfId="309" priority="23">
-      <formula>OR($E28="Needs answer",$E28="Explain why",LEFT($E28,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B29:E29">
+      <formula>OR($E15="Needs answer",$E15="Explain why",LEFT($E15,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16:E16">
     <cfRule type="expression" dxfId="310" priority="24">
-      <formula>$E29="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E29:E29">
+      <formula>$E16="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E16:E16">
     <cfRule type="expression" dxfId="311" priority="25">
-      <formula>OR($E29="Needs answer",$E29="Explain why",LEFT($E29,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B30:E30">
+      <formula>OR($E16="Needs answer",$E16="Explain why",LEFT($E16,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B17:E17">
     <cfRule type="expression" dxfId="312" priority="26">
-      <formula>$E30="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E30:E30">
+      <formula>$E17="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E17:E17">
     <cfRule type="expression" dxfId="313" priority="27">
-      <formula>OR($E30="Needs answer",$E30="Explain why",LEFT($E30,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B31:E31">
+      <formula>OR($E17="Needs answer",$E17="Explain why",LEFT($E17,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18:E18">
     <cfRule type="expression" dxfId="314" priority="28">
-      <formula>$E31="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E31:E31">
+      <formula>$E18="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E18:E18">
     <cfRule type="expression" dxfId="315" priority="29">
-      <formula>OR($E31="Needs answer",$E31="Explain why",LEFT($E31,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B32:E32">
+      <formula>OR($E18="Needs answer",$E18="Explain why",LEFT($E18,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19:E19">
     <cfRule type="expression" dxfId="316" priority="30">
-      <formula>$E32="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E32:E32">
+      <formula>$E19="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E19:E19">
     <cfRule type="expression" dxfId="317" priority="31">
-      <formula>OR($E32="Needs answer",$E32="Explain why",LEFT($E32,6)="Review")</formula>
+      <formula>OR($E19="Needs answer",$E19="Explain why",LEFT($E19,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33:E33">
@@ -6984,13 +6984,13 @@
     <dataValidation type="list" sqref="C6">
       <formula1>"LPS,TCon,Murphy's,Non-Conserved"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C25">
+    <dataValidation type="list" sqref="C11">
       <formula1>"Yes,No,Unable to assess"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C26">
+    <dataValidation type="list" sqref="C12">
       <formula1>"Yes,No,Unable to assess"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="C27">
+    <dataValidation type="list" sqref="C13">
       <formula1>"Yes,No,Unable to assess"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7157,10 +7157,10 @@
     </row>
     <row r="11" ht="72" customHeight="1">
       <c r="A11" s="3" t="str">
-        <v>preferred_facility_characteristics</v>
+        <v>discharge_planning_goals</v>
       </c>
       <c r="B11" s="13" t="str">
-        <v>Preferred facility characteristics</v>
+        <v>Discharge planning goals</v>
       </c>
       <c r="C11" t="str" s="50"/>
       <c r="D11" t="str" s="48"/>
@@ -7171,10 +7171,10 @@
     </row>
     <row r="12" ht="72" customHeight="1">
       <c r="A12" s="3" t="str">
-        <v>discharge_planning_goals</v>
+        <v>placement_preferences_concerns</v>
       </c>
       <c r="B12" s="13" t="str">
-        <v>Discharge planning goals</v>
+        <v>Placement preferences and concerns</v>
       </c>
       <c r="C12" t="str" s="50"/>
       <c r="D12" t="str" s="48"/>
@@ -7183,18 +7183,36 @@
         <v>Optional</v>
       </c>
     </row>
-    <row r="13" ht="72" customHeight="1">
+    <row r="13" ht="54" customHeight="1">
       <c r="A13" s="3" t="str">
-        <v>placement_preferences_concerns</v>
-      </c>
-      <c r="B13" s="13" t="str">
-        <v>Placement preferences and concerns</v>
-      </c>
-      <c r="C13" t="str" s="50"/>
-      <c r="D13" t="str" s="48"/>
+        <v>preferred_facility_characteristics</v>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="12"/>
+              <color rgb="FF233B32"/>
+            </rPr>
+            <t>Preferred facility characteristics</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="0"/>
+              <sz val="10"/>
+              <color rgb="FF59675F"/>
+            </rPr>
+            <t xml:space="preserve">
+Reference only.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C13" s="23" t="str"/>
+      <c r="D13" s="15" t="str"/>
       <c r="E13" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C13))&gt;0,LEN(TRIM(D13))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D13))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D13))&gt;0)),"Explain why",IF(LEN(TRIM(C13))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
+        <f>"Reference only"</f>
+        <v>Reference only</v>
       </c>
     </row>
   </sheetData>
@@ -8007,7 +8025,7 @@
         <v>Questionnaire fingerprint</v>
       </c>
       <c r="B2" t="str">
-        <v>a411199d0450c15c3e8fce1cba5e44bb4ace2fe3931c189ead5e4f7a7bec55c7</v>
+        <v>d01f4e8eb2fa55dffca35c74bf99212eef02e9d6e83b2b40d0e5de806481fee8</v>
       </c>
     </row>
     <row r="3">
@@ -9890,7 +9908,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>hospitalization_timeline</v>
+        <v>prior_hospitalizations_count</v>
       </c>
       <c r="B84" t="str">
         <v>07 Recent care and history!C9</v>
@@ -9914,10 +9932,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>prior_hospitalizations_count</v>
+        <v>most_recent_hospitalization</v>
       </c>
       <c r="B85" t="str">
-        <v>07 Recent care and history!C23</v>
+        <v>07 Recent care and history!C10</v>
       </c>
       <c r="C85" t="str"/>
       <c r="D85" t="str"/>
@@ -9938,10 +9956,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>most_recent_hospitalization</v>
+        <v>prior_5150_5250_holds</v>
       </c>
       <c r="B86" t="str">
-        <v>07 Recent care and history!C24</v>
+        <v>07 Recent care and history!C11</v>
       </c>
       <c r="C86" t="str"/>
       <c r="D86" t="str"/>
@@ -9962,10 +9980,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>prior_5150_5250_holds</v>
+        <v>hospitalization_timeline</v>
       </c>
       <c r="B87" t="str">
-        <v>07 Recent care and history!C25</v>
+        <v>07 Recent care and history!C12</v>
       </c>
       <c r="C87" t="str"/>
       <c r="D87" t="str"/>
@@ -11258,7 +11276,7 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>forensic_timeline</v>
+        <v>pc290_registration</v>
       </c>
       <c r="B141" t="str">
         <v>10 Decisions and legal support!C11</v>
@@ -11282,10 +11300,10 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>pc290_registration</v>
+        <v>arson_history</v>
       </c>
       <c r="B142" t="str">
-        <v>10 Decisions and legal support!C25</v>
+        <v>10 Decisions and legal support!C12</v>
       </c>
       <c r="C142" t="str"/>
       <c r="D142" t="str"/>
@@ -11306,10 +11324,10 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>arson_history</v>
+        <v>diversion_client</v>
       </c>
       <c r="B143" t="str">
-        <v>10 Decisions and legal support!C26</v>
+        <v>10 Decisions and legal support!C13</v>
       </c>
       <c r="C143" t="str"/>
       <c r="D143" t="str"/>
@@ -11330,10 +11348,10 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>diversion_client</v>
+        <v>court_requirements</v>
       </c>
       <c r="B144" t="str">
-        <v>10 Decisions and legal support!C27</v>
+        <v>10 Decisions and legal support!C14</v>
       </c>
       <c r="C144" t="str"/>
       <c r="D144" t="str"/>
@@ -11354,10 +11372,10 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>court_requirements</v>
+        <v>court_dates</v>
       </c>
       <c r="B145" t="str">
-        <v>10 Decisions and legal support!C28</v>
+        <v>10 Decisions and legal support!C15</v>
       </c>
       <c r="C145" t="str"/>
       <c r="D145" t="str"/>
@@ -11378,10 +11396,10 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>court_dates</v>
+        <v>probation_parole_justice</v>
       </c>
       <c r="B146" t="str">
-        <v>10 Decisions and legal support!C29</v>
+        <v>10 Decisions and legal support!C16</v>
       </c>
       <c r="C146" t="str"/>
       <c r="D146" t="str"/>
@@ -11402,10 +11420,10 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>probation_parole_justice</v>
+        <v>forensic_involvement</v>
       </c>
       <c r="B147" t="str">
-        <v>10 Decisions and legal support!C30</v>
+        <v>10 Decisions and legal support!C17</v>
       </c>
       <c r="C147" t="str"/>
       <c r="D147" t="str"/>
@@ -11426,10 +11444,10 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>forensic_involvement</v>
+        <v>forensic_involvement_details</v>
       </c>
       <c r="B148" t="str">
-        <v>10 Decisions and legal support!C31</v>
+        <v>10 Decisions and legal support!C18</v>
       </c>
       <c r="C148" t="str"/>
       <c r="D148" t="str"/>
@@ -11450,10 +11468,10 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>forensic_involvement_details</v>
+        <v>forensic_timeline</v>
       </c>
       <c r="B149" t="str">
-        <v>10 Decisions and legal support!C32</v>
+        <v>10 Decisions and legal support!C19</v>
       </c>
       <c r="C149" t="str"/>
       <c r="D149" t="str"/>
@@ -11762,7 +11780,7 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>preferred_facility_characteristics</v>
+        <v>discharge_planning_goals</v>
       </c>
       <c r="B162" t="str">
         <v>11 What matters next!C11</v>
@@ -11786,7 +11804,7 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>discharge_planning_goals</v>
+        <v>placement_preferences_concerns</v>
       </c>
       <c r="B163" t="str">
         <v>11 What matters next!C12</v>
@@ -11810,7 +11828,7 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>placement_preferences_concerns</v>
+        <v>preferred_facility_characteristics</v>
       </c>
       <c r="B164" t="str">
         <v>11 What matters next!C13</v>
@@ -13033,10 +13051,10 @@
     <row r="80" ht="34" customHeight="1">
       <c r="A80" s="3"/>
       <c r="B80" s="29" t="str">
-        <v>Hospitalization timeline</v>
+        <v>Prior hospitalizations</v>
       </c>
       <c r="C80" s="29" t="str">
-        <v>One item per line</v>
+        <v>Whole number</v>
       </c>
       <c r="D80" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -13046,10 +13064,10 @@
     <row r="81" ht="34" customHeight="1">
       <c r="A81" s="3"/>
       <c r="B81" s="29" t="str">
-        <v>Prior hospitalizations</v>
+        <v>Most recent hospitalization</v>
       </c>
       <c r="C81" s="29" t="str">
-        <v>Whole number</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D81" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -13059,10 +13077,10 @@
     <row r="82" ht="34" customHeight="1">
       <c r="A82" s="3"/>
       <c r="B82" s="29" t="str">
-        <v>Most recent hospitalization</v>
+        <v>Prior 5150 / 5250 holds</v>
       </c>
       <c r="C82" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D82" s="29" t="str">
         <v>07 Recent care and history</v>
@@ -13072,7 +13090,7 @@
     <row r="83" ht="34" customHeight="1">
       <c r="A83" s="3"/>
       <c r="B83" s="29" t="str">
-        <v>Prior 5150 / 5250 holds</v>
+        <v>Crisis / ER utilization</v>
       </c>
       <c r="C83" s="29" t="str">
         <v>Text or notes</v>
@@ -13085,20 +13103,20 @@
     <row r="84" ht="34" customHeight="1">
       <c r="A84" s="3"/>
       <c r="B84" s="29" t="str">
-        <v>Crisis / ER utilization</v>
+        <v>History of substance abuse</v>
       </c>
       <c r="C84" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D84" s="29" t="str">
-        <v>07 Recent care and history</v>
+        <v>08 Substance use and recovery</v>
       </c>
       <c r="E84" s="3"/>
     </row>
     <row r="85" ht="34" customHeight="1">
       <c r="A85" s="3"/>
       <c r="B85" s="29" t="str">
-        <v>History of substance abuse</v>
+        <v>Active substance use</v>
       </c>
       <c r="C85" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13111,10 +13129,10 @@
     <row r="86" ht="34" customHeight="1">
       <c r="A86" s="3"/>
       <c r="B86" s="29" t="str">
-        <v>Active substance use</v>
+        <v>Substances</v>
       </c>
       <c r="C86" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Opioids; Amphetamines; Marijuana; Alcohol; Other</v>
       </c>
       <c r="D86" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13124,10 +13142,10 @@
     <row r="87" ht="34" customHeight="1">
       <c r="A87" s="3"/>
       <c r="B87" s="29" t="str">
-        <v>Substances</v>
+        <v>Last substance use</v>
       </c>
       <c r="C87" s="29" t="str">
-        <v>Opioids; Amphetamines; Marijuana; Alcohol; Other</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D87" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13137,10 +13155,10 @@
     <row r="88" ht="34" customHeight="1">
       <c r="A88" s="3"/>
       <c r="B88" s="29" t="str">
-        <v>Last substance use</v>
+        <v>Use pattern</v>
       </c>
       <c r="C88" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Daily; Weekly; Sporadic; Rarely</v>
       </c>
       <c r="D88" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13150,49 +13168,49 @@
     <row r="89" ht="34" customHeight="1">
       <c r="A89" s="3"/>
       <c r="B89" s="29" t="str">
-        <v>Use pattern</v>
+        <v>Effect on baseline behavior</v>
       </c>
       <c r="C89" s="29" t="str">
-        <v>Daily; Weekly; Sporadic; Rarely</v>
+        <v>Text or notes</v>
       </c>
       <c r="D89" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E89" s="3"/>
     </row>
-    <row r="90" ht="34" customHeight="1">
+    <row r="90" ht="60" customHeight="1">
       <c r="A90" s="3"/>
       <c r="B90" s="29" t="str">
-        <v>Effect on baseline behavior</v>
+        <v>Longest sobriety in the last five years</v>
       </c>
       <c r="C90" s="29" t="str">
-        <v>Text or notes</v>
+        <v>1 month; 2 months; 3 months; 4 months; 5 months; 6 months; 7 months; 8 months; 9 months; 10 months; 11 months; 1 year; 18 months; 2 years; More than 2 years</v>
       </c>
       <c r="D90" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E90" s="3"/>
     </row>
-    <row r="91" ht="60" customHeight="1">
+    <row r="91" ht="44" customHeight="1">
       <c r="A91" s="3"/>
       <c r="B91" s="29" t="str">
-        <v>Longest sobriety in the last five years</v>
+        <v>Acknowledgment of substance-use impact</v>
       </c>
       <c r="C91" s="29" t="str">
-        <v>1 month; 2 months; 3 months; 4 months; 5 months; 6 months; 7 months; 8 months; 9 months; 10 months; 11 months; 1 year; 18 months; 2 years; More than 2 years</v>
+        <v>Acknowledges impact; Partially acknowledges impact; Does not acknowledge impact; Not discussed</v>
       </c>
       <c r="D91" s="29" t="str">
         <v>08 Substance use and recovery</v>
       </c>
       <c r="E91" s="3"/>
     </row>
-    <row r="92" ht="44" customHeight="1">
+    <row r="92" ht="34" customHeight="1">
       <c r="A92" s="3"/>
       <c r="B92" s="29" t="str">
-        <v>Acknowledgment of substance-use impact</v>
+        <v>Substance-use impact notes</v>
       </c>
       <c r="C92" s="29" t="str">
-        <v>Acknowledges impact; Partially acknowledges impact; Does not acknowledge impact; Not discussed</v>
+        <v>Text or notes</v>
       </c>
       <c r="D92" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13202,7 +13220,7 @@
     <row r="93" ht="34" customHeight="1">
       <c r="A93" s="3"/>
       <c r="B93" s="29" t="str">
-        <v>Substance-use impact notes</v>
+        <v>Treatment history</v>
       </c>
       <c r="C93" s="29" t="str">
         <v>Text or notes</v>
@@ -13215,10 +13233,10 @@
     <row r="94" ht="34" customHeight="1">
       <c r="A94" s="3"/>
       <c r="B94" s="29" t="str">
-        <v>Treatment history</v>
+        <v>Longest sobriety in the last five years</v>
       </c>
       <c r="C94" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D94" s="29" t="str">
         <v>08 Substance use and recovery</v>
@@ -13228,23 +13246,23 @@
     <row r="95" ht="34" customHeight="1">
       <c r="A95" s="3"/>
       <c r="B95" s="29" t="str">
-        <v>Longest sobriety in the last five years</v>
+        <v>Behavioral history</v>
       </c>
       <c r="C95" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D95" s="29" t="str">
-        <v>08 Substance use and recovery</v>
+        <v>09 Safety and support</v>
       </c>
       <c r="E95" s="3"/>
     </row>
     <row r="96" ht="34" customHeight="1">
       <c r="A96" s="3"/>
       <c r="B96" s="29" t="str">
-        <v>Behavioral history</v>
+        <v>Physical altercations</v>
       </c>
       <c r="C96" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D96" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13254,10 +13272,10 @@
     <row r="97" ht="34" customHeight="1">
       <c r="A97" s="3"/>
       <c r="B97" s="29" t="str">
-        <v>Physical altercations</v>
+        <v>Physical altercation details</v>
       </c>
       <c r="C97" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D97" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13267,10 +13285,10 @@
     <row r="98" ht="34" customHeight="1">
       <c r="A98" s="3"/>
       <c r="B98" s="29" t="str">
-        <v>Physical altercation details</v>
+        <v>History of self-harm</v>
       </c>
       <c r="C98" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D98" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13280,10 +13298,10 @@
     <row r="99" ht="34" customHeight="1">
       <c r="A99" s="3"/>
       <c r="B99" s="29" t="str">
-        <v>History of self-harm</v>
+        <v>Last documented self-harm incident</v>
       </c>
       <c r="C99" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D99" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13293,10 +13311,10 @@
     <row r="100" ht="34" customHeight="1">
       <c r="A100" s="3"/>
       <c r="B100" s="29" t="str">
-        <v>Last documented self-harm incident</v>
+        <v>Current self-harm ideation</v>
       </c>
       <c r="C100" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D100" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13306,10 +13324,10 @@
     <row r="101" ht="34" customHeight="1">
       <c r="A101" s="3"/>
       <c r="B101" s="29" t="str">
-        <v>Current self-harm ideation</v>
+        <v>Current self-harm ideation details</v>
       </c>
       <c r="C101" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D101" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13319,7 +13337,7 @@
     <row r="102" ht="34" customHeight="1">
       <c r="A102" s="3"/>
       <c r="B102" s="29" t="str">
-        <v>Current self-harm ideation details</v>
+        <v>Current safety measures</v>
       </c>
       <c r="C102" s="29" t="str">
         <v>Text or notes</v>
@@ -13332,10 +13350,10 @@
     <row r="103" ht="34" customHeight="1">
       <c r="A103" s="3"/>
       <c r="B103" s="29" t="str">
-        <v>Current safety measures</v>
+        <v>History of assaults</v>
       </c>
       <c r="C103" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D103" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13345,10 +13363,10 @@
     <row r="104" ht="34" customHeight="1">
       <c r="A104" s="3"/>
       <c r="B104" s="29" t="str">
-        <v>History of assaults</v>
+        <v>Most recent assault</v>
       </c>
       <c r="C104" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D104" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13358,10 +13376,10 @@
     <row r="105" ht="34" customHeight="1">
       <c r="A105" s="3"/>
       <c r="B105" s="29" t="str">
-        <v>Most recent assault</v>
+        <v>Assaults in the last two years</v>
       </c>
       <c r="C105" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D105" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13371,10 +13389,10 @@
     <row r="106" ht="34" customHeight="1">
       <c r="A106" s="3"/>
       <c r="B106" s="29" t="str">
-        <v>Assaults in the last two years</v>
+        <v>History of elopement</v>
       </c>
       <c r="C106" s="29" t="str">
-        <v>Whole number</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D106" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13384,10 +13402,10 @@
     <row r="107" ht="34" customHeight="1">
       <c r="A107" s="3"/>
       <c r="B107" s="29" t="str">
-        <v>History of elopement</v>
+        <v>Elopement risk</v>
       </c>
       <c r="C107" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D107" s="29" t="str">
         <v>09 Safety and support</v>
@@ -13397,7 +13415,7 @@
     <row r="108" ht="34" customHeight="1">
       <c r="A108" s="3"/>
       <c r="B108" s="29" t="str">
-        <v>Elopement risk</v>
+        <v>SI / HI history</v>
       </c>
       <c r="C108" s="29" t="str">
         <v>Text or notes</v>
@@ -13410,7 +13428,7 @@
     <row r="109" ht="34" customHeight="1">
       <c r="A109" s="3"/>
       <c r="B109" s="29" t="str">
-        <v>SI / HI history</v>
+        <v>Triggers and what helps</v>
       </c>
       <c r="C109" s="29" t="str">
         <v>Text or notes</v>
@@ -13423,7 +13441,7 @@
     <row r="110" ht="34" customHeight="1">
       <c r="A110" s="3"/>
       <c r="B110" s="29" t="str">
-        <v>Triggers and what helps</v>
+        <v>Aggression risk</v>
       </c>
       <c r="C110" s="29" t="str">
         <v>Text or notes</v>
@@ -13436,7 +13454,7 @@
     <row r="111" ht="34" customHeight="1">
       <c r="A111" s="3"/>
       <c r="B111" s="29" t="str">
-        <v>Aggression risk</v>
+        <v>Responds to internal stimuli</v>
       </c>
       <c r="C111" s="29" t="str">
         <v>Text or notes</v>
@@ -13449,7 +13467,7 @@
     <row r="112" ht="34" customHeight="1">
       <c r="A112" s="3"/>
       <c r="B112" s="29" t="str">
-        <v>Responds to internal stimuli</v>
+        <v>Auditory hallucinations</v>
       </c>
       <c r="C112" s="29" t="str">
         <v>Text or notes</v>
@@ -13462,7 +13480,7 @@
     <row r="113" ht="34" customHeight="1">
       <c r="A113" s="3"/>
       <c r="B113" s="29" t="str">
-        <v>Auditory hallucinations</v>
+        <v>Nature of auditory hallucinations</v>
       </c>
       <c r="C113" s="29" t="str">
         <v>Text or notes</v>
@@ -13475,7 +13493,7 @@
     <row r="114" ht="34" customHeight="1">
       <c r="A114" s="3"/>
       <c r="B114" s="29" t="str">
-        <v>Nature of auditory hallucinations</v>
+        <v>Current auditory frequency</v>
       </c>
       <c r="C114" s="29" t="str">
         <v>Text or notes</v>
@@ -13488,7 +13506,7 @@
     <row r="115" ht="34" customHeight="1">
       <c r="A115" s="3"/>
       <c r="B115" s="29" t="str">
-        <v>Current auditory frequency</v>
+        <v>Auditory triggers</v>
       </c>
       <c r="C115" s="29" t="str">
         <v>Text or notes</v>
@@ -13501,7 +13519,7 @@
     <row r="116" ht="34" customHeight="1">
       <c r="A116" s="3"/>
       <c r="B116" s="29" t="str">
-        <v>Auditory triggers</v>
+        <v>Visual hallucinations</v>
       </c>
       <c r="C116" s="29" t="str">
         <v>Text or notes</v>
@@ -13514,7 +13532,7 @@
     <row r="117" ht="34" customHeight="1">
       <c r="A117" s="3"/>
       <c r="B117" s="29" t="str">
-        <v>Visual hallucinations</v>
+        <v>Nature and frequency of visual hallucinations</v>
       </c>
       <c r="C117" s="29" t="str">
         <v>Text or notes</v>
@@ -13527,7 +13545,7 @@
     <row r="118" ht="34" customHeight="1">
       <c r="A118" s="3"/>
       <c r="B118" s="29" t="str">
-        <v>Nature and frequency of visual hallucinations</v>
+        <v>Recent visual hallucinations</v>
       </c>
       <c r="C118" s="29" t="str">
         <v>Text or notes</v>
@@ -13540,7 +13558,7 @@
     <row r="119" ht="34" customHeight="1">
       <c r="A119" s="3"/>
       <c r="B119" s="29" t="str">
-        <v>Recent visual hallucinations</v>
+        <v>Olfactory hallucinations</v>
       </c>
       <c r="C119" s="29" t="str">
         <v>Text or notes</v>
@@ -13553,7 +13571,7 @@
     <row r="120" ht="34" customHeight="1">
       <c r="A120" s="3"/>
       <c r="B120" s="29" t="str">
-        <v>Olfactory hallucinations</v>
+        <v>Olfactory hallucination details</v>
       </c>
       <c r="C120" s="29" t="str">
         <v>Text or notes</v>
@@ -13566,7 +13584,7 @@
     <row r="121" ht="34" customHeight="1">
       <c r="A121" s="3"/>
       <c r="B121" s="29" t="str">
-        <v>Olfactory hallucination details</v>
+        <v>Impact of olfactory hallucinations</v>
       </c>
       <c r="C121" s="29" t="str">
         <v>Text or notes</v>
@@ -13579,7 +13597,7 @@
     <row r="122" ht="34" customHeight="1">
       <c r="A122" s="3"/>
       <c r="B122" s="29" t="str">
-        <v>Impact of olfactory hallucinations</v>
+        <v>Tactile hallucinations</v>
       </c>
       <c r="C122" s="29" t="str">
         <v>Text or notes</v>
@@ -13592,7 +13610,7 @@
     <row r="123" ht="34" customHeight="1">
       <c r="A123" s="3"/>
       <c r="B123" s="29" t="str">
-        <v>Tactile hallucinations</v>
+        <v>Tactile hallucination details</v>
       </c>
       <c r="C123" s="29" t="str">
         <v>Text or notes</v>
@@ -13605,7 +13623,7 @@
     <row r="124" ht="34" customHeight="1">
       <c r="A124" s="3"/>
       <c r="B124" s="29" t="str">
-        <v>Tactile hallucination details</v>
+        <v>Tactile hallucination frequency</v>
       </c>
       <c r="C124" s="29" t="str">
         <v>Text or notes</v>
@@ -13618,7 +13636,7 @@
     <row r="125" ht="34" customHeight="1">
       <c r="A125" s="3"/>
       <c r="B125" s="29" t="str">
-        <v>Tactile hallucination frequency</v>
+        <v>Gustatory hallucinations</v>
       </c>
       <c r="C125" s="29" t="str">
         <v>Text or notes</v>
@@ -13631,7 +13649,7 @@
     <row r="126" ht="34" customHeight="1">
       <c r="A126" s="3"/>
       <c r="B126" s="29" t="str">
-        <v>Gustatory hallucinations</v>
+        <v>Gustatory hallucination details</v>
       </c>
       <c r="C126" s="29" t="str">
         <v>Text or notes</v>
@@ -13644,7 +13662,7 @@
     <row r="127" ht="34" customHeight="1">
       <c r="A127" s="3"/>
       <c r="B127" s="29" t="str">
-        <v>Gustatory hallucination details</v>
+        <v>Hallucination coping strategies</v>
       </c>
       <c r="C127" s="29" t="str">
         <v>Text or notes</v>
@@ -13657,7 +13675,7 @@
     <row r="128" ht="34" customHeight="1">
       <c r="A128" s="3"/>
       <c r="B128" s="29" t="str">
-        <v>Hallucination coping strategies</v>
+        <v>Hallucination distress or impairment</v>
       </c>
       <c r="C128" s="29" t="str">
         <v>Text or notes</v>
@@ -13670,7 +13688,7 @@
     <row r="129" ht="34" customHeight="1">
       <c r="A129" s="3"/>
       <c r="B129" s="29" t="str">
-        <v>Hallucination distress or impairment</v>
+        <v>Impact on daily functioning</v>
       </c>
       <c r="C129" s="29" t="str">
         <v>Text or notes</v>
@@ -13683,7 +13701,7 @@
     <row r="130" ht="34" customHeight="1">
       <c r="A130" s="3"/>
       <c r="B130" s="29" t="str">
-        <v>Impact on daily functioning</v>
+        <v>Professional discussion and treatment</v>
       </c>
       <c r="C130" s="29" t="str">
         <v>Text or notes</v>
@@ -13696,23 +13714,23 @@
     <row r="131" ht="34" customHeight="1">
       <c r="A131" s="3"/>
       <c r="B131" s="29" t="str">
-        <v>Professional discussion and treatment</v>
+        <v>Conserved status</v>
       </c>
       <c r="C131" s="29" t="str">
-        <v>Text or notes</v>
+        <v>LPS; TCon; Murphy's; Non-Conserved</v>
       </c>
       <c r="D131" s="29" t="str">
-        <v>09 Safety and support</v>
+        <v>10 Decisions and legal support</v>
       </c>
       <c r="E131" s="3"/>
     </row>
     <row r="132" ht="34" customHeight="1">
       <c r="A132" s="3"/>
       <c r="B132" s="29" t="str">
-        <v>Conserved status</v>
+        <v>Conservator name</v>
       </c>
       <c r="C132" s="29" t="str">
-        <v>LPS; TCon; Murphy's; Non-Conserved</v>
+        <v>Text or notes</v>
       </c>
       <c r="D132" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13722,7 +13740,7 @@
     <row r="133" ht="34" customHeight="1">
       <c r="A133" s="3"/>
       <c r="B133" s="29" t="str">
-        <v>Conservator name</v>
+        <v>Conservatorship details</v>
       </c>
       <c r="C133" s="29" t="str">
         <v>Text or notes</v>
@@ -13735,7 +13753,7 @@
     <row r="134" ht="34" customHeight="1">
       <c r="A134" s="3"/>
       <c r="B134" s="29" t="str">
-        <v>Conservatorship details</v>
+        <v>Hold type</v>
       </c>
       <c r="C134" s="29" t="str">
         <v>Text or notes</v>
@@ -13748,7 +13766,7 @@
     <row r="135" ht="34" customHeight="1">
       <c r="A135" s="3"/>
       <c r="B135" s="29" t="str">
-        <v>Hold type</v>
+        <v>Forensic history</v>
       </c>
       <c r="C135" s="29" t="str">
         <v>Text or notes</v>
@@ -13761,10 +13779,10 @@
     <row r="136" ht="34" customHeight="1">
       <c r="A136" s="3"/>
       <c r="B136" s="29" t="str">
-        <v>Forensic history</v>
+        <v>PC 290 registration</v>
       </c>
       <c r="C136" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D136" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13774,10 +13792,10 @@
     <row r="137" ht="34" customHeight="1">
       <c r="A137" s="3"/>
       <c r="B137" s="29" t="str">
-        <v>Forensic timeline</v>
+        <v>Arson history</v>
       </c>
       <c r="C137" s="29" t="str">
-        <v>One item per line</v>
+        <v>Yes; No; Unable to assess</v>
       </c>
       <c r="D137" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13787,7 +13805,7 @@
     <row r="138" ht="34" customHeight="1">
       <c r="A138" s="3"/>
       <c r="B138" s="29" t="str">
-        <v>PC 290 registration</v>
+        <v>Diversion client</v>
       </c>
       <c r="C138" s="29" t="str">
         <v>Yes; No; Unable to assess</v>
@@ -13800,10 +13818,10 @@
     <row r="139" ht="34" customHeight="1">
       <c r="A139" s="3"/>
       <c r="B139" s="29" t="str">
-        <v>Arson history</v>
+        <v>Court requirements</v>
       </c>
       <c r="C139" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D139" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13813,10 +13831,10 @@
     <row r="140" ht="34" customHeight="1">
       <c r="A140" s="3"/>
       <c r="B140" s="29" t="str">
-        <v>Diversion client</v>
+        <v>Court dates</v>
       </c>
       <c r="C140" s="29" t="str">
-        <v>Yes; No; Unable to assess</v>
+        <v>Text or notes</v>
       </c>
       <c r="D140" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13826,7 +13844,7 @@
     <row r="141" ht="34" customHeight="1">
       <c r="A141" s="3"/>
       <c r="B141" s="29" t="str">
-        <v>Court requirements</v>
+        <v>Probation / parole / justice</v>
       </c>
       <c r="C141" s="29" t="str">
         <v>Text or notes</v>
@@ -13839,7 +13857,7 @@
     <row r="142" ht="34" customHeight="1">
       <c r="A142" s="3"/>
       <c r="B142" s="29" t="str">
-        <v>Court dates</v>
+        <v>Forensic involvement</v>
       </c>
       <c r="C142" s="29" t="str">
         <v>Text or notes</v>
@@ -13852,7 +13870,7 @@
     <row r="143" ht="34" customHeight="1">
       <c r="A143" s="3"/>
       <c r="B143" s="29" t="str">
-        <v>Probation / parole / justice</v>
+        <v>Forensic involvement details</v>
       </c>
       <c r="C143" s="29" t="str">
         <v>Text or notes</v>
@@ -13865,7 +13883,7 @@
     <row r="144" ht="34" customHeight="1">
       <c r="A144" s="3"/>
       <c r="B144" s="29" t="str">
-        <v>Forensic involvement</v>
+        <v>History of arrest</v>
       </c>
       <c r="C144" s="29" t="str">
         <v>Text or notes</v>
@@ -13878,10 +13896,10 @@
     <row r="145" ht="34" customHeight="1">
       <c r="A145" s="3"/>
       <c r="B145" s="29" t="str">
-        <v>Forensic involvement details</v>
+        <v>Most recent arrest date</v>
       </c>
       <c r="C145" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Date (YYYY-MM-DD)</v>
       </c>
       <c r="D145" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13891,7 +13909,7 @@
     <row r="146" ht="34" customHeight="1">
       <c r="A146" s="3"/>
       <c r="B146" s="29" t="str">
-        <v>History of arrest</v>
+        <v>Most recent arrest charge</v>
       </c>
       <c r="C146" s="29" t="str">
         <v>Text or notes</v>
@@ -13904,10 +13922,10 @@
     <row r="147" ht="34" customHeight="1">
       <c r="A147" s="3"/>
       <c r="B147" s="29" t="str">
-        <v>Most recent arrest date</v>
+        <v>Time in jail</v>
       </c>
       <c r="C147" s="29" t="str">
-        <v>Date (YYYY-MM-DD)</v>
+        <v>Text or notes</v>
       </c>
       <c r="D147" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13917,7 +13935,7 @@
     <row r="148" ht="34" customHeight="1">
       <c r="A148" s="3"/>
       <c r="B148" s="29" t="str">
-        <v>Most recent arrest charge</v>
+        <v>Arrest in the last two years</v>
       </c>
       <c r="C148" s="29" t="str">
         <v>Text or notes</v>
@@ -13930,7 +13948,7 @@
     <row r="149" ht="34" customHeight="1">
       <c r="A149" s="3"/>
       <c r="B149" s="29" t="str">
-        <v>Time in jail</v>
+        <v>Recent arrest details</v>
       </c>
       <c r="C149" s="29" t="str">
         <v>Text or notes</v>
@@ -13943,10 +13961,10 @@
     <row r="150" ht="34" customHeight="1">
       <c r="A150" s="3"/>
       <c r="B150" s="29" t="str">
-        <v>Arrest in the last two years</v>
+        <v>Total recorded arrests</v>
       </c>
       <c r="C150" s="29" t="str">
-        <v>Text or notes</v>
+        <v>Whole number</v>
       </c>
       <c r="D150" s="29" t="str">
         <v>10 Decisions and legal support</v>
@@ -13956,33 +13974,33 @@
     <row r="151" ht="34" customHeight="1">
       <c r="A151" s="3"/>
       <c r="B151" s="29" t="str">
-        <v>Recent arrest details</v>
+        <v>Family involvement</v>
       </c>
       <c r="C151" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D151" s="29" t="str">
-        <v>10 Decisions and legal support</v>
+        <v>11 What matters next</v>
       </c>
       <c r="E151" s="3"/>
     </row>
     <row r="152" ht="34" customHeight="1">
       <c r="A152" s="3"/>
       <c r="B152" s="29" t="str">
-        <v>Total recorded arrests</v>
+        <v>Friendships and social connections</v>
       </c>
       <c r="C152" s="29" t="str">
-        <v>Whole number</v>
+        <v>Text or notes</v>
       </c>
       <c r="D152" s="29" t="str">
-        <v>10 Decisions and legal support</v>
+        <v>11 What matters next</v>
       </c>
       <c r="E152" s="3"/>
     </row>
     <row r="153" ht="34" customHeight="1">
       <c r="A153" s="3"/>
       <c r="B153" s="29" t="str">
-        <v>Family involvement</v>
+        <v>Home and housing history</v>
       </c>
       <c r="C153" s="29" t="str">
         <v>Text or notes</v>
@@ -13995,7 +14013,7 @@
     <row r="154" ht="34" customHeight="1">
       <c r="A154" s="3"/>
       <c r="B154" s="29" t="str">
-        <v>Friendships and social connections</v>
+        <v>Benefits / income status</v>
       </c>
       <c r="C154" s="29" t="str">
         <v>Text or notes</v>
@@ -14008,7 +14026,7 @@
     <row r="155" ht="34" customHeight="1">
       <c r="A155" s="3"/>
       <c r="B155" s="29" t="str">
-        <v>Home and housing history</v>
+        <v>Discharge planning goals</v>
       </c>
       <c r="C155" s="29" t="str">
         <v>Text or notes</v>
@@ -14021,7 +14039,7 @@
     <row r="156" ht="34" customHeight="1">
       <c r="A156" s="3"/>
       <c r="B156" s="29" t="str">
-        <v>Benefits / income status</v>
+        <v>Placement preferences and concerns</v>
       </c>
       <c r="C156" s="29" t="str">
         <v>Text or notes</v>
@@ -14034,79 +14052,61 @@
     <row r="157" ht="34" customHeight="1">
       <c r="A157" s="3"/>
       <c r="B157" s="29" t="str">
-        <v>Preferred facility characteristics</v>
+        <v>Additional information</v>
       </c>
       <c r="C157" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D157" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>12 Anything else</v>
       </c>
       <c r="E157" s="3"/>
     </row>
     <row r="158" ht="34" customHeight="1">
       <c r="A158" s="3"/>
       <c r="B158" s="29" t="str">
-        <v>Discharge planning goals</v>
+        <v>Placement questions or concerns</v>
       </c>
       <c r="C158" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D158" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>12 Anything else</v>
       </c>
       <c r="E158" s="3"/>
     </row>
     <row r="159" ht="34" customHeight="1">
       <c r="A159" s="3"/>
       <c r="B159" s="29" t="str">
-        <v>Placement preferences and concerns</v>
+        <v>Assessment notes</v>
       </c>
       <c r="C159" s="29" t="str">
         <v>Text or notes</v>
       </c>
       <c r="D159" s="29" t="str">
-        <v>11 What matters next</v>
+        <v>12 Anything else</v>
       </c>
       <c r="E159" s="3"/>
     </row>
-    <row r="160" ht="34" customHeight="1">
+    <row r="160">
       <c r="A160" s="3"/>
-      <c r="B160" s="29" t="str">
-        <v>Additional information</v>
-      </c>
-      <c r="C160" s="29" t="str">
-        <v>Text or notes</v>
-      </c>
-      <c r="D160" s="29" t="str">
-        <v>12 Anything else</v>
-      </c>
+      <c r="B160" s="3"/>
+      <c r="C160" s="3"/>
+      <c r="D160" s="3"/>
       <c r="E160" s="3"/>
     </row>
-    <row r="161" ht="34" customHeight="1">
+    <row r="161">
       <c r="A161" s="3"/>
-      <c r="B161" s="29" t="str">
-        <v>Placement questions or concerns</v>
-      </c>
-      <c r="C161" s="29" t="str">
-        <v>Text or notes</v>
-      </c>
-      <c r="D161" s="29" t="str">
-        <v>12 Anything else</v>
-      </c>
+      <c r="B161" s="3"/>
+      <c r="C161" s="3"/>
+      <c r="D161" s="3"/>
       <c r="E161" s="3"/>
     </row>
-    <row r="162" ht="34" customHeight="1">
+    <row r="162">
       <c r="A162" s="3"/>
-      <c r="B162" s="29" t="str">
-        <v>Assessment notes</v>
-      </c>
-      <c r="C162" s="29" t="str">
-        <v>Text or notes</v>
-      </c>
-      <c r="D162" s="29" t="str">
-        <v>12 Anything else</v>
-      </c>
+      <c r="B162" s="3"/>
+      <c r="C162" s="3"/>
+      <c r="D162" s="3"/>
       <c r="E162" s="3"/>
     </row>
     <row r="163">
@@ -15918,12 +15918,30 @@
         <v>Check</v>
       </c>
     </row>
-    <row r="6" ht="34" customHeight="1">
+    <row r="6" ht="63" customHeight="1">
       <c r="A6" s="3" t="str">
         <v>physical_health_concerns</v>
       </c>
-      <c r="B6" s="13" t="str">
-        <v>Physical health concerns</v>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="12"/>
+              <color rgb="FF233B32"/>
+            </rPr>
+            <t>Physical health concerns</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="0"/>
+              <sz val="10"/>
+              <color rgb="FF59675F"/>
+            </rPr>
+            <t xml:space="preserve">
+Use this for other health concerns. Diabetes, diet, and skin have their own questions below.</t>
+          </r>
+        </is>
       </c>
       <c r="C6" t="str" s="50"/>
       <c r="D6" t="str" s="48"/>
@@ -17652,11 +17670,53 @@
         <v>Optional</v>
       </c>
     </row>
-    <row r="9" ht="72" customHeight="1">
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="3" t="str">
+        <v>prior_hospitalizations_count</v>
+      </c>
+      <c r="B9" s="13" t="str">
+        <v>Prior hospitalizations</v>
+      </c>
+      <c r="C9" t="str" s="58"/>
+      <c r="D9" t="str" s="48"/>
+      <c r="E9" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C9))&gt;0,LEN(TRIM(D9))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D9))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D9))&gt;0)),"Explain why",IF(LEN(TRIM(C9))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="3" t="str">
+        <v>most_recent_hospitalization</v>
+      </c>
+      <c r="B10" s="13" t="str">
+        <v>Most recent hospitalization</v>
+      </c>
+      <c r="C10" t="str" s="51"/>
+      <c r="D10" t="str" s="48"/>
+      <c r="E10" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C10))&gt;0,LEN(TRIM(D10))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D10))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D10))&gt;0)),"Explain why",IF(LEN(TRIM(C10))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="3" t="str">
+        <v>prior_5150_5250_holds</v>
+      </c>
+      <c r="B11" s="13" t="str">
+        <v>Prior 5150 / 5250 holds</v>
+      </c>
+      <c r="C11" t="str" s="50"/>
+      <c r="D11" t="str" s="48"/>
+      <c r="E11" s="16" t="str">
+        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C11))&gt;0,LEN(TRIM(D11))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D11))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D11))&gt;0)),"Explain why",IF(LEN(TRIM(C11))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
+        <v>Optional</v>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1">
+      <c r="A12" s="3" t="str">
         <v>hospitalization_timeline</v>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -17673,201 +17733,159 @@
               <color rgb="FF59675F"/>
             </rPr>
             <t xml:space="preserve">
-Optional. Add an event only when you know enough to describe it; approximate timing is fine.</t>
+Reference only.</t>
           </r>
         </is>
       </c>
-      <c r="C9" t="str" s="50"/>
-      <c r="D9" t="str" s="48"/>
-      <c r="E9" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C9&amp;""&amp;C10&amp;""&amp;C11&amp;""&amp;C12&amp;""&amp;C13&amp;""&amp;C14&amp;""&amp;C15&amp;""&amp;C16&amp;""&amp;C17&amp;""&amp;C18&amp;""&amp;C19&amp;""&amp;C20&amp;""&amp;C21&amp;""&amp;C22))&gt;0,LEN(TRIM(D9))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D9))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D9))&gt;0)),"Explain why",IF(LEN(TRIM(C9&amp;""&amp;C10&amp;""&amp;C11&amp;""&amp;C12&amp;""&amp;C13&amp;""&amp;C14&amp;""&amp;C15&amp;""&amp;C16&amp;""&amp;C17&amp;""&amp;C18&amp;""&amp;C19&amp;""&amp;C20&amp;""&amp;C21&amp;""&amp;C22))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
-    </row>
-    <row r="10" ht="88" customHeight="1" hidden="1">
-      <c r="A10" s="3" t="str">
-        <v>hospitalization_timeline:1</v>
-      </c>
-      <c r="B10" s="3" t="str">
-        <v>Hospitalization timeline (continued)</v>
-      </c>
-      <c r="C10" t="str" s="57"/>
-      <c r="D10" s="3" t="str"/>
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" ht="88" customHeight="1" hidden="1">
-      <c r="A11" s="3" t="str">
-        <v>hospitalization_timeline:2</v>
-      </c>
-      <c r="B11" s="3" t="str">
-        <v>Hospitalization timeline (continued)</v>
-      </c>
-      <c r="C11" t="str" s="57"/>
-      <c r="D11" s="3" t="str"/>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="12" ht="88" customHeight="1" hidden="1">
-      <c r="A12" s="3" t="str">
-        <v>hospitalization_timeline:3</v>
-      </c>
-      <c r="B12" s="3" t="str">
-        <v>Hospitalization timeline (continued)</v>
-      </c>
-      <c r="C12" t="str" s="57"/>
-      <c r="D12" s="3" t="str"/>
-      <c r="E12" s="3"/>
+      <c r="C12" s="23" t="str"/>
+      <c r="D12" s="15" t="str"/>
+      <c r="E12" s="16" t="str">
+        <f>"Reference only"</f>
+        <v>Reference only</v>
+      </c>
     </row>
     <row r="13" ht="88" customHeight="1" hidden="1">
       <c r="A13" s="3" t="str">
-        <v>hospitalization_timeline:4</v>
+        <v>hospitalization_timeline:1</v>
       </c>
       <c r="B13" s="3" t="str">
         <v>Hospitalization timeline (continued)</v>
       </c>
-      <c r="C13" t="str" s="57"/>
+      <c r="C13" s="24" t="str"/>
       <c r="D13" s="3" t="str"/>
       <c r="E13" s="3"/>
     </row>
     <row r="14" ht="88" customHeight="1" hidden="1">
       <c r="A14" s="3" t="str">
-        <v>hospitalization_timeline:5</v>
+        <v>hospitalization_timeline:2</v>
       </c>
       <c r="B14" s="3" t="str">
         <v>Hospitalization timeline (continued)</v>
       </c>
-      <c r="C14" t="str" s="57"/>
+      <c r="C14" s="24" t="str"/>
       <c r="D14" s="3" t="str"/>
       <c r="E14" s="3"/>
     </row>
     <row r="15" ht="88" customHeight="1" hidden="1">
       <c r="A15" s="3" t="str">
-        <v>hospitalization_timeline:6</v>
+        <v>hospitalization_timeline:3</v>
       </c>
       <c r="B15" s="3" t="str">
         <v>Hospitalization timeline (continued)</v>
       </c>
-      <c r="C15" t="str" s="57"/>
+      <c r="C15" s="24" t="str"/>
       <c r="D15" s="3" t="str"/>
       <c r="E15" s="3"/>
     </row>
     <row r="16" ht="88" customHeight="1" hidden="1">
       <c r="A16" s="3" t="str">
-        <v>hospitalization_timeline:7</v>
+        <v>hospitalization_timeline:4</v>
       </c>
       <c r="B16" s="3" t="str">
         <v>Hospitalization timeline (continued)</v>
       </c>
-      <c r="C16" t="str" s="57"/>
+      <c r="C16" s="24" t="str"/>
       <c r="D16" s="3" t="str"/>
       <c r="E16" s="3"/>
     </row>
     <row r="17" ht="88" customHeight="1" hidden="1">
       <c r="A17" s="3" t="str">
-        <v>hospitalization_timeline:8</v>
+        <v>hospitalization_timeline:5</v>
       </c>
       <c r="B17" s="3" t="str">
         <v>Hospitalization timeline (continued)</v>
       </c>
-      <c r="C17" t="str" s="57"/>
+      <c r="C17" s="24" t="str"/>
       <c r="D17" s="3" t="str"/>
       <c r="E17" s="3"/>
     </row>
     <row r="18" ht="88" customHeight="1" hidden="1">
       <c r="A18" s="3" t="str">
-        <v>hospitalization_timeline:9</v>
+        <v>hospitalization_timeline:6</v>
       </c>
       <c r="B18" s="3" t="str">
         <v>Hospitalization timeline (continued)</v>
       </c>
-      <c r="C18" t="str" s="57"/>
+      <c r="C18" s="24" t="str"/>
       <c r="D18" s="3" t="str"/>
       <c r="E18" s="3"/>
     </row>
     <row r="19" ht="88" customHeight="1" hidden="1">
       <c r="A19" s="3" t="str">
-        <v>hospitalization_timeline:10</v>
+        <v>hospitalization_timeline:7</v>
       </c>
       <c r="B19" s="3" t="str">
         <v>Hospitalization timeline (continued)</v>
       </c>
-      <c r="C19" t="str" s="57"/>
+      <c r="C19" s="24" t="str"/>
       <c r="D19" s="3" t="str"/>
       <c r="E19" s="3"/>
     </row>
     <row r="20" ht="88" customHeight="1" hidden="1">
       <c r="A20" s="3" t="str">
-        <v>hospitalization_timeline:11</v>
+        <v>hospitalization_timeline:8</v>
       </c>
       <c r="B20" s="3" t="str">
         <v>Hospitalization timeline (continued)</v>
       </c>
-      <c r="C20" t="str" s="57"/>
+      <c r="C20" s="24" t="str"/>
       <c r="D20" s="3" t="str"/>
       <c r="E20" s="3"/>
     </row>
     <row r="21" ht="88" customHeight="1" hidden="1">
       <c r="A21" s="3" t="str">
-        <v>hospitalization_timeline:12</v>
+        <v>hospitalization_timeline:9</v>
       </c>
       <c r="B21" s="3" t="str">
         <v>Hospitalization timeline (continued)</v>
       </c>
-      <c r="C21" t="str" s="57"/>
+      <c r="C21" s="24" t="str"/>
       <c r="D21" s="3" t="str"/>
       <c r="E21" s="3"/>
     </row>
     <row r="22" ht="88" customHeight="1" hidden="1">
       <c r="A22" s="3" t="str">
-        <v>hospitalization_timeline:13</v>
+        <v>hospitalization_timeline:10</v>
       </c>
       <c r="B22" s="3" t="str">
         <v>Hospitalization timeline (continued)</v>
       </c>
-      <c r="C22" t="str" s="57"/>
+      <c r="C22" s="24" t="str"/>
       <c r="D22" s="3" t="str"/>
       <c r="E22" s="3"/>
     </row>
-    <row r="23" ht="34" customHeight="1">
+    <row r="23" ht="88" customHeight="1" hidden="1">
       <c r="A23" s="3" t="str">
-        <v>prior_hospitalizations_count</v>
-      </c>
-      <c r="B23" s="13" t="str">
-        <v>Prior hospitalizations</v>
-      </c>
-      <c r="C23" t="str" s="58"/>
-      <c r="D23" t="str" s="48"/>
-      <c r="E23" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C23))&gt;0,LEN(TRIM(D23))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D23))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D23))&gt;0)),"Explain why",IF(LEN(TRIM(C23))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
-    </row>
-    <row r="24" ht="34" customHeight="1">
+        <v>hospitalization_timeline:11</v>
+      </c>
+      <c r="B23" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C23" s="24" t="str"/>
+      <c r="D23" s="3" t="str"/>
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" ht="88" customHeight="1" hidden="1">
       <c r="A24" s="3" t="str">
-        <v>most_recent_hospitalization</v>
-      </c>
-      <c r="B24" s="13" t="str">
-        <v>Most recent hospitalization</v>
-      </c>
-      <c r="C24" t="str" s="51"/>
-      <c r="D24" t="str" s="48"/>
-      <c r="E24" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C24))&gt;0,LEN(TRIM(D24))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D24))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D24))&gt;0)),"Explain why",IF(LEN(TRIM(C24))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
-    </row>
-    <row r="25" ht="34" customHeight="1">
+        <v>hospitalization_timeline:12</v>
+      </c>
+      <c r="B24" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C24" s="24" t="str"/>
+      <c r="D24" s="3" t="str"/>
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" ht="88" customHeight="1" hidden="1">
       <c r="A25" s="3" t="str">
-        <v>prior_5150_5250_holds</v>
-      </c>
-      <c r="B25" s="13" t="str">
-        <v>Prior 5150 / 5250 holds</v>
-      </c>
-      <c r="C25" t="str" s="50"/>
-      <c r="D25" t="str" s="48"/>
-      <c r="E25" s="16" t="str">
-        <f>IF(NOT(TRUE),IF(OR(LEN(TRIM(C25))&gt;0,LEN(TRIM(D25))&gt;0),"Review previous answer","Not applicable"),IF(AND(LEN(TRIM(D25))&gt;0,NOT(FALSE)),"Review previous reason",IF(AND(FALSE,NOT(LEN(TRIM(D25))&gt;0)),"Explain why",IF(LEN(TRIM(C25))&gt;0,"Answered",IF(FALSE,"Needs answer","Optional")))))</f>
-        <v>Optional</v>
-      </c>
+        <v>hospitalization_timeline:13</v>
+      </c>
+      <c r="B25" s="3" t="str">
+        <v>Hospitalization timeline (continued)</v>
+      </c>
+      <c r="C25" s="24" t="str"/>
+      <c r="D25" s="3" t="str"/>
+      <c r="E25" s="3"/>
     </row>
     <row r="26" ht="34" customHeight="1">
       <c r="A26" s="3" t="str">
@@ -17931,34 +17949,34 @@
       <formula>OR($E9="Needs answer",$E9="Explain why",LEFT($E9,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B23:E23">
+  <conditionalFormatting sqref="B10:E10">
     <cfRule type="expression" dxfId="178" priority="9">
-      <formula>$E23="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E23:E23">
+      <formula>$E10="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E10:E10">
     <cfRule type="expression" dxfId="179" priority="10">
-      <formula>OR($E23="Needs answer",$E23="Explain why",LEFT($E23,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B24:E24">
+      <formula>OR($E10="Needs answer",$E10="Explain why",LEFT($E10,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11:E11">
     <cfRule type="expression" dxfId="180" priority="11">
-      <formula>$E24="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E24:E24">
+      <formula>$E11="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E11:E11">
     <cfRule type="expression" dxfId="181" priority="12">
-      <formula>OR($E24="Needs answer",$E24="Explain why",LEFT($E24,6)="Review")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B25:E25">
+      <formula>OR($E11="Needs answer",$E11="Explain why",LEFT($E11,6)="Review")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B12:E12">
     <cfRule type="expression" dxfId="182" priority="13">
-      <formula>$E25="Not applicable"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E25:E25">
+      <formula>$E12="Not applicable"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12:E12">
     <cfRule type="expression" dxfId="183" priority="14">
-      <formula>OR($E25="Needs answer",$E25="Explain why",LEFT($E25,6)="Review")</formula>
+      <formula>OR($E12="Needs answer",$E12="Explain why",LEFT($E12,6)="Review")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B26:E26">

</xml_diff>

<commit_message>
Clarify safety questions and retire Excel assessment controls
</commit_message>
<xml_diff>
--- a/public/templates/pipeline-assessment-workbook.xlsx
+++ b/public/templates/pipeline-assessment-workbook.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Re56b9b25da424454"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="Rb8877295a23342e9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R5792cea647164f84"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="R8adede638d3b48a0"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="Recf645d799044eef"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="R7f05fc8c83b04708"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="Re5e59df1ad974e31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="Rb4d5de57739849d5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="Rb6ac36abfee240bb"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R5f1f749efc254059"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="R01d5c1a26d264a9e"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R9e31f31815b14ef9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="R8b6b6ea4958b4d38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="R5748b07ebda94d82" state="veryHidden"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="R99a8451577a8493e"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rf9e855ce1b754673"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Confirm the basics" sheetId="2" r:id="R3a223790d1584ee6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 How things are now" sheetId="3" r:id="R2b8c3995c13348c2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 A usual day" sheetId="4" r:id="R3071e861218445af"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Health and comfort" sheetId="5" r:id="R7c54bb215b0140f7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Medication" sheetId="6" r:id="Ra8fa11ef59de4a86"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Living situation" sheetId="7" r:id="Rb8e0d0af5a5c4946"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Recent care and history" sheetId="8" r:id="R2624aab392ee47eb"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Substance use and recovery" sheetId="9" r:id="R91cd2bffc7a44ef7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Safety and support" sheetId="10" r:id="R0158aeef1a634632"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Decisions and legal support" sheetId="11" r:id="Rdfcc5cb75f2347d5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 What matters next" sheetId="12" r:id="R1fe734867cbd45a8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Anything else" sheetId="13" r:id="R3e5f6d6c3ae54e2b"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline_Data" sheetId="14" r:id="Rf373fc7a741a40c5" state="veryHidden"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codebook" sheetId="15" r:id="R40bdbabde5c84b09"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Confirm the basics'!$B$1:$E$16</definedName>
@@ -5152,12 +5152,30 @@
         <v>Optional</v>
       </c>
     </row>
-    <row r="7" ht="34" customHeight="1">
+    <row r="7" ht="51" customHeight="1">
       <c r="A7" s="3" t="str">
         <v>physical_altercations</v>
       </c>
-      <c r="B7" s="13" t="str">
-        <v>Physical altercations</v>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="12"/>
+              <color rgb="FF233B32"/>
+            </rPr>
+            <t>Physical altercations</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="0"/>
+              <sz val="10"/>
+              <color rgb="FF59675F"/>
+            </rPr>
+            <t xml:space="preserve">
+With staff, other clients, or family members in a care setting.</t>
+          </r>
+        </is>
       </c>
       <c r="C7" t="str" s="50"/>
       <c r="D7" t="str" s="48"/>
@@ -5323,12 +5341,30 @@
         <v>Not applicable</v>
       </c>
     </row>
-    <row r="14" ht="34" customHeight="1">
+    <row r="14" ht="51" customHeight="1">
       <c r="A14" s="3" t="str">
         <v>assault_history</v>
       </c>
-      <c r="B14" s="13" t="str">
-        <v>History of assaults</v>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="12"/>
+              <color rgb="FF233B32"/>
+            </rPr>
+            <t>History of assaults</t>
+          </r>
+          <r>
+            <rPr>
+              <b val="0"/>
+              <sz val="10"/>
+              <color rgb="FF59675F"/>
+            </rPr>
+            <t xml:space="preserve">
+Outside care settings or involving criminal charges.</t>
+          </r>
+        </is>
       </c>
       <c r="C14" t="str" s="50"/>
       <c r="D14" t="str" s="48"/>
@@ -8025,7 +8061,7 @@
         <v>Questionnaire fingerprint</v>
       </c>
       <c r="B2" t="str">
-        <v>d01f4e8eb2fa55dffca35c74bf99212eef02e9d6e83b2b40d0e5de806481fee8</v>
+        <v>abb8ea3d3c86c8749559278d11d52373dba873f4d10aa8ff44567fdc2f788818</v>
       </c>
     </row>
     <row r="3">

</xml_diff>